<commit_message>
Updated data and fixes
</commit_message>
<xml_diff>
--- a/www/flightdata/xlsx/eoss-300.xlsx
+++ b/www/flightdata/xlsx/eoss-300.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="650" uniqueCount="252">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="655" uniqueCount="257">
   <si>
     <t>flight</t>
   </si>
@@ -36,6 +36,18 @@
     <t>h2fill</t>
   </si>
   <si>
+    <t>maxaltitude</t>
+  </si>
+  <si>
+    <t>numpoints</t>
+  </si>
+  <si>
+    <t>flighttime</t>
+  </si>
+  <si>
+    <t>flighttime_secs</t>
+  </si>
+  <si>
     <t>weights.client</t>
   </si>
   <si>
@@ -73,6 +85,9 @@
   </si>
   <si>
     <t>198</t>
+  </si>
+  <si>
+    <t>0hrs 24mins 56secs</t>
   </si>
   <si>
     <t>0.12</t>
@@ -1133,10 +1148,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:Q2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:13">
+    <row r="1" spans="1:17">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1176,46 +1191,70 @@
       <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="2" spans="1:13">
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17">
       <c r="A2" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B2" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C2" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="D2" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="E2" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="F2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G2" t="s">
-        <v>19</v>
-      </c>
-      <c r="H2" t="s">
-        <v>20</v>
+        <v>22</v>
+      </c>
+      <c r="G2">
+        <v>11223</v>
+      </c>
+      <c r="H2">
+        <v>94</v>
       </c>
       <c r="I2" t="s">
-        <v>21</v>
-      </c>
-      <c r="J2" t="s">
-        <v>22</v>
+        <v>23</v>
+      </c>
+      <c r="J2">
+        <v>1496</v>
       </c>
       <c r="K2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="L2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="M2" t="s">
-        <v>25</v>
+        <v>26</v>
+      </c>
+      <c r="N2" t="s">
+        <v>27</v>
+      </c>
+      <c r="O2" t="s">
+        <v>28</v>
+      </c>
+      <c r="P2" t="s">
+        <v>29</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -1230,102 +1269,102 @@
   <sheetData>
     <row r="1" spans="1:30">
       <c r="A1" s="1" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="U1" s="1" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="V1" s="1" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="W1" s="1" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="X1" s="1" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="Y1" s="1" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="Z1" s="1" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="AA1" s="1" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="AB1" s="1" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="AC1" s="1" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="AD1" s="1" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
     </row>
     <row r="2" spans="1:30">
       <c r="A2" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B2" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="C2" s="2">
         <v>44023.34644167824</v>
@@ -1343,13 +1382,13 @@
         <v>0</v>
       </c>
       <c r="H2" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="I2" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="J2" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="K2">
         <v>204</v>
@@ -1385,7 +1424,7 @@
         <v>4.53333333</v>
       </c>
       <c r="V2" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="X2">
         <v>4.533333</v>
@@ -1396,10 +1435,10 @@
     </row>
     <row r="3" spans="1:30">
       <c r="A3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B3" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="C3" s="2">
         <v>44023.34667440972</v>
@@ -1417,13 +1456,13 @@
         <v>26</v>
       </c>
       <c r="H3" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="I3" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="J3" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="K3">
         <v>214</v>
@@ -1447,7 +1486,7 @@
         <v>6.66666667</v>
       </c>
       <c r="V3" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="W3">
         <v>0.035556</v>
@@ -1470,10 +1509,10 @@
     </row>
     <row r="4" spans="1:30">
       <c r="A4" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B4" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="C4" s="2">
         <v>44023.34674237268</v>
@@ -1491,13 +1530,13 @@
         <v>30</v>
       </c>
       <c r="H4" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="I4" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="J4" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="K4">
         <v>209</v>
@@ -1533,7 +1572,7 @@
         <v>14.8</v>
       </c>
       <c r="V4" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="W4">
         <v>0.271111</v>
@@ -1562,10 +1601,10 @@
     </row>
     <row r="5" spans="1:30">
       <c r="A5" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B5" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="C5" s="2">
         <v>44023.34702186342</v>
@@ -1583,13 +1622,13 @@
         <v>56</v>
       </c>
       <c r="H5" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="I5" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="J5" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="K5">
         <v>210</v>
@@ -1613,7 +1652,7 @@
         <v>16.73333333</v>
       </c>
       <c r="V5" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="W5">
         <v>0.064444</v>
@@ -1642,10 +1681,10 @@
     </row>
     <row r="6" spans="1:30">
       <c r="A6" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B6" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="C6" s="2">
         <v>44023.34707267361</v>
@@ -1663,13 +1702,13 @@
         <v>60</v>
       </c>
       <c r="H6" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="I6" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="J6" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="K6">
         <v>211</v>
@@ -1705,7 +1744,7 @@
         <v>16.5</v>
       </c>
       <c r="V6" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="W6">
         <v>-0.007778</v>
@@ -1734,10 +1773,10 @@
     </row>
     <row r="7" spans="1:30">
       <c r="A7" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B7" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="C7" s="2">
         <v>44023.3473683912</v>
@@ -1755,13 +1794,13 @@
         <v>86</v>
       </c>
       <c r="H7" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="I7" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="J7" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="K7">
         <v>165</v>
@@ -1785,7 +1824,7 @@
         <v>17.16666667</v>
       </c>
       <c r="V7" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="W7">
         <v>0.022222</v>
@@ -1814,10 +1853,10 @@
     </row>
     <row r="8" spans="1:30">
       <c r="A8" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B8" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="C8" s="2">
         <v>44023.34744381945</v>
@@ -1835,13 +1874,13 @@
         <v>90</v>
       </c>
       <c r="H8" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="I8" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="J8" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="K8">
         <v>157</v>
@@ -1877,7 +1916,7 @@
         <v>12.75</v>
       </c>
       <c r="V8" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="W8">
         <v>-0.036806</v>
@@ -1906,10 +1945,10 @@
     </row>
     <row r="9" spans="1:30">
       <c r="A9" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B9" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="C9" s="2">
         <v>44023.34741728009</v>
@@ -1927,13 +1966,13 @@
         <v>90</v>
       </c>
       <c r="H9" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="I9" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="J9" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="K9">
         <v>157</v>
@@ -1969,7 +2008,7 @@
         <v>17.23333333</v>
       </c>
       <c r="V9" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="W9">
         <v>0.149444</v>
@@ -1998,10 +2037,10 @@
     </row>
     <row r="10" spans="1:30">
       <c r="A10" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B10" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="C10" s="2">
         <v>44023.34771681713</v>
@@ -2019,13 +2058,13 @@
         <v>116</v>
       </c>
       <c r="H10" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="I10" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="J10" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="K10">
         <v>119</v>
@@ -2049,7 +2088,7 @@
         <v>16.73333333</v>
       </c>
       <c r="V10" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="W10">
         <v>-0.016667</v>
@@ -2078,10 +2117,10 @@
     </row>
     <row r="11" spans="1:30">
       <c r="A11" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B11" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="C11" s="2">
         <v>44023.34776537037</v>
@@ -2099,13 +2138,13 @@
         <v>120</v>
       </c>
       <c r="H11" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="I11" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="J11" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="K11">
         <v>118</v>
@@ -2141,7 +2180,7 @@
         <v>17.03333333</v>
       </c>
       <c r="V11" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="W11">
         <v>0.01</v>
@@ -2170,10 +2209,10 @@
     </row>
     <row r="12" spans="1:30">
       <c r="A12" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B12" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="C12" s="2">
         <v>44023.34806101852</v>
@@ -2191,13 +2230,13 @@
         <v>146</v>
       </c>
       <c r="H12" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="I12" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="J12" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="K12">
         <v>178</v>
@@ -2221,7 +2260,7 @@
         <v>15.53333333</v>
       </c>
       <c r="V12" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="W12">
         <v>-0.05</v>
@@ -2250,10 +2289,10 @@
     </row>
     <row r="13" spans="1:30">
       <c r="A13" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B13" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="C13" s="2">
         <v>44023.34813881944</v>
@@ -2271,13 +2310,13 @@
         <v>150</v>
       </c>
       <c r="H13" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="I13" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="J13" t="s">
-        <v>118</v>
+        <v>123</v>
       </c>
       <c r="K13">
         <v>103</v>
@@ -2313,7 +2352,7 @@
         <v>15.85</v>
       </c>
       <c r="V13" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="W13">
         <v>0.005278</v>
@@ -2342,10 +2381,10 @@
     </row>
     <row r="14" spans="1:30">
       <c r="A14" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B14" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="C14" s="2">
         <v>44023.34811263889</v>
@@ -2363,13 +2402,13 @@
         <v>150</v>
       </c>
       <c r="H14" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="I14" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="J14" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="K14">
         <v>112</v>
@@ -2405,7 +2444,7 @@
         <v>15.1</v>
       </c>
       <c r="V14" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="W14">
         <v>-0.025</v>
@@ -2434,10 +2473,10 @@
     </row>
     <row r="15" spans="1:30">
       <c r="A15" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B15" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="C15" s="2">
         <v>44023.3484072338</v>
@@ -2455,13 +2494,13 @@
         <v>176</v>
       </c>
       <c r="H15" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="I15" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="J15" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="K15">
         <v>149</v>
@@ -2485,7 +2524,7 @@
         <v>13.8</v>
       </c>
       <c r="V15" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="W15">
         <v>-0.043333</v>
@@ -2514,10 +2553,10 @@
     </row>
     <row r="16" spans="1:30">
       <c r="A16" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B16" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="C16" s="2">
         <v>44023.3484581713</v>
@@ -2535,13 +2574,13 @@
         <v>180</v>
       </c>
       <c r="H16" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="I16" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="J16" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="K16">
         <v>137</v>
@@ -2577,7 +2616,7 @@
         <v>13.8</v>
       </c>
       <c r="V16" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="W16">
         <v>0</v>
@@ -2606,10 +2645,10 @@
     </row>
     <row r="17" spans="1:30">
       <c r="A17" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B17" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="C17" s="2">
         <v>44023.34846752314</v>
@@ -2627,13 +2666,13 @@
         <v>180</v>
       </c>
       <c r="H17" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="I17" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="J17" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="K17">
         <v>134</v>
@@ -2669,7 +2708,7 @@
         <v>14.43333333</v>
       </c>
       <c r="V17" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="W17">
         <v>0.021111</v>
@@ -2698,10 +2737,10 @@
     </row>
     <row r="18" spans="1:30">
       <c r="A18" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="C18" s="2">
         <v>44023.34880686343</v>
@@ -2719,13 +2758,13 @@
         <v>210</v>
       </c>
       <c r="H18" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="I18" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="J18" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="K18">
         <v>95</v>
@@ -2761,7 +2800,7 @@
         <v>13.33333333</v>
       </c>
       <c r="V18" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="W18">
         <v>-0.036667</v>
@@ -2790,10 +2829,10 @@
     </row>
     <row r="19" spans="1:30">
       <c r="A19" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B19" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="C19" s="2">
         <v>44023.34883809028</v>
@@ -2811,13 +2850,13 @@
         <v>210</v>
       </c>
       <c r="H19" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="I19" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="J19" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="K19">
         <v>100</v>
@@ -2853,7 +2892,7 @@
         <v>12.53333333</v>
       </c>
       <c r="V19" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="W19">
         <v>-0.026667</v>
@@ -2882,10 +2921,10 @@
     </row>
     <row r="20" spans="1:30">
       <c r="A20" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B20" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="C20" s="2">
         <v>44023.34915288194</v>
@@ -2903,13 +2942,13 @@
         <v>240</v>
       </c>
       <c r="H20" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="I20" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="J20" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="K20">
         <v>106</v>
@@ -2945,7 +2984,7 @@
         <v>15.6</v>
       </c>
       <c r="V20" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="W20">
         <v>0.102222</v>
@@ -2974,10 +3013,10 @@
     </row>
     <row r="21" spans="1:30">
       <c r="A21" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B21" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="C21" s="2">
         <v>44023.34916229167</v>
@@ -2995,13 +3034,13 @@
         <v>240</v>
       </c>
       <c r="H21" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="I21" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="J21" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="K21">
         <v>111</v>
@@ -3037,7 +3076,7 @@
         <v>14.9</v>
       </c>
       <c r="V21" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="W21">
         <v>-0.023333</v>
@@ -3066,10 +3105,10 @@
     </row>
     <row r="22" spans="1:30">
       <c r="A22" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B22" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="C22" s="2">
         <v>44023.34945041667</v>
@@ -3087,13 +3126,13 @@
         <v>266</v>
       </c>
       <c r="H22" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="I22" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="J22" t="s">
-        <v>127</v>
+        <v>132</v>
       </c>
       <c r="K22">
         <v>109</v>
@@ -3117,7 +3156,7 @@
         <v>14.51111111</v>
       </c>
       <c r="V22" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="W22">
         <v>-0.004321</v>
@@ -3146,10 +3185,10 @@
     </row>
     <row r="23" spans="1:30">
       <c r="A23" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B23" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="C23" s="2">
         <v>44023.34949959491</v>
@@ -3167,13 +3206,13 @@
         <v>270</v>
       </c>
       <c r="H23" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="I23" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="J23" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="K23">
         <v>102</v>
@@ -3209,7 +3248,7 @@
         <v>14.43333333</v>
       </c>
       <c r="V23" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="W23">
         <v>-0.002593</v>
@@ -3238,10 +3277,10 @@
     </row>
     <row r="24" spans="1:30">
       <c r="A24" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B24" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="C24" s="2">
         <v>44023.34952732639</v>
@@ -3259,13 +3298,13 @@
         <v>270</v>
       </c>
       <c r="H24" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="I24" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="J24" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
       <c r="K24">
         <v>104</v>
@@ -3301,7 +3340,7 @@
         <v>15.36666667</v>
       </c>
       <c r="V24" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="W24">
         <v>0.031111</v>
@@ -3330,10 +3369,10 @@
     </row>
     <row r="25" spans="1:30">
       <c r="A25" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B25" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="C25" s="2">
         <v>44023.34979804398</v>
@@ -3351,13 +3390,13 @@
         <v>296</v>
       </c>
       <c r="H25" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="I25" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="J25" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
       <c r="K25">
         <v>128</v>
@@ -3381,7 +3420,7 @@
         <v>12.9</v>
       </c>
       <c r="V25" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="W25">
         <v>-0.082222</v>
@@ -3410,10 +3449,10 @@
     </row>
     <row r="26" spans="1:30">
       <c r="A26" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B26" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="C26" s="2">
         <v>44023.34984708334</v>
@@ -3431,13 +3470,13 @@
         <v>300</v>
       </c>
       <c r="H26" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="I26" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="J26" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
       <c r="K26">
         <v>111</v>
@@ -3473,7 +3512,7 @@
         <v>13.63333333</v>
       </c>
       <c r="V26" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="W26">
         <v>0.024444</v>
@@ -3502,10 +3541,10 @@
     </row>
     <row r="27" spans="1:30">
       <c r="A27" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B27" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="C27" s="2">
         <v>44023.35019421297</v>
@@ -3523,13 +3562,13 @@
         <v>330</v>
       </c>
       <c r="H27" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="I27" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="J27" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="K27">
         <v>122</v>
@@ -3565,7 +3604,7 @@
         <v>14.06666667</v>
       </c>
       <c r="V27" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="W27">
         <v>0.014444</v>
@@ -3594,10 +3633,10 @@
     </row>
     <row r="28" spans="1:30">
       <c r="A28" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B28" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="C28" s="2">
         <v>44023.3502215625</v>
@@ -3615,13 +3654,13 @@
         <v>330</v>
       </c>
       <c r="H28" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="I28" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="J28" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
       <c r="K28">
         <v>125</v>
@@ -3657,7 +3696,7 @@
         <v>13.7</v>
       </c>
       <c r="V28" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="W28">
         <v>-0.006111</v>
@@ -3686,10 +3725,10 @@
     </row>
     <row r="29" spans="1:30">
       <c r="A29" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B29" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="C29" s="2">
         <v>44023.35055107639</v>
@@ -3707,13 +3746,13 @@
         <v>360</v>
       </c>
       <c r="H29" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="I29" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="J29" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="K29">
         <v>121</v>
@@ -3749,7 +3788,7 @@
         <v>9.5</v>
       </c>
       <c r="V29" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="W29">
         <v>-0.14</v>
@@ -3778,10 +3817,10 @@
     </row>
     <row r="30" spans="1:30">
       <c r="A30" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B30" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="C30" s="2">
         <v>44023.35054172454</v>
@@ -3799,13 +3838,13 @@
         <v>360</v>
       </c>
       <c r="H30" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="I30" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="J30" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="K30">
         <v>123</v>
@@ -3841,7 +3880,7 @@
         <v>8.16666667</v>
       </c>
       <c r="V30" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="W30">
         <v>-0.044444</v>
@@ -3870,10 +3909,10 @@
     </row>
     <row r="31" spans="1:30">
       <c r="A31" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B31" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="C31" s="2">
         <v>44023.35083818287</v>
@@ -3891,13 +3930,13 @@
         <v>386</v>
       </c>
       <c r="H31" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="I31" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="J31" t="s">
-        <v>136</v>
+        <v>141</v>
       </c>
       <c r="K31">
         <v>125</v>
@@ -3921,7 +3960,7 @@
         <v>9.811111110000001</v>
       </c>
       <c r="V31" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="W31">
         <v>0.018272</v>
@@ -3950,10 +3989,10 @@
     </row>
     <row r="32" spans="1:30">
       <c r="A32" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B32" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="C32" s="2">
         <v>44023.35091582176</v>
@@ -3971,13 +4010,13 @@
         <v>389</v>
       </c>
       <c r="H32" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="I32" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="J32" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="K32">
         <v>117</v>
@@ -4013,7 +4052,7 @@
         <v>4.03448276</v>
       </c>
       <c r="V32" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="W32">
         <v>-0.199194</v>
@@ -4042,10 +4081,10 @@
     </row>
     <row r="33" spans="1:30">
       <c r="A33" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B33" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="C33" s="2">
         <v>44023.35088921296</v>
@@ -4063,13 +4102,13 @@
         <v>390</v>
       </c>
       <c r="H33" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="I33" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="J33" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="K33">
         <v>117</v>
@@ -4105,7 +4144,7 @@
         <v>5.8</v>
       </c>
       <c r="V33" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="W33">
         <v>0.058851</v>
@@ -4134,10 +4173,10 @@
     </row>
     <row r="34" spans="1:30">
       <c r="A34" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B34" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="C34" s="2">
         <v>44023.35118658565</v>
@@ -4155,13 +4194,13 @@
         <v>416</v>
       </c>
       <c r="H34" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="I34" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="J34" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="K34">
         <v>109</v>
@@ -4185,7 +4224,7 @@
         <v>5.46666667</v>
       </c>
       <c r="V34" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="W34">
         <v>-0.011111</v>
@@ -4214,10 +4253,10 @@
     </row>
     <row r="35" spans="1:30">
       <c r="A35" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B35" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="C35" s="2">
         <v>44023.35123702546</v>
@@ -4235,13 +4274,13 @@
         <v>420</v>
       </c>
       <c r="H35" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="I35" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="J35" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="K35">
         <v>110</v>
@@ -4277,7 +4316,7 @@
         <v>5.4</v>
       </c>
       <c r="V35" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="W35">
         <v>-0.002222</v>
@@ -4306,10 +4345,10 @@
     </row>
     <row r="36" spans="1:30">
       <c r="A36" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B36" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="C36" s="2">
         <v>44023.35124731481</v>
@@ -4327,13 +4366,13 @@
         <v>420</v>
       </c>
       <c r="H36" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="I36" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="J36" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="K36">
         <v>111</v>
@@ -4369,7 +4408,7 @@
         <v>6.06451613</v>
       </c>
       <c r="V36" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="W36">
         <v>0.021436</v>
@@ -4398,10 +4437,10 @@
     </row>
     <row r="37" spans="1:30">
       <c r="A37" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B37" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="C37" s="2">
         <v>44023.35153310185</v>
@@ -4419,13 +4458,13 @@
         <v>446</v>
       </c>
       <c r="H37" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="I37" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="J37" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="K37">
         <v>114</v>
@@ -4449,7 +4488,7 @@
         <v>5.66666667</v>
       </c>
       <c r="V37" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="W37">
         <v>-0.013262</v>
@@ -4478,10 +4517,10 @@
     </row>
     <row r="38" spans="1:30">
       <c r="A38" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B38" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="C38" s="2">
         <v>44023.35158375</v>
@@ -4499,13 +4538,13 @@
         <v>450</v>
       </c>
       <c r="H38" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="I38" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="J38" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="K38">
         <v>116</v>
@@ -4541,7 +4580,7 @@
         <v>5.8</v>
       </c>
       <c r="V38" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="W38">
         <v>0.004444</v>
@@ -4570,10 +4609,10 @@
     </row>
     <row r="39" spans="1:30">
       <c r="A39" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B39" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="C39" s="2">
         <v>44023.35161115741</v>
@@ -4591,13 +4630,13 @@
         <v>450</v>
       </c>
       <c r="H39" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="I39" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="J39" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="K39">
         <v>114</v>
@@ -4633,7 +4672,7 @@
         <v>6.16666667</v>
       </c>
       <c r="V39" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="W39">
         <v>0.012222</v>
@@ -4662,10 +4701,10 @@
     </row>
     <row r="40" spans="1:30">
       <c r="A40" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B40" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="C40" s="2">
         <v>44023.35187935185</v>
@@ -4683,13 +4722,13 @@
         <v>476</v>
       </c>
       <c r="H40" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="I40" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="J40" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
       <c r="K40">
         <v>118</v>
@@ -4713,7 +4752,7 @@
         <v>5.7</v>
       </c>
       <c r="V40" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="W40">
         <v>-0.015556</v>
@@ -4742,10 +4781,10 @@
     </row>
     <row r="41" spans="1:30">
       <c r="A41" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B41" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="C41" s="2">
         <v>44023.35193064815</v>
@@ -4763,13 +4802,13 @@
         <v>480</v>
       </c>
       <c r="H41" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="I41" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="J41" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
       <c r="K41">
         <v>118</v>
@@ -4805,7 +4844,7 @@
         <v>5.36666667</v>
       </c>
       <c r="V41" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="W41">
         <v>-0.011111</v>
@@ -4834,10 +4873,10 @@
     </row>
     <row r="42" spans="1:30">
       <c r="A42" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B42" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="C42" s="2">
         <v>44023.35194001158</v>
@@ -4855,13 +4894,13 @@
         <v>480</v>
       </c>
       <c r="H42" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="I42" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="J42" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="K42">
         <v>118</v>
@@ -4897,7 +4936,7 @@
         <v>5.3</v>
       </c>
       <c r="V42" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="W42">
         <v>-0.002222</v>
@@ -4926,10 +4965,10 @@
     </row>
     <row r="43" spans="1:30">
       <c r="A43" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B43" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="C43" s="2">
         <v>44023.35227842593</v>
@@ -4947,13 +4986,13 @@
         <v>510</v>
       </c>
       <c r="H43" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="I43" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="J43" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="K43">
         <v>120</v>
@@ -4989,7 +5028,7 @@
         <v>3.76666667</v>
       </c>
       <c r="V43" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="W43">
         <v>-0.051111</v>
@@ -5018,10 +5057,10 @@
     </row>
     <row r="44" spans="1:30">
       <c r="A44" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B44" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="C44" s="2">
         <v>44023.35230556713</v>
@@ -5039,13 +5078,13 @@
         <v>510</v>
       </c>
       <c r="H44" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="I44" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="J44" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
       <c r="K44">
         <v>119</v>
@@ -5081,7 +5120,7 @@
         <v>3.06666667</v>
       </c>
       <c r="V44" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="W44">
         <v>-0.023333</v>
@@ -5110,10 +5149,10 @@
     </row>
     <row r="45" spans="1:30">
       <c r="A45" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B45" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="C45" s="2">
         <v>44023.35257471065</v>
@@ -5131,13 +5170,13 @@
         <v>536</v>
       </c>
       <c r="H45" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="I45" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="J45" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="K45">
         <v>121</v>
@@ -5161,7 +5200,7 @@
         <v>3.38333333</v>
       </c>
       <c r="V45" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="W45">
         <v>0.005278</v>
@@ -5190,10 +5229,10 @@
     </row>
     <row r="46" spans="1:30">
       <c r="A46" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B46" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="C46" s="2">
         <v>44023.35262537037</v>
@@ -5211,13 +5250,13 @@
         <v>540</v>
       </c>
       <c r="H46" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="I46" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="J46" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="K46">
         <v>121</v>
@@ -5253,7 +5292,7 @@
         <v>2.73333333</v>
       </c>
       <c r="V46" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="W46">
         <v>-0.021667</v>
@@ -5282,10 +5321,10 @@
     </row>
     <row r="47" spans="1:30">
       <c r="A47" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B47" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="C47" s="2">
         <v>44023.35292203704</v>
@@ -5303,13 +5342,13 @@
         <v>566</v>
       </c>
       <c r="H47" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="I47" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="J47" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="K47">
         <v>121</v>
@@ -5333,7 +5372,7 @@
         <v>1.43333333</v>
       </c>
       <c r="V47" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="W47">
         <v>-0.043333</v>
@@ -5362,10 +5401,10 @@
     </row>
     <row r="48" spans="1:30">
       <c r="A48" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B48" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="C48" s="2">
         <v>44023.35297302083</v>
@@ -5383,13 +5422,13 @@
         <v>570</v>
       </c>
       <c r="H48" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="I48" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="J48" t="s">
-        <v>153</v>
+        <v>158</v>
       </c>
       <c r="K48">
         <v>121</v>
@@ -5425,7 +5464,7 @@
         <v>1.23333333</v>
       </c>
       <c r="V48" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="W48">
         <v>-0.006667</v>
@@ -5464,102 +5503,102 @@
   <sheetData>
     <row r="1" spans="1:30">
       <c r="A1" s="1" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="U1" s="1" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="V1" s="1" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="W1" s="1" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="X1" s="1" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="Y1" s="1" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="Z1" s="1" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="AA1" s="1" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="AB1" s="1" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="AC1" s="1" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="AD1" s="1" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
     </row>
     <row r="2" spans="1:30">
       <c r="A2" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B2" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="C2" s="2">
         <v>44023.35299995371</v>
@@ -5577,13 +5616,13 @@
         <v>0</v>
       </c>
       <c r="H2" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="I2" t="s">
-        <v>157</v>
+        <v>162</v>
       </c>
       <c r="J2" t="s">
-        <v>204</v>
+        <v>209</v>
       </c>
       <c r="K2">
         <v>120</v>
@@ -5619,7 +5658,7 @@
         <v>2.15</v>
       </c>
       <c r="V2" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="X2">
         <v>2.15</v>
@@ -5630,10 +5669,10 @@
     </row>
     <row r="3" spans="1:30">
       <c r="A3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B3" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="C3" s="2">
         <v>44023.35333020833</v>
@@ -5651,13 +5690,13 @@
         <v>29</v>
       </c>
       <c r="H3" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="I3" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="J3" t="s">
-        <v>205</v>
+        <v>210</v>
       </c>
       <c r="K3">
         <v>121</v>
@@ -5693,7 +5732,7 @@
         <v>-0.10344828</v>
       </c>
       <c r="V3" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="W3">
         <v>-0.077705</v>
@@ -5716,10 +5755,10 @@
     </row>
     <row r="4" spans="1:30">
       <c r="A4" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B4" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="C4" s="2">
         <v>44023.35331981481</v>
@@ -5737,13 +5776,13 @@
         <v>30</v>
       </c>
       <c r="H4" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="I4" t="s">
-        <v>159</v>
+        <v>164</v>
       </c>
       <c r="J4" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
       <c r="K4">
         <v>121</v>
@@ -5779,7 +5818,7 @@
         <v>-0.7</v>
       </c>
       <c r="V4" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="W4">
         <v>-0.019885</v>
@@ -5808,10 +5847,10 @@
     </row>
     <row r="5" spans="1:30">
       <c r="A5" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B5" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="C5" s="2">
         <v>44023.35361952546</v>
@@ -5829,13 +5868,13 @@
         <v>56</v>
       </c>
       <c r="H5" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="I5" t="s">
-        <v>160</v>
+        <v>165</v>
       </c>
       <c r="J5" t="s">
-        <v>207</v>
+        <v>212</v>
       </c>
       <c r="K5">
         <v>122</v>
@@ -5859,7 +5898,7 @@
         <v>-1.41666667</v>
       </c>
       <c r="V5" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="W5">
         <v>-0.011944</v>
@@ -5888,10 +5927,10 @@
     </row>
     <row r="6" spans="1:30">
       <c r="A6" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B6" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="C6" s="2">
         <v>44023.35369785879</v>
@@ -5909,13 +5948,13 @@
         <v>60</v>
       </c>
       <c r="H6" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="I6" t="s">
-        <v>161</v>
+        <v>166</v>
       </c>
       <c r="J6" t="s">
-        <v>208</v>
+        <v>213</v>
       </c>
       <c r="K6">
         <v>121</v>
@@ -5951,7 +5990,7 @@
         <v>-3.41935484</v>
       </c>
       <c r="V6" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="W6">
         <v>-0.06460299999999999</v>
@@ -5980,10 +6019,10 @@
     </row>
     <row r="7" spans="1:30">
       <c r="A7" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B7" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="C7" s="2">
         <v>44023.35366663194</v>
@@ -6001,13 +6040,13 @@
         <v>60</v>
       </c>
       <c r="H7" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="I7" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="J7" t="s">
-        <v>209</v>
+        <v>214</v>
       </c>
       <c r="K7">
         <v>122</v>
@@ -6043,7 +6082,7 @@
         <v>-2.8</v>
       </c>
       <c r="V7" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="W7">
         <v>0.020645</v>
@@ -6072,10 +6111,10 @@
     </row>
     <row r="8" spans="1:30">
       <c r="A8" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B8" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="C8" s="2">
         <v>44023.35396462963</v>
@@ -6093,13 +6132,13 @@
         <v>86</v>
       </c>
       <c r="H8" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="I8" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="J8" t="s">
-        <v>210</v>
+        <v>215</v>
       </c>
       <c r="K8">
         <v>122</v>
@@ -6123,7 +6162,7 @@
         <v>-3.3</v>
       </c>
       <c r="V8" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="W8">
         <v>-0.016667</v>
@@ -6152,10 +6191,10 @@
     </row>
     <row r="9" spans="1:30">
       <c r="A9" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B9" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="C9" s="2">
         <v>44023.35401414352</v>
@@ -6173,13 +6212,13 @@
         <v>90</v>
       </c>
       <c r="H9" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="I9" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
       <c r="J9" t="s">
-        <v>211</v>
+        <v>216</v>
       </c>
       <c r="K9">
         <v>122</v>
@@ -6215,7 +6254,7 @@
         <v>-3.43333333</v>
       </c>
       <c r="V9" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="W9">
         <v>-0.004444</v>
@@ -6244,10 +6283,10 @@
     </row>
     <row r="10" spans="1:30">
       <c r="A10" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B10" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="C10" s="2">
         <v>44023.35431188657</v>
@@ -6265,13 +6304,13 @@
         <v>116</v>
       </c>
       <c r="H10" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="I10" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
       <c r="J10" t="s">
-        <v>212</v>
+        <v>217</v>
       </c>
       <c r="K10">
         <v>122</v>
@@ -6295,7 +6334,7 @@
         <v>-4.36666667</v>
       </c>
       <c r="V10" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="W10">
         <v>-0.031111</v>
@@ -6324,10 +6363,10 @@
     </row>
     <row r="11" spans="1:30">
       <c r="A11" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B11" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="C11" s="2">
         <v>44023.35436167824</v>
@@ -6345,13 +6384,13 @@
         <v>120</v>
       </c>
       <c r="H11" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="I11" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="J11" t="s">
-        <v>213</v>
+        <v>218</v>
       </c>
       <c r="K11">
         <v>119</v>
@@ -6387,7 +6426,7 @@
         <v>-4.53333333</v>
       </c>
       <c r="V11" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="W11">
         <v>-0.005556</v>
@@ -6416,10 +6455,10 @@
     </row>
     <row r="12" spans="1:30">
       <c r="A12" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B12" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="C12" s="2">
         <v>44023.35438840277</v>
@@ -6437,13 +6476,13 @@
         <v>120</v>
       </c>
       <c r="H12" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="I12" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
       <c r="J12" t="s">
-        <v>214</v>
+        <v>219</v>
       </c>
       <c r="K12">
         <v>119</v>
@@ -6479,7 +6518,7 @@
         <v>-4.01666667</v>
       </c>
       <c r="V12" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="W12">
         <v>0.008611000000000001</v>
@@ -6508,10 +6547,10 @@
     </row>
     <row r="13" spans="1:30">
       <c r="A13" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B13" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="C13" s="2">
         <v>44023.35470967593</v>
@@ -6529,13 +6568,13 @@
         <v>150</v>
       </c>
       <c r="H13" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="I13" t="s">
-        <v>168</v>
+        <v>173</v>
       </c>
       <c r="J13" t="s">
-        <v>215</v>
+        <v>220</v>
       </c>
       <c r="K13">
         <v>119</v>
@@ -6571,7 +6610,7 @@
         <v>-5.86666667</v>
       </c>
       <c r="V13" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="W13">
         <v>-0.061667</v>
@@ -6600,10 +6639,10 @@
     </row>
     <row r="14" spans="1:30">
       <c r="A14" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B14" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="C14" s="2">
         <v>44023.35500557871</v>
@@ -6621,13 +6660,13 @@
         <v>176</v>
       </c>
       <c r="H14" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="I14" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
       <c r="J14" t="s">
-        <v>216</v>
+        <v>221</v>
       </c>
       <c r="K14">
         <v>122</v>
@@ -6651,7 +6690,7 @@
         <v>-5.9</v>
       </c>
       <c r="V14" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="W14">
         <v>-0.000556</v>
@@ -6680,10 +6719,10 @@
     </row>
     <row r="15" spans="1:30">
       <c r="A15" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B15" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="C15" s="2">
         <v>44023.35505572917</v>
@@ -6701,13 +6740,13 @@
         <v>180</v>
       </c>
       <c r="H15" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="I15" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="J15" t="s">
-        <v>217</v>
+        <v>222</v>
       </c>
       <c r="K15">
         <v>119</v>
@@ -6743,7 +6782,7 @@
         <v>-5.96666667</v>
       </c>
       <c r="V15" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="W15">
         <v>-0.002222</v>
@@ -6772,10 +6811,10 @@
     </row>
     <row r="16" spans="1:30">
       <c r="A16" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B16" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="C16" s="2">
         <v>44023.35535255787</v>
@@ -6793,13 +6832,13 @@
         <v>206</v>
       </c>
       <c r="H16" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="I16" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
       <c r="J16" t="s">
-        <v>218</v>
+        <v>223</v>
       </c>
       <c r="K16">
         <v>118</v>
@@ -6823,7 +6862,7 @@
         <v>-5.7</v>
       </c>
       <c r="V16" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="W16">
         <v>0.008888999999999999</v>
@@ -6852,10 +6891,10 @@
     </row>
     <row r="17" spans="1:30">
       <c r="A17" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B17" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="C17" s="2">
         <v>44023.3554027662</v>
@@ -6873,13 +6912,13 @@
         <v>210</v>
       </c>
       <c r="H17" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="I17" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="J17" t="s">
-        <v>219</v>
+        <v>224</v>
       </c>
       <c r="K17">
         <v>124</v>
@@ -6915,7 +6954,7 @@
         <v>-5.73333333</v>
       </c>
       <c r="V17" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="W17">
         <v>-0.001111</v>
@@ -6944,10 +6983,10 @@
     </row>
     <row r="18" spans="1:30">
       <c r="A18" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="C18" s="2">
         <v>44023.35569953704</v>
@@ -6965,13 +7004,13 @@
         <v>236</v>
       </c>
       <c r="H18" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="I18" t="s">
-        <v>173</v>
+        <v>178</v>
       </c>
       <c r="J18" t="s">
-        <v>220</v>
+        <v>225</v>
       </c>
       <c r="K18">
         <v>113</v>
@@ -6995,7 +7034,7 @@
         <v>-7.1</v>
       </c>
       <c r="V18" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="W18">
         <v>-0.045556</v>
@@ -7024,10 +7063,10 @@
     </row>
     <row r="19" spans="1:30">
       <c r="A19" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B19" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="C19" s="2">
         <v>44023.35575015046</v>
@@ -7045,13 +7084,13 @@
         <v>240</v>
       </c>
       <c r="H19" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="I19" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="J19" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="K19">
         <v>118</v>
@@ -7087,7 +7126,7 @@
         <v>-7.3</v>
       </c>
       <c r="V19" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="W19">
         <v>-0.006667</v>
@@ -7116,10 +7155,10 @@
     </row>
     <row r="20" spans="1:30">
       <c r="A20" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B20" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="C20" s="2">
         <v>44023.35604671296</v>
@@ -7137,13 +7176,13 @@
         <v>266</v>
       </c>
       <c r="H20" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="I20" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="J20" t="s">
-        <v>222</v>
+        <v>227</v>
       </c>
       <c r="K20">
         <v>107</v>
@@ -7167,7 +7206,7 @@
         <v>-8.43333333</v>
       </c>
       <c r="V20" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="W20">
         <v>-0.037778</v>
@@ -7196,10 +7235,10 @@
     </row>
     <row r="21" spans="1:30">
       <c r="A21" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B21" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="C21" s="2">
         <v>44023.35609765046</v>
@@ -7217,13 +7256,13 @@
         <v>270</v>
       </c>
       <c r="H21" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="I21" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="J21" t="s">
-        <v>223</v>
+        <v>228</v>
       </c>
       <c r="K21">
         <v>109</v>
@@ -7259,7 +7298,7 @@
         <v>-8.199999999999999</v>
       </c>
       <c r="V21" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="W21">
         <v>0.007778</v>
@@ -7288,10 +7327,10 @@
     </row>
     <row r="22" spans="1:30">
       <c r="A22" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B22" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="C22" s="2">
         <v>44023.35647199074</v>
@@ -7309,13 +7348,13 @@
         <v>300</v>
       </c>
       <c r="H22" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="I22" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="J22" t="s">
-        <v>224</v>
+        <v>229</v>
       </c>
       <c r="K22">
         <v>102</v>
@@ -7351,7 +7390,7 @@
         <v>-6.95</v>
       </c>
       <c r="V22" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="W22">
         <v>0.006944</v>
@@ -7380,10 +7419,10 @@
     </row>
     <row r="23" spans="1:30">
       <c r="A23" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B23" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="C23" s="2">
         <v>44023.35644489584</v>
@@ -7401,13 +7440,13 @@
         <v>300</v>
       </c>
       <c r="H23" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="I23" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="J23" t="s">
-        <v>225</v>
+        <v>230</v>
       </c>
       <c r="K23">
         <v>99</v>
@@ -7443,7 +7482,7 @@
         <v>-9.133333329999999</v>
       </c>
       <c r="V23" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="W23">
         <v>-0.072778</v>
@@ -7472,10 +7511,10 @@
     </row>
     <row r="24" spans="1:30">
       <c r="A24" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B24" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="C24" s="2">
         <v>44023.35674206018</v>
@@ -7493,13 +7532,13 @@
         <v>326</v>
       </c>
       <c r="H24" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="I24" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="J24" t="s">
-        <v>226</v>
+        <v>231</v>
       </c>
       <c r="K24">
         <v>102</v>
@@ -7523,7 +7562,7 @@
         <v>-9.516666669999999</v>
       </c>
       <c r="V24" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="W24">
         <v>-0.006389</v>
@@ -7552,10 +7591,10 @@
     </row>
     <row r="25" spans="1:30">
       <c r="A25" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B25" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="C25" s="2">
         <v>44023.35679211806</v>
@@ -7573,13 +7612,13 @@
         <v>330</v>
       </c>
       <c r="H25" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="I25" t="s">
-        <v>180</v>
+        <v>185</v>
       </c>
       <c r="J25" t="s">
-        <v>227</v>
+        <v>232</v>
       </c>
       <c r="K25">
         <v>98</v>
@@ -7615,7 +7654,7 @@
         <v>-10.5</v>
       </c>
       <c r="V25" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="W25">
         <v>-0.032778</v>
@@ -7644,10 +7683,10 @@
     </row>
     <row r="26" spans="1:30">
       <c r="A26" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B26" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="C26" s="2">
         <v>44023.35713885417</v>
@@ -7665,13 +7704,13 @@
         <v>360</v>
       </c>
       <c r="H26" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="I26" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
       <c r="J26" t="s">
-        <v>228</v>
+        <v>233</v>
       </c>
       <c r="K26">
         <v>98</v>
@@ -7707,7 +7746,7 @@
         <v>-11.23333333</v>
       </c>
       <c r="V26" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="W26">
         <v>-0.024444</v>
@@ -7736,10 +7775,10 @@
     </row>
     <row r="27" spans="1:30">
       <c r="A27" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B27" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="C27" s="2">
         <v>44023.35743622685</v>
@@ -7757,13 +7796,13 @@
         <v>386</v>
       </c>
       <c r="H27" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="I27" t="s">
-        <v>182</v>
+        <v>187</v>
       </c>
       <c r="J27" t="s">
-        <v>229</v>
+        <v>234</v>
       </c>
       <c r="K27">
         <v>118</v>
@@ -7787,7 +7826,7 @@
         <v>-10.83333333</v>
       </c>
       <c r="V27" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="W27">
         <v>0.006667</v>
@@ -7816,10 +7855,10 @@
     </row>
     <row r="28" spans="1:30">
       <c r="A28" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B28" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="C28" s="2">
         <v>44023.35748664352</v>
@@ -7837,13 +7876,13 @@
         <v>390</v>
       </c>
       <c r="H28" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="I28" t="s">
-        <v>183</v>
+        <v>188</v>
       </c>
       <c r="J28" t="s">
-        <v>230</v>
+        <v>235</v>
       </c>
       <c r="K28">
         <v>118</v>
@@ -7879,7 +7918,7 @@
         <v>-10.16666667</v>
       </c>
       <c r="V28" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="W28">
         <v>0.022222</v>
@@ -7908,10 +7947,10 @@
     </row>
     <row r="29" spans="1:30">
       <c r="A29" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B29" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="C29" s="2">
         <v>44023.35778332176</v>
@@ -7929,13 +7968,13 @@
         <v>416</v>
       </c>
       <c r="H29" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="I29" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
       <c r="J29" t="s">
-        <v>231</v>
+        <v>236</v>
       </c>
       <c r="K29">
         <v>84</v>
@@ -7959,7 +7998,7 @@
         <v>-11.7</v>
       </c>
       <c r="V29" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="W29">
         <v>-0.051111</v>
@@ -7988,10 +8027,10 @@
     </row>
     <row r="30" spans="1:30">
       <c r="A30" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B30" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="C30" s="2">
         <v>44023.35783324074</v>
@@ -8009,13 +8048,13 @@
         <v>420</v>
       </c>
       <c r="H30" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="I30" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
       <c r="J30" t="s">
-        <v>232</v>
+        <v>237</v>
       </c>
       <c r="K30">
         <v>119</v>
@@ -8051,7 +8090,7 @@
         <v>-11.93333333</v>
       </c>
       <c r="V30" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="W30">
         <v>-0.007778</v>
@@ -8080,10 +8119,10 @@
     </row>
     <row r="31" spans="1:30">
       <c r="A31" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B31" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="C31" s="2">
         <v>44023.35786231481</v>
@@ -8101,13 +8140,13 @@
         <v>420</v>
       </c>
       <c r="H31" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="I31" t="s">
-        <v>186</v>
+        <v>191</v>
       </c>
       <c r="J31" t="s">
-        <v>233</v>
+        <v>238</v>
       </c>
       <c r="K31">
         <v>120</v>
@@ -8143,7 +8182,7 @@
         <v>-11.075</v>
       </c>
       <c r="V31" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="W31">
         <v>0.007153</v>
@@ -8172,10 +8211,10 @@
     </row>
     <row r="32" spans="1:30">
       <c r="A32" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B32" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="C32" s="2">
         <v>44023.35818081019</v>
@@ -8193,13 +8232,13 @@
         <v>450</v>
       </c>
       <c r="H32" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="I32" t="s">
-        <v>187</v>
+        <v>192</v>
       </c>
       <c r="J32" t="s">
-        <v>234</v>
+        <v>239</v>
       </c>
       <c r="K32">
         <v>110</v>
@@ -8235,7 +8274,7 @@
         <v>-13.36666667</v>
       </c>
       <c r="V32" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="W32">
         <v>-0.076389</v>
@@ -8264,10 +8303,10 @@
     </row>
     <row r="33" spans="1:30">
       <c r="A33" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B33" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="C33" s="2">
         <v>44023.35819207176</v>
@@ -8285,13 +8324,13 @@
         <v>450</v>
       </c>
       <c r="H33" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="I33" t="s">
-        <v>188</v>
+        <v>193</v>
       </c>
       <c r="J33" t="s">
-        <v>235</v>
+        <v>240</v>
       </c>
       <c r="K33">
         <v>115</v>
@@ -8327,7 +8366,7 @@
         <v>-13.3</v>
       </c>
       <c r="V33" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="W33">
         <v>0.002222</v>
@@ -8356,10 +8395,10 @@
     </row>
     <row r="34" spans="1:30">
       <c r="A34" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B34" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="C34" s="2">
         <v>44023.35847700232</v>
@@ -8377,13 +8416,13 @@
         <v>476</v>
       </c>
       <c r="H34" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="I34" t="s">
-        <v>189</v>
+        <v>194</v>
       </c>
       <c r="J34" t="s">
-        <v>236</v>
+        <v>241</v>
       </c>
       <c r="K34">
         <v>95</v>
@@ -8407,7 +8446,7 @@
         <v>-12.9</v>
       </c>
       <c r="V34" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="W34">
         <v>0.006667</v>
@@ -8436,10 +8475,10 @@
     </row>
     <row r="35" spans="1:30">
       <c r="A35" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B35" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="C35" s="2">
         <v>44023.35852927083</v>
@@ -8457,13 +8496,13 @@
         <v>480</v>
       </c>
       <c r="H35" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="I35" t="s">
-        <v>190</v>
+        <v>195</v>
       </c>
       <c r="J35" t="s">
-        <v>237</v>
+        <v>242</v>
       </c>
       <c r="K35">
         <v>93</v>
@@ -8499,7 +8538,7 @@
         <v>-12.6</v>
       </c>
       <c r="V35" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="W35">
         <v>0.01</v>
@@ -8528,10 +8567,10 @@
     </row>
     <row r="36" spans="1:30">
       <c r="A36" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B36" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="C36" s="2">
         <v>44023.3585559375</v>
@@ -8549,13 +8588,13 @@
         <v>480</v>
       </c>
       <c r="H36" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="I36" t="s">
-        <v>191</v>
+        <v>196</v>
       </c>
       <c r="J36" t="s">
-        <v>238</v>
+        <v>243</v>
       </c>
       <c r="K36">
         <v>99</v>
@@ -8591,7 +8630,7 @@
         <v>-12.7</v>
       </c>
       <c r="V36" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="W36">
         <v>-0.003333</v>
@@ -8620,10 +8659,10 @@
     </row>
     <row r="37" spans="1:30">
       <c r="A37" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B37" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="C37" s="2">
         <v>44023.3588266088</v>
@@ -8641,13 +8680,13 @@
         <v>506</v>
       </c>
       <c r="H37" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="I37" t="s">
-        <v>192</v>
+        <v>197</v>
       </c>
       <c r="J37" t="s">
-        <v>239</v>
+        <v>244</v>
       </c>
       <c r="K37">
         <v>138</v>
@@ -8671,7 +8710,7 @@
         <v>-11.8</v>
       </c>
       <c r="V37" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="W37">
         <v>0.03</v>
@@ -8700,10 +8739,10 @@
     </row>
     <row r="38" spans="1:30">
       <c r="A38" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B38" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="C38" s="2">
         <v>44023.35887934027</v>
@@ -8721,13 +8760,13 @@
         <v>510</v>
       </c>
       <c r="H38" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="I38" t="s">
-        <v>193</v>
+        <v>198</v>
       </c>
       <c r="J38" t="s">
-        <v>240</v>
+        <v>245</v>
       </c>
       <c r="K38">
         <v>108</v>
@@ -8763,7 +8802,7 @@
         <v>-11.9</v>
       </c>
       <c r="V38" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="W38">
         <v>-0.003333</v>
@@ -8792,10 +8831,10 @@
     </row>
     <row r="39" spans="1:30">
       <c r="A39" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B39" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="C39" s="2">
         <v>44023.3591712963</v>
@@ -8813,13 +8852,13 @@
         <v>536</v>
       </c>
       <c r="H39" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="I39" t="s">
-        <v>194</v>
+        <v>199</v>
       </c>
       <c r="J39" t="s">
-        <v>241</v>
+        <v>246</v>
       </c>
       <c r="K39">
         <v>133</v>
@@ -8843,7 +8882,7 @@
         <v>-11.16666667</v>
       </c>
       <c r="V39" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="W39">
         <v>0.024444</v>
@@ -8872,10 +8911,10 @@
     </row>
     <row r="40" spans="1:30">
       <c r="A40" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B40" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="C40" s="2">
         <v>44023.35922280093</v>
@@ -8893,13 +8932,13 @@
         <v>540</v>
       </c>
       <c r="H40" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="I40" t="s">
-        <v>195</v>
+        <v>200</v>
       </c>
       <c r="J40" t="s">
-        <v>242</v>
+        <v>247</v>
       </c>
       <c r="K40">
         <v>120</v>
@@ -8935,7 +8974,7 @@
         <v>-10.9</v>
       </c>
       <c r="V40" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="W40">
         <v>0.008888999999999999</v>
@@ -8964,10 +9003,10 @@
     </row>
     <row r="41" spans="1:30">
       <c r="A41" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B41" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="C41" s="2">
         <v>44023.35952256944</v>
@@ -8985,13 +9024,13 @@
         <v>566</v>
       </c>
       <c r="H41" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="I41" t="s">
-        <v>196</v>
+        <v>201</v>
       </c>
       <c r="J41" t="s">
-        <v>243</v>
+        <v>248</v>
       </c>
       <c r="K41">
         <v>193</v>
@@ -9015,7 +9054,7 @@
         <v>-11.6</v>
       </c>
       <c r="V41" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="W41">
         <v>-0.023333</v>
@@ -9044,10 +9083,10 @@
     </row>
     <row r="42" spans="1:30">
       <c r="A42" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B42" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="C42" s="2">
         <v>44023.35956898148</v>
@@ -9065,13 +9104,13 @@
         <v>570</v>
       </c>
       <c r="H42" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="I42" t="s">
-        <v>197</v>
+        <v>202</v>
       </c>
       <c r="J42" t="s">
-        <v>244</v>
+        <v>249</v>
       </c>
       <c r="K42">
         <v>176</v>
@@ -9107,7 +9146,7 @@
         <v>-12.16666667</v>
       </c>
       <c r="V42" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="W42">
         <v>-0.018889</v>
@@ -9136,10 +9175,10 @@
     </row>
     <row r="43" spans="1:30">
       <c r="A43" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B43" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="C43" s="2">
         <v>44023.35986965278</v>
@@ -9157,13 +9196,13 @@
         <v>596</v>
       </c>
       <c r="H43" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="I43" t="s">
-        <v>198</v>
+        <v>203</v>
       </c>
       <c r="J43" t="s">
-        <v>245</v>
+        <v>250</v>
       </c>
       <c r="K43">
         <v>195</v>
@@ -9187,7 +9226,7 @@
         <v>-11.7</v>
       </c>
       <c r="V43" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="W43">
         <v>0.015556</v>
@@ -9216,10 +9255,10 @@
     </row>
     <row r="44" spans="1:30">
       <c r="A44" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B44" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="C44" s="2">
         <v>44023.35991907407</v>
@@ -9237,13 +9276,13 @@
         <v>600</v>
       </c>
       <c r="H44" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="I44" t="s">
-        <v>199</v>
+        <v>204</v>
       </c>
       <c r="J44" t="s">
-        <v>246</v>
+        <v>251</v>
       </c>
       <c r="K44">
         <v>200</v>
@@ -9279,7 +9318,7 @@
         <v>-11.13333333</v>
       </c>
       <c r="V44" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="W44">
         <v>0.018889</v>
@@ -9308,10 +9347,10 @@
     </row>
     <row r="45" spans="1:30">
       <c r="A45" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B45" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="C45" s="2">
         <v>44023.36026780093</v>
@@ -9329,13 +9368,13 @@
         <v>630</v>
       </c>
       <c r="H45" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="I45" t="s">
-        <v>200</v>
+        <v>205</v>
       </c>
       <c r="J45" t="s">
-        <v>247</v>
+        <v>252</v>
       </c>
       <c r="K45">
         <v>193</v>
@@ -9371,7 +9410,7 @@
         <v>-13.3</v>
       </c>
       <c r="V45" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="W45">
         <v>-0.07222199999999999</v>
@@ -9400,10 +9439,10 @@
     </row>
     <row r="46" spans="1:30">
       <c r="A46" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B46" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="C46" s="2">
         <v>44023.36056296296</v>
@@ -9421,13 +9460,13 @@
         <v>656</v>
       </c>
       <c r="H46" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="I46" t="s">
-        <v>201</v>
+        <v>206</v>
       </c>
       <c r="J46" t="s">
-        <v>248</v>
+        <v>253</v>
       </c>
       <c r="K46">
         <v>203</v>
@@ -9451,7 +9490,7 @@
         <v>-13.78333333</v>
       </c>
       <c r="V46" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="W46">
         <v>-0.008056000000000001</v>
@@ -9480,10 +9519,10 @@
     </row>
     <row r="47" spans="1:30">
       <c r="A47" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B47" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="C47" s="2">
         <v>44023.36061483796</v>
@@ -9501,13 +9540,13 @@
         <v>660</v>
       </c>
       <c r="H47" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="I47" t="s">
-        <v>202</v>
+        <v>207</v>
       </c>
       <c r="J47" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="K47">
         <v>193</v>
@@ -9543,7 +9582,7 @@
         <v>-14.6</v>
       </c>
       <c r="V47" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="W47">
         <v>-0.027222</v>
@@ -9572,10 +9611,10 @@
     </row>
     <row r="48" spans="1:30">
       <c r="A48" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B48" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="C48" s="2">
         <v>44023.36369013889</v>
@@ -9593,13 +9632,13 @@
         <v>926</v>
       </c>
       <c r="H48" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="I48" t="s">
-        <v>203</v>
+        <v>208</v>
       </c>
       <c r="J48" t="s">
-        <v>250</v>
+        <v>255</v>
       </c>
       <c r="K48">
         <v>204</v>
@@ -9623,7 +9662,7 @@
         <v>-1.38518519</v>
       </c>
       <c r="V48" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="W48">
         <v>0.048944</v>

</xml_diff>

<commit_message>
Updates to telemetry page, styles, and data
</commit_message>
<xml_diff>
--- a/www/flightdata/xlsx/eoss-300.xlsx
+++ b/www/flightdata/xlsx/eoss-300.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="665" uniqueCount="266">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="668" uniqueCount="268">
   <si>
     <t>flight</t>
   </si>
@@ -228,6 +228,9 @@
     <t>velocity_curvefit</t>
   </si>
   <si>
+    <t>reynolds_transition</t>
+  </si>
+  <si>
     <t>KC0D-1</t>
   </si>
   <si>
@@ -526,6 +529,9 @@
   </si>
   <si>
     <t>low Re</t>
+  </si>
+  <si>
+    <t>high_to_low</t>
   </si>
   <si>
     <t>descending</t>
@@ -1339,10 +1345,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AE48"/>
+  <dimension ref="A1:AF48"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:31">
+    <row r="1" spans="1:32">
       <c r="A1" s="1" t="s">
         <v>39</v>
       </c>
@@ -1436,13 +1442,16 @@
       <c r="AE1" s="1" t="s">
         <v>69</v>
       </c>
+      <c r="AF1" s="1" t="s">
+        <v>70</v>
+      </c>
     </row>
-    <row r="2" spans="1:31">
+    <row r="2" spans="1:32">
       <c r="A2" t="s">
         <v>25</v>
       </c>
       <c r="B2" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C2" s="2">
         <v>44023.34644167824</v>
@@ -1460,13 +1469,13 @@
         <v>0</v>
       </c>
       <c r="H2" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="I2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="J2" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="K2">
         <v>204</v>
@@ -1505,7 +1514,7 @@
         <v>4.53333333</v>
       </c>
       <c r="W2" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="Y2">
         <v>4.533333</v>
@@ -1514,12 +1523,12 @@
         <v>3.26514</v>
       </c>
     </row>
-    <row r="3" spans="1:31">
+    <row r="3" spans="1:32">
       <c r="A3" t="s">
         <v>25</v>
       </c>
       <c r="B3" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C3" s="2">
         <v>44023.34667440972</v>
@@ -1537,13 +1546,13 @@
         <v>26</v>
       </c>
       <c r="H3" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="I3" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="J3" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="K3">
         <v>214</v>
@@ -1570,7 +1579,7 @@
         <v>6.66666667</v>
       </c>
       <c r="W3" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="X3">
         <v>0.035556</v>
@@ -1591,12 +1600,12 @@
         <v>10.119081</v>
       </c>
     </row>
-    <row r="4" spans="1:31">
+    <row r="4" spans="1:32">
       <c r="A4" t="s">
         <v>25</v>
       </c>
       <c r="B4" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C4" s="2">
         <v>44023.34674237268</v>
@@ -1614,13 +1623,13 @@
         <v>30</v>
       </c>
       <c r="H4" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="I4" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="J4" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="K4">
         <v>209</v>
@@ -1659,7 +1668,7 @@
         <v>14.8</v>
       </c>
       <c r="W4" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="X4">
         <v>0.271111</v>
@@ -1686,12 +1695,12 @@
         <v>12.920151</v>
       </c>
     </row>
-    <row r="5" spans="1:31">
+    <row r="5" spans="1:32">
       <c r="A5" t="s">
         <v>25</v>
       </c>
       <c r="B5" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C5" s="2">
         <v>44023.34702186342</v>
@@ -1709,13 +1718,13 @@
         <v>56</v>
       </c>
       <c r="H5" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="I5" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="J5" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="K5">
         <v>210</v>
@@ -1742,7 +1751,7 @@
         <v>16.73333333</v>
       </c>
       <c r="W5" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="X5">
         <v>0.064444</v>
@@ -1769,12 +1778,12 @@
         <v>15.893677</v>
       </c>
     </row>
-    <row r="6" spans="1:31">
+    <row r="6" spans="1:32">
       <c r="A6" t="s">
         <v>25</v>
       </c>
       <c r="B6" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C6" s="2">
         <v>44023.34707267361</v>
@@ -1792,13 +1801,13 @@
         <v>60</v>
       </c>
       <c r="H6" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="I6" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="J6" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="K6">
         <v>211</v>
@@ -1837,7 +1846,7 @@
         <v>16.5</v>
       </c>
       <c r="W6" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="X6">
         <v>-0.007778</v>
@@ -1864,12 +1873,12 @@
         <v>16.525017</v>
       </c>
     </row>
-    <row r="7" spans="1:31">
+    <row r="7" spans="1:32">
       <c r="A7" t="s">
         <v>25</v>
       </c>
       <c r="B7" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C7" s="2">
         <v>44023.3473683912</v>
@@ -1887,13 +1896,13 @@
         <v>86</v>
       </c>
       <c r="H7" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="I7" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="J7" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="K7">
         <v>165</v>
@@ -1920,7 +1929,7 @@
         <v>17.16666667</v>
       </c>
       <c r="W7" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="X7">
         <v>0.022222</v>
@@ -1947,12 +1956,12 @@
         <v>16.714391</v>
       </c>
     </row>
-    <row r="8" spans="1:31">
+    <row r="8" spans="1:32">
       <c r="A8" t="s">
         <v>25</v>
       </c>
       <c r="B8" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C8" s="2">
         <v>44023.34744381945</v>
@@ -1970,13 +1979,13 @@
         <v>90</v>
       </c>
       <c r="H8" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="I8" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="J8" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="K8">
         <v>157</v>
@@ -2015,7 +2024,7 @@
         <v>12.75</v>
       </c>
       <c r="W8" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="X8">
         <v>-0.036806</v>
@@ -2042,12 +2051,12 @@
         <v>16.544965</v>
       </c>
     </row>
-    <row r="9" spans="1:31">
+    <row r="9" spans="1:32">
       <c r="A9" t="s">
         <v>25</v>
       </c>
       <c r="B9" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C9" s="2">
         <v>44023.34741728009</v>
@@ -2065,13 +2074,13 @@
         <v>90</v>
       </c>
       <c r="H9" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="I9" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="J9" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="K9">
         <v>157</v>
@@ -2110,7 +2119,7 @@
         <v>17.23333333</v>
       </c>
       <c r="W9" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="X9">
         <v>0.149444</v>
@@ -2137,12 +2146,12 @@
         <v>16.47621</v>
       </c>
     </row>
-    <row r="10" spans="1:31">
+    <row r="10" spans="1:32">
       <c r="A10" t="s">
         <v>25</v>
       </c>
       <c r="B10" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C10" s="2">
         <v>44023.34771681713</v>
@@ -2160,13 +2169,13 @@
         <v>116</v>
       </c>
       <c r="H10" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="I10" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="J10" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="K10">
         <v>119</v>
@@ -2193,7 +2202,7 @@
         <v>16.73333333</v>
       </c>
       <c r="W10" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="X10">
         <v>-0.016667</v>
@@ -2220,12 +2229,12 @@
         <v>15.761494</v>
       </c>
     </row>
-    <row r="11" spans="1:31">
+    <row r="11" spans="1:32">
       <c r="A11" t="s">
         <v>25</v>
       </c>
       <c r="B11" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C11" s="2">
         <v>44023.34776537037</v>
@@ -2243,13 +2252,13 @@
         <v>120</v>
       </c>
       <c r="H11" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="I11" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="J11" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="K11">
         <v>118</v>
@@ -2288,7 +2297,7 @@
         <v>17.03333333</v>
       </c>
       <c r="W11" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="X11">
         <v>0.01</v>
@@ -2315,12 +2324,12 @@
         <v>15.377842</v>
       </c>
     </row>
-    <row r="12" spans="1:31">
+    <row r="12" spans="1:32">
       <c r="A12" t="s">
         <v>25</v>
       </c>
       <c r="B12" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C12" s="2">
         <v>44023.34806101852</v>
@@ -2338,13 +2347,13 @@
         <v>146</v>
       </c>
       <c r="H12" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="I12" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="J12" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="K12">
         <v>178</v>
@@ -2371,7 +2380,7 @@
         <v>15.53333333</v>
       </c>
       <c r="W12" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="X12">
         <v>-0.05</v>
@@ -2398,12 +2407,12 @@
         <v>14.866984</v>
       </c>
     </row>
-    <row r="13" spans="1:31">
+    <row r="13" spans="1:32">
       <c r="A13" t="s">
         <v>25</v>
       </c>
       <c r="B13" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C13" s="2">
         <v>44023.34813881944</v>
@@ -2421,13 +2430,13 @@
         <v>150</v>
       </c>
       <c r="H13" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="I13" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="J13" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="K13">
         <v>103</v>
@@ -2466,7 +2475,7 @@
         <v>15.85</v>
       </c>
       <c r="W13" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="X13">
         <v>0.005278</v>
@@ -2493,12 +2502,12 @@
         <v>14.729125</v>
       </c>
     </row>
-    <row r="14" spans="1:31">
+    <row r="14" spans="1:32">
       <c r="A14" t="s">
         <v>25</v>
       </c>
       <c r="B14" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C14" s="2">
         <v>44023.34811263889</v>
@@ -2516,13 +2525,13 @@
         <v>150</v>
       </c>
       <c r="H14" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="I14" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="J14" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="K14">
         <v>112</v>
@@ -2561,7 +2570,7 @@
         <v>15.1</v>
       </c>
       <c r="W14" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="X14">
         <v>-0.025</v>
@@ -2588,12 +2597,12 @@
         <v>14.674833</v>
       </c>
     </row>
-    <row r="15" spans="1:31">
+    <row r="15" spans="1:32">
       <c r="A15" t="s">
         <v>25</v>
       </c>
       <c r="B15" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C15" s="2">
         <v>44023.3484072338</v>
@@ -2611,13 +2620,13 @@
         <v>176</v>
       </c>
       <c r="H15" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="I15" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J15" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="K15">
         <v>149</v>
@@ -2644,7 +2653,7 @@
         <v>13.8</v>
       </c>
       <c r="W15" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="X15">
         <v>-0.043333</v>
@@ -2671,12 +2680,12 @@
         <v>14.523325</v>
       </c>
     </row>
-    <row r="16" spans="1:31">
+    <row r="16" spans="1:32">
       <c r="A16" t="s">
         <v>25</v>
       </c>
       <c r="B16" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C16" s="2">
         <v>44023.3484581713</v>
@@ -2694,13 +2703,13 @@
         <v>180</v>
       </c>
       <c r="H16" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="I16" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="J16" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="K16">
         <v>137</v>
@@ -2739,7 +2748,7 @@
         <v>13.8</v>
       </c>
       <c r="W16" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="X16">
         <v>0</v>
@@ -2766,12 +2775,12 @@
         <v>14.509255</v>
       </c>
     </row>
-    <row r="17" spans="1:31">
+    <row r="17" spans="1:32">
       <c r="A17" t="s">
         <v>25</v>
       </c>
       <c r="B17" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C17" s="2">
         <v>44023.34846752314</v>
@@ -2789,13 +2798,13 @@
         <v>180</v>
       </c>
       <c r="H17" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="I17" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="J17" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="K17">
         <v>134</v>
@@ -2834,7 +2843,7 @@
         <v>14.43333333</v>
       </c>
       <c r="W17" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="X17">
         <v>0.021111</v>
@@ -2861,12 +2870,12 @@
         <v>14.507455</v>
       </c>
     </row>
-    <row r="18" spans="1:31">
+    <row r="18" spans="1:32">
       <c r="A18" t="s">
         <v>25</v>
       </c>
       <c r="B18" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C18" s="2">
         <v>44023.34880686343</v>
@@ -2884,13 +2893,13 @@
         <v>210</v>
       </c>
       <c r="H18" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="I18" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="J18" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="K18">
         <v>95</v>
@@ -2929,7 +2938,7 @@
         <v>13.33333333</v>
       </c>
       <c r="W18" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="X18">
         <v>-0.036667</v>
@@ -2956,12 +2965,12 @@
         <v>14.650473</v>
       </c>
     </row>
-    <row r="19" spans="1:31">
+    <row r="19" spans="1:32">
       <c r="A19" t="s">
         <v>25</v>
       </c>
       <c r="B19" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C19" s="2">
         <v>44023.34883809028</v>
@@ -2979,13 +2988,13 @@
         <v>210</v>
       </c>
       <c r="H19" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="I19" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="J19" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="K19">
         <v>100</v>
@@ -3024,7 +3033,7 @@
         <v>12.53333333</v>
       </c>
       <c r="W19" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="X19">
         <v>-0.026667</v>
@@ -3051,12 +3060,12 @@
         <v>14.622291</v>
       </c>
     </row>
-    <row r="20" spans="1:31">
+    <row r="20" spans="1:32">
       <c r="A20" t="s">
         <v>25</v>
       </c>
       <c r="B20" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C20" s="2">
         <v>44023.34915288194</v>
@@ -3074,13 +3083,13 @@
         <v>240</v>
       </c>
       <c r="H20" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="I20" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="J20" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="K20">
         <v>106</v>
@@ -3119,7 +3128,7 @@
         <v>15.6</v>
       </c>
       <c r="W20" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="X20">
         <v>0.102222</v>
@@ -3146,12 +3155,12 @@
         <v>14.773221</v>
       </c>
     </row>
-    <row r="21" spans="1:31">
+    <row r="21" spans="1:32">
       <c r="A21" t="s">
         <v>25</v>
       </c>
       <c r="B21" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C21" s="2">
         <v>44023.34916229167</v>
@@ -3169,13 +3178,13 @@
         <v>240</v>
       </c>
       <c r="H21" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="I21" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="J21" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="K21">
         <v>111</v>
@@ -3214,7 +3223,7 @@
         <v>14.9</v>
       </c>
       <c r="W21" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="X21">
         <v>-0.023333</v>
@@ -3241,12 +3250,12 @@
         <v>14.779267</v>
       </c>
     </row>
-    <row r="22" spans="1:31">
+    <row r="22" spans="1:32">
       <c r="A22" t="s">
         <v>25</v>
       </c>
       <c r="B22" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C22" s="2">
         <v>44023.34945041667</v>
@@ -3264,13 +3273,13 @@
         <v>266</v>
       </c>
       <c r="H22" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="I22" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="J22" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="K22">
         <v>109</v>
@@ -3297,7 +3306,7 @@
         <v>14.51111111</v>
       </c>
       <c r="W22" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="X22">
         <v>-0.004321</v>
@@ -3324,12 +3333,12 @@
         <v>14.596409</v>
       </c>
     </row>
-    <row r="23" spans="1:31">
+    <row r="23" spans="1:32">
       <c r="A23" t="s">
         <v>25</v>
       </c>
       <c r="B23" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C23" s="2">
         <v>44023.34949959491</v>
@@ -3347,13 +3356,13 @@
         <v>270</v>
       </c>
       <c r="H23" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="I23" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="J23" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="K23">
         <v>102</v>
@@ -3392,7 +3401,7 @@
         <v>14.43333333</v>
       </c>
       <c r="W23" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="X23">
         <v>-0.002593</v>
@@ -3419,12 +3428,12 @@
         <v>14.354163</v>
       </c>
     </row>
-    <row r="24" spans="1:31">
+    <row r="24" spans="1:32">
       <c r="A24" t="s">
         <v>25</v>
       </c>
       <c r="B24" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C24" s="2">
         <v>44023.34952732639</v>
@@ -3442,13 +3451,13 @@
         <v>270</v>
       </c>
       <c r="H24" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="I24" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="J24" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="K24">
         <v>104</v>
@@ -3487,7 +3496,7 @@
         <v>15.36666667</v>
       </c>
       <c r="W24" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="X24">
         <v>0.031111</v>
@@ -3514,12 +3523,12 @@
         <v>14.445267</v>
       </c>
     </row>
-    <row r="25" spans="1:31">
+    <row r="25" spans="1:32">
       <c r="A25" t="s">
         <v>25</v>
       </c>
       <c r="B25" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C25" s="2">
         <v>44023.34979804398</v>
@@ -3537,13 +3546,13 @@
         <v>296</v>
       </c>
       <c r="H25" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="I25" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="J25" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="K25">
         <v>128</v>
@@ -3570,7 +3579,7 @@
         <v>12.9</v>
       </c>
       <c r="W25" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="X25">
         <v>-0.082222</v>
@@ -3597,12 +3606,12 @@
         <v>13.777135</v>
       </c>
     </row>
-    <row r="26" spans="1:31">
+    <row r="26" spans="1:32">
       <c r="A26" t="s">
         <v>25</v>
       </c>
       <c r="B26" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C26" s="2">
         <v>44023.34984708334</v>
@@ -3620,13 +3629,13 @@
         <v>300</v>
       </c>
       <c r="H26" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="I26" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="J26" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="K26">
         <v>111</v>
@@ -3665,7 +3674,7 @@
         <v>13.63333333</v>
       </c>
       <c r="W26" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="X26">
         <v>0.024444</v>
@@ -3692,12 +3701,12 @@
         <v>13.114407</v>
       </c>
     </row>
-    <row r="27" spans="1:31">
+    <row r="27" spans="1:32">
       <c r="A27" t="s">
         <v>25</v>
       </c>
       <c r="B27" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C27" s="2">
         <v>44023.35019421297</v>
@@ -3715,13 +3724,13 @@
         <v>330</v>
       </c>
       <c r="H27" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="I27" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="J27" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="K27">
         <v>122</v>
@@ -3760,7 +3769,7 @@
         <v>14.06666667</v>
       </c>
       <c r="W27" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="X27">
         <v>0.014444</v>
@@ -3786,13 +3795,16 @@
       <c r="AE27">
         <v>10.809557</v>
       </c>
+      <c r="AF27" t="s">
+        <v>171</v>
+      </c>
     </row>
-    <row r="28" spans="1:31">
+    <row r="28" spans="1:32">
       <c r="A28" t="s">
         <v>25</v>
       </c>
       <c r="B28" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C28" s="2">
         <v>44023.3502215625</v>
@@ -3810,13 +3822,13 @@
         <v>330</v>
       </c>
       <c r="H28" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="I28" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="J28" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="K28">
         <v>125</v>
@@ -3855,7 +3867,7 @@
         <v>13.7</v>
       </c>
       <c r="W28" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="X28">
         <v>-0.006111</v>
@@ -3882,12 +3894,12 @@
         <v>11.198955</v>
       </c>
     </row>
-    <row r="29" spans="1:31">
+    <row r="29" spans="1:32">
       <c r="A29" t="s">
         <v>25</v>
       </c>
       <c r="B29" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C29" s="2">
         <v>44023.35055107639</v>
@@ -3905,13 +3917,13 @@
         <v>360</v>
       </c>
       <c r="H29" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="I29" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="J29" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="K29">
         <v>121</v>
@@ -3950,7 +3962,7 @@
         <v>9.5</v>
       </c>
       <c r="W29" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="X29">
         <v>-0.14</v>
@@ -3977,12 +3989,12 @@
         <v>9.194838000000001</v>
       </c>
     </row>
-    <row r="30" spans="1:31">
+    <row r="30" spans="1:32">
       <c r="A30" t="s">
         <v>25</v>
       </c>
       <c r="B30" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C30" s="2">
         <v>44023.35054172454</v>
@@ -4000,13 +4012,13 @@
         <v>360</v>
       </c>
       <c r="H30" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="I30" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="J30" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="K30">
         <v>123</v>
@@ -4045,7 +4057,7 @@
         <v>8.16666667</v>
       </c>
       <c r="W30" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="X30">
         <v>-0.044444</v>
@@ -4072,12 +4084,12 @@
         <v>9.041117</v>
       </c>
     </row>
-    <row r="31" spans="1:31">
+    <row r="31" spans="1:32">
       <c r="A31" t="s">
         <v>25</v>
       </c>
       <c r="B31" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C31" s="2">
         <v>44023.35083818287</v>
@@ -4095,13 +4107,13 @@
         <v>386</v>
       </c>
       <c r="H31" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="I31" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="J31" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="K31">
         <v>125</v>
@@ -4128,7 +4140,7 @@
         <v>9.811111110000001</v>
       </c>
       <c r="W31" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="X31">
         <v>0.018272</v>
@@ -4155,12 +4167,12 @@
         <v>8.760968999999999</v>
       </c>
     </row>
-    <row r="32" spans="1:31">
+    <row r="32" spans="1:32">
       <c r="A32" t="s">
         <v>25</v>
       </c>
       <c r="B32" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C32" s="2">
         <v>44023.35091582176</v>
@@ -4178,13 +4190,13 @@
         <v>389</v>
       </c>
       <c r="H32" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="I32" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="J32" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="K32">
         <v>117</v>
@@ -4223,7 +4235,7 @@
         <v>4.03448276</v>
       </c>
       <c r="W32" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="X32">
         <v>-0.199194</v>
@@ -4255,7 +4267,7 @@
         <v>25</v>
       </c>
       <c r="B33" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C33" s="2">
         <v>44023.35088921296</v>
@@ -4273,13 +4285,13 @@
         <v>390</v>
       </c>
       <c r="H33" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="I33" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="J33" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="K33">
         <v>117</v>
@@ -4318,7 +4330,7 @@
         <v>5.8</v>
       </c>
       <c r="W33" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="X33">
         <v>0.058851</v>
@@ -4350,7 +4362,7 @@
         <v>25</v>
       </c>
       <c r="B34" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C34" s="2">
         <v>44023.35118658565</v>
@@ -4368,13 +4380,13 @@
         <v>416</v>
       </c>
       <c r="H34" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="I34" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="J34" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="K34">
         <v>109</v>
@@ -4401,7 +4413,7 @@
         <v>5.46666667</v>
       </c>
       <c r="W34" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="X34">
         <v>-0.011111</v>
@@ -4433,7 +4445,7 @@
         <v>25</v>
       </c>
       <c r="B35" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C35" s="2">
         <v>44023.35123702546</v>
@@ -4451,13 +4463,13 @@
         <v>420</v>
       </c>
       <c r="H35" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="I35" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="J35" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="K35">
         <v>110</v>
@@ -4496,7 +4508,7 @@
         <v>5.4</v>
       </c>
       <c r="W35" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="X35">
         <v>-0.002222</v>
@@ -4528,7 +4540,7 @@
         <v>25</v>
       </c>
       <c r="B36" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C36" s="2">
         <v>44023.35124731481</v>
@@ -4546,13 +4558,13 @@
         <v>420</v>
       </c>
       <c r="H36" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="I36" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="J36" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="K36">
         <v>111</v>
@@ -4591,7 +4603,7 @@
         <v>6.06451613</v>
       </c>
       <c r="W36" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="X36">
         <v>0.021436</v>
@@ -4623,7 +4635,7 @@
         <v>25</v>
       </c>
       <c r="B37" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C37" s="2">
         <v>44023.35153310185</v>
@@ -4641,13 +4653,13 @@
         <v>446</v>
       </c>
       <c r="H37" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="I37" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="J37" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="K37">
         <v>114</v>
@@ -4674,7 +4686,7 @@
         <v>5.66666667</v>
       </c>
       <c r="W37" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="X37">
         <v>-0.013262</v>
@@ -4706,7 +4718,7 @@
         <v>25</v>
       </c>
       <c r="B38" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C38" s="2">
         <v>44023.35158375</v>
@@ -4724,13 +4736,13 @@
         <v>450</v>
       </c>
       <c r="H38" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="I38" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="J38" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="K38">
         <v>116</v>
@@ -4769,7 +4781,7 @@
         <v>5.8</v>
       </c>
       <c r="W38" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="X38">
         <v>0.004444</v>
@@ -4801,7 +4813,7 @@
         <v>25</v>
       </c>
       <c r="B39" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C39" s="2">
         <v>44023.35161115741</v>
@@ -4819,13 +4831,13 @@
         <v>450</v>
       </c>
       <c r="H39" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="I39" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="J39" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="K39">
         <v>114</v>
@@ -4864,7 +4876,7 @@
         <v>6.16666667</v>
       </c>
       <c r="W39" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="X39">
         <v>0.012222</v>
@@ -4896,7 +4908,7 @@
         <v>25</v>
       </c>
       <c r="B40" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C40" s="2">
         <v>44023.35187935185</v>
@@ -4914,13 +4926,13 @@
         <v>476</v>
       </c>
       <c r="H40" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="I40" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="J40" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="K40">
         <v>118</v>
@@ -4947,7 +4959,7 @@
         <v>5.7</v>
       </c>
       <c r="W40" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="X40">
         <v>-0.015556</v>
@@ -4979,7 +4991,7 @@
         <v>25</v>
       </c>
       <c r="B41" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C41" s="2">
         <v>44023.35193064815</v>
@@ -4997,13 +5009,13 @@
         <v>480</v>
       </c>
       <c r="H41" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="I41" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="J41" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="K41">
         <v>118</v>
@@ -5042,7 +5054,7 @@
         <v>5.36666667</v>
       </c>
       <c r="W41" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="X41">
         <v>-0.011111</v>
@@ -5074,7 +5086,7 @@
         <v>25</v>
       </c>
       <c r="B42" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C42" s="2">
         <v>44023.35194001158</v>
@@ -5092,13 +5104,13 @@
         <v>480</v>
       </c>
       <c r="H42" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="I42" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="J42" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="K42">
         <v>118</v>
@@ -5137,7 +5149,7 @@
         <v>5.3</v>
       </c>
       <c r="W42" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="X42">
         <v>-0.002222</v>
@@ -5169,7 +5181,7 @@
         <v>25</v>
       </c>
       <c r="B43" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C43" s="2">
         <v>44023.35227842593</v>
@@ -5187,13 +5199,13 @@
         <v>510</v>
       </c>
       <c r="H43" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="I43" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="J43" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="K43">
         <v>120</v>
@@ -5232,7 +5244,7 @@
         <v>3.76666667</v>
       </c>
       <c r="W43" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="X43">
         <v>-0.051111</v>
@@ -5264,7 +5276,7 @@
         <v>25</v>
       </c>
       <c r="B44" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C44" s="2">
         <v>44023.35230556713</v>
@@ -5282,13 +5294,13 @@
         <v>510</v>
       </c>
       <c r="H44" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="I44" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="J44" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="K44">
         <v>119</v>
@@ -5327,7 +5339,7 @@
         <v>3.06666667</v>
       </c>
       <c r="W44" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="X44">
         <v>-0.023333</v>
@@ -5359,7 +5371,7 @@
         <v>25</v>
       </c>
       <c r="B45" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C45" s="2">
         <v>44023.35257471065</v>
@@ -5377,13 +5389,13 @@
         <v>536</v>
       </c>
       <c r="H45" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="I45" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="J45" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="K45">
         <v>121</v>
@@ -5410,7 +5422,7 @@
         <v>3.38333333</v>
       </c>
       <c r="W45" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="X45">
         <v>0.005278</v>
@@ -5442,7 +5454,7 @@
         <v>25</v>
       </c>
       <c r="B46" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C46" s="2">
         <v>44023.35262537037</v>
@@ -5460,13 +5472,13 @@
         <v>540</v>
       </c>
       <c r="H46" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="I46" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="J46" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="K46">
         <v>121</v>
@@ -5505,7 +5517,7 @@
         <v>2.73333333</v>
       </c>
       <c r="W46" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="X46">
         <v>-0.021667</v>
@@ -5537,7 +5549,7 @@
         <v>25</v>
       </c>
       <c r="B47" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C47" s="2">
         <v>44023.35292203704</v>
@@ -5555,13 +5567,13 @@
         <v>566</v>
       </c>
       <c r="H47" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="I47" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="J47" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="K47">
         <v>121</v>
@@ -5588,7 +5600,7 @@
         <v>1.43333333</v>
       </c>
       <c r="W47" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="X47">
         <v>-0.043333</v>
@@ -5620,7 +5632,7 @@
         <v>25</v>
       </c>
       <c r="B48" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C48" s="2">
         <v>44023.35297302083</v>
@@ -5638,13 +5650,13 @@
         <v>570</v>
       </c>
       <c r="H48" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="I48" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="J48" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="K48">
         <v>121</v>
@@ -5683,7 +5695,7 @@
         <v>1.23333333</v>
       </c>
       <c r="W48" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="X48">
         <v>-0.006667</v>
@@ -5717,10 +5729,10 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AE48"/>
+  <dimension ref="A1:AF48"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:31">
+    <row r="1" spans="1:32">
       <c r="A1" s="1" t="s">
         <v>39</v>
       </c>
@@ -5814,13 +5826,16 @@
       <c r="AE1" s="1" t="s">
         <v>69</v>
       </c>
+      <c r="AF1" s="1" t="s">
+        <v>70</v>
+      </c>
     </row>
-    <row r="2" spans="1:31">
+    <row r="2" spans="1:32">
       <c r="A2" t="s">
         <v>25</v>
       </c>
       <c r="B2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C2" s="2">
         <v>44023.35299995371</v>
@@ -5838,13 +5853,13 @@
         <v>0</v>
       </c>
       <c r="H2" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="I2" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="J2" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="K2">
         <v>120</v>
@@ -5883,7 +5898,7 @@
         <v>2.15</v>
       </c>
       <c r="W2" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="Y2">
         <v>2.15</v>
@@ -5892,12 +5907,12 @@
         <v>-0.31442</v>
       </c>
     </row>
-    <row r="3" spans="1:31">
+    <row r="3" spans="1:32">
       <c r="A3" t="s">
         <v>25</v>
       </c>
       <c r="B3" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C3" s="2">
         <v>44023.35333020833</v>
@@ -5915,13 +5930,13 @@
         <v>29</v>
       </c>
       <c r="H3" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="I3" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="J3" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="K3">
         <v>121</v>
@@ -5960,7 +5975,7 @@
         <v>-0.10344828</v>
       </c>
       <c r="W3" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="X3">
         <v>-0.077705</v>
@@ -5981,12 +5996,12 @@
         <v>-0.394813</v>
       </c>
     </row>
-    <row r="4" spans="1:31">
+    <row r="4" spans="1:32">
       <c r="A4" t="s">
         <v>25</v>
       </c>
       <c r="B4" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C4" s="2">
         <v>44023.35331981481</v>
@@ -6004,13 +6019,13 @@
         <v>30</v>
       </c>
       <c r="H4" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="I4" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="J4" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="K4">
         <v>121</v>
@@ -6049,7 +6064,7 @@
         <v>-0.7</v>
       </c>
       <c r="W4" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="X4">
         <v>-0.019885</v>
@@ -6076,12 +6091,12 @@
         <v>0.669476</v>
       </c>
     </row>
-    <row r="5" spans="1:31">
+    <row r="5" spans="1:32">
       <c r="A5" t="s">
         <v>25</v>
       </c>
       <c r="B5" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C5" s="2">
         <v>44023.35361952546</v>
@@ -6099,13 +6114,13 @@
         <v>56</v>
       </c>
       <c r="H5" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="I5" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="J5" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="K5">
         <v>122</v>
@@ -6132,7 +6147,7 @@
         <v>-1.41666667</v>
       </c>
       <c r="W5" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="X5">
         <v>-0.011944</v>
@@ -6159,12 +6174,12 @@
         <v>-2.827954</v>
       </c>
     </row>
-    <row r="6" spans="1:31">
+    <row r="6" spans="1:32">
       <c r="A6" t="s">
         <v>25</v>
       </c>
       <c r="B6" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C6" s="2">
         <v>44023.35369785879</v>
@@ -6182,13 +6197,13 @@
         <v>60</v>
       </c>
       <c r="H6" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="I6" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="J6" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="K6">
         <v>121</v>
@@ -6227,7 +6242,7 @@
         <v>-3.41935484</v>
       </c>
       <c r="W6" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="X6">
         <v>-0.06460299999999999</v>
@@ -6254,12 +6269,12 @@
         <v>-2.368774</v>
       </c>
     </row>
-    <row r="7" spans="1:31">
+    <row r="7" spans="1:32">
       <c r="A7" t="s">
         <v>25</v>
       </c>
       <c r="B7" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C7" s="2">
         <v>44023.35366663194</v>
@@ -6277,13 +6292,13 @@
         <v>60</v>
       </c>
       <c r="H7" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="I7" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="J7" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="K7">
         <v>122</v>
@@ -6322,7 +6337,7 @@
         <v>-2.8</v>
       </c>
       <c r="W7" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="X7">
         <v>0.020645</v>
@@ -6349,12 +6364,12 @@
         <v>-1.483951</v>
       </c>
     </row>
-    <row r="8" spans="1:31">
+    <row r="8" spans="1:32">
       <c r="A8" t="s">
         <v>25</v>
       </c>
       <c r="B8" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C8" s="2">
         <v>44023.35396462963</v>
@@ -6372,13 +6387,13 @@
         <v>86</v>
       </c>
       <c r="H8" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="I8" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="J8" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="K8">
         <v>122</v>
@@ -6405,7 +6420,7 @@
         <v>-3.3</v>
       </c>
       <c r="W8" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="X8">
         <v>-0.016667</v>
@@ -6432,12 +6447,12 @@
         <v>-3.715523</v>
       </c>
     </row>
-    <row r="9" spans="1:31">
+    <row r="9" spans="1:32">
       <c r="A9" t="s">
         <v>25</v>
       </c>
       <c r="B9" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C9" s="2">
         <v>44023.35401414352</v>
@@ -6455,13 +6470,13 @@
         <v>90</v>
       </c>
       <c r="H9" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="I9" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="J9" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="K9">
         <v>122</v>
@@ -6500,7 +6515,7 @@
         <v>-3.43333333</v>
       </c>
       <c r="W9" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="X9">
         <v>-0.004444</v>
@@ -6527,12 +6542,12 @@
         <v>-2.901682</v>
       </c>
     </row>
-    <row r="10" spans="1:31">
+    <row r="10" spans="1:32">
       <c r="A10" t="s">
         <v>25</v>
       </c>
       <c r="B10" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C10" s="2">
         <v>44023.35431188657</v>
@@ -6550,13 +6565,13 @@
         <v>116</v>
       </c>
       <c r="H10" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="I10" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="J10" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="K10">
         <v>122</v>
@@ -6583,7 +6598,7 @@
         <v>-4.36666667</v>
       </c>
       <c r="W10" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="X10">
         <v>-0.031111</v>
@@ -6610,12 +6625,12 @@
         <v>-4.607338</v>
       </c>
     </row>
-    <row r="11" spans="1:31">
+    <row r="11" spans="1:32">
       <c r="A11" t="s">
         <v>25</v>
       </c>
       <c r="B11" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C11" s="2">
         <v>44023.35436167824</v>
@@ -6633,13 +6648,13 @@
         <v>120</v>
       </c>
       <c r="H11" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="I11" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="J11" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="K11">
         <v>119</v>
@@ -6678,7 +6693,7 @@
         <v>-4.53333333</v>
       </c>
       <c r="W11" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="X11">
         <v>-0.005556</v>
@@ -6705,12 +6720,12 @@
         <v>-4.039655</v>
       </c>
     </row>
-    <row r="12" spans="1:31">
+    <row r="12" spans="1:32">
       <c r="A12" t="s">
         <v>25</v>
       </c>
       <c r="B12" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C12" s="2">
         <v>44023.35438840277</v>
@@ -6728,13 +6743,13 @@
         <v>120</v>
       </c>
       <c r="H12" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="I12" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="J12" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="K12">
         <v>119</v>
@@ -6773,7 +6788,7 @@
         <v>-4.01666667</v>
       </c>
       <c r="W12" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="X12">
         <v>0.008611000000000001</v>
@@ -6800,12 +6815,12 @@
         <v>-4.434036</v>
       </c>
     </row>
-    <row r="13" spans="1:31">
+    <row r="13" spans="1:32">
       <c r="A13" t="s">
         <v>25</v>
       </c>
       <c r="B13" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C13" s="2">
         <v>44023.35470967593</v>
@@ -6823,13 +6838,13 @@
         <v>150</v>
       </c>
       <c r="H13" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="I13" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="J13" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="K13">
         <v>119</v>
@@ -6868,7 +6883,7 @@
         <v>-5.86666667</v>
       </c>
       <c r="W13" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="X13">
         <v>-0.061667</v>
@@ -6895,12 +6910,12 @@
         <v>-5.100315</v>
       </c>
     </row>
-    <row r="14" spans="1:31">
+    <row r="14" spans="1:32">
       <c r="A14" t="s">
         <v>25</v>
       </c>
       <c r="B14" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C14" s="2">
         <v>44023.35500557871</v>
@@ -6918,13 +6933,13 @@
         <v>176</v>
       </c>
       <c r="H14" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="I14" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="J14" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="K14">
         <v>122</v>
@@ -6951,7 +6966,7 @@
         <v>-5.9</v>
       </c>
       <c r="W14" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="X14">
         <v>-0.000556</v>
@@ -6978,12 +6993,12 @@
         <v>-6.042201</v>
       </c>
     </row>
-    <row r="15" spans="1:31">
+    <row r="15" spans="1:32">
       <c r="A15" t="s">
         <v>25</v>
       </c>
       <c r="B15" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C15" s="2">
         <v>44023.35505572917</v>
@@ -7001,13 +7016,13 @@
         <v>180</v>
       </c>
       <c r="H15" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="I15" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="J15" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="K15">
         <v>119</v>
@@ -7046,7 +7061,7 @@
         <v>-5.96666667</v>
       </c>
       <c r="W15" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="X15">
         <v>-0.002222</v>
@@ -7073,12 +7088,12 @@
         <v>-5.814394</v>
       </c>
     </row>
-    <row r="16" spans="1:31">
+    <row r="16" spans="1:32">
       <c r="A16" t="s">
         <v>25</v>
       </c>
       <c r="B16" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C16" s="2">
         <v>44023.35535255787</v>
@@ -7096,13 +7111,13 @@
         <v>206</v>
       </c>
       <c r="H16" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="I16" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="J16" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="K16">
         <v>118</v>
@@ -7129,7 +7144,7 @@
         <v>-5.7</v>
       </c>
       <c r="W16" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="X16">
         <v>0.008888999999999999</v>
@@ -7161,7 +7176,7 @@
         <v>25</v>
       </c>
       <c r="B17" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C17" s="2">
         <v>44023.3554027662</v>
@@ -7179,13 +7194,13 @@
         <v>210</v>
       </c>
       <c r="H17" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="I17" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="J17" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="K17">
         <v>124</v>
@@ -7224,7 +7239,7 @@
         <v>-5.73333333</v>
       </c>
       <c r="W17" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="X17">
         <v>-0.001111</v>
@@ -7256,7 +7271,7 @@
         <v>25</v>
       </c>
       <c r="B18" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C18" s="2">
         <v>44023.35569953704</v>
@@ -7274,13 +7289,13 @@
         <v>236</v>
       </c>
       <c r="H18" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="I18" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="J18" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="K18">
         <v>113</v>
@@ -7307,7 +7322,7 @@
         <v>-7.1</v>
       </c>
       <c r="W18" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="X18">
         <v>-0.045556</v>
@@ -7339,7 +7354,7 @@
         <v>25</v>
       </c>
       <c r="B19" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C19" s="2">
         <v>44023.35575015046</v>
@@ -7357,13 +7372,13 @@
         <v>240</v>
       </c>
       <c r="H19" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="I19" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="J19" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="K19">
         <v>118</v>
@@ -7402,7 +7417,7 @@
         <v>-7.3</v>
       </c>
       <c r="W19" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="X19">
         <v>-0.006667</v>
@@ -7434,7 +7449,7 @@
         <v>25</v>
       </c>
       <c r="B20" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C20" s="2">
         <v>44023.35604671296</v>
@@ -7452,13 +7467,13 @@
         <v>266</v>
       </c>
       <c r="H20" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="I20" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="J20" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="K20">
         <v>107</v>
@@ -7485,7 +7500,7 @@
         <v>-8.43333333</v>
       </c>
       <c r="W20" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="X20">
         <v>-0.037778</v>
@@ -7517,7 +7532,7 @@
         <v>25</v>
       </c>
       <c r="B21" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C21" s="2">
         <v>44023.35609765046</v>
@@ -7535,13 +7550,13 @@
         <v>270</v>
       </c>
       <c r="H21" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="I21" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="J21" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="K21">
         <v>109</v>
@@ -7580,7 +7595,7 @@
         <v>-8.199999999999999</v>
       </c>
       <c r="W21" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="X21">
         <v>0.007778</v>
@@ -7612,7 +7627,7 @@
         <v>25</v>
       </c>
       <c r="B22" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C22" s="2">
         <v>44023.35647199074</v>
@@ -7630,13 +7645,13 @@
         <v>300</v>
       </c>
       <c r="H22" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="I22" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="J22" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="K22">
         <v>102</v>
@@ -7675,7 +7690,7 @@
         <v>-6.95</v>
       </c>
       <c r="W22" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="X22">
         <v>0.006944</v>
@@ -7707,7 +7722,7 @@
         <v>25</v>
       </c>
       <c r="B23" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C23" s="2">
         <v>44023.35644489584</v>
@@ -7725,13 +7740,13 @@
         <v>300</v>
       </c>
       <c r="H23" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="I23" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="J23" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="K23">
         <v>99</v>
@@ -7770,7 +7785,7 @@
         <v>-9.133333329999999</v>
       </c>
       <c r="W23" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="X23">
         <v>-0.072778</v>
@@ -7802,7 +7817,7 @@
         <v>25</v>
       </c>
       <c r="B24" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C24" s="2">
         <v>44023.35674206018</v>
@@ -7820,13 +7835,13 @@
         <v>326</v>
       </c>
       <c r="H24" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="I24" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="J24" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="K24">
         <v>102</v>
@@ -7853,7 +7868,7 @@
         <v>-9.516666669999999</v>
       </c>
       <c r="W24" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="X24">
         <v>-0.006389</v>
@@ -7885,7 +7900,7 @@
         <v>25</v>
       </c>
       <c r="B25" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C25" s="2">
         <v>44023.35679211806</v>
@@ -7903,13 +7918,13 @@
         <v>330</v>
       </c>
       <c r="H25" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="I25" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="J25" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="K25">
         <v>98</v>
@@ -7948,7 +7963,7 @@
         <v>-10.5</v>
       </c>
       <c r="W25" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="X25">
         <v>-0.032778</v>
@@ -7980,7 +7995,7 @@
         <v>25</v>
       </c>
       <c r="B26" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C26" s="2">
         <v>44023.35713885417</v>
@@ -7998,13 +8013,13 @@
         <v>360</v>
       </c>
       <c r="H26" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="I26" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="J26" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="K26">
         <v>98</v>
@@ -8043,7 +8058,7 @@
         <v>-11.23333333</v>
       </c>
       <c r="W26" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="X26">
         <v>-0.024444</v>
@@ -8075,7 +8090,7 @@
         <v>25</v>
       </c>
       <c r="B27" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C27" s="2">
         <v>44023.35743622685</v>
@@ -8093,13 +8108,13 @@
         <v>386</v>
       </c>
       <c r="H27" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="I27" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="J27" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="K27">
         <v>118</v>
@@ -8126,7 +8141,7 @@
         <v>-10.83333333</v>
       </c>
       <c r="W27" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="X27">
         <v>0.006667</v>
@@ -8158,7 +8173,7 @@
         <v>25</v>
       </c>
       <c r="B28" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C28" s="2">
         <v>44023.35748664352</v>
@@ -8176,13 +8191,13 @@
         <v>390</v>
       </c>
       <c r="H28" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="I28" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="J28" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="K28">
         <v>118</v>
@@ -8221,7 +8236,7 @@
         <v>-10.16666667</v>
       </c>
       <c r="W28" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="X28">
         <v>0.022222</v>
@@ -8253,7 +8268,7 @@
         <v>25</v>
       </c>
       <c r="B29" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C29" s="2">
         <v>44023.35778332176</v>
@@ -8271,13 +8286,13 @@
         <v>416</v>
       </c>
       <c r="H29" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="I29" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="J29" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="K29">
         <v>84</v>
@@ -8304,7 +8319,7 @@
         <v>-11.7</v>
       </c>
       <c r="W29" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="X29">
         <v>-0.051111</v>
@@ -8336,7 +8351,7 @@
         <v>25</v>
       </c>
       <c r="B30" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C30" s="2">
         <v>44023.35783324074</v>
@@ -8354,13 +8369,13 @@
         <v>420</v>
       </c>
       <c r="H30" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="I30" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="J30" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="K30">
         <v>119</v>
@@ -8399,7 +8414,7 @@
         <v>-11.93333333</v>
       </c>
       <c r="W30" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="X30">
         <v>-0.007778</v>
@@ -8431,7 +8446,7 @@
         <v>25</v>
       </c>
       <c r="B31" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C31" s="2">
         <v>44023.35786231481</v>
@@ -8449,13 +8464,13 @@
         <v>420</v>
       </c>
       <c r="H31" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="I31" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="J31" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="K31">
         <v>120</v>
@@ -8494,7 +8509,7 @@
         <v>-11.075</v>
       </c>
       <c r="W31" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="X31">
         <v>0.007153</v>
@@ -8526,7 +8541,7 @@
         <v>25</v>
       </c>
       <c r="B32" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C32" s="2">
         <v>44023.35818081019</v>
@@ -8544,13 +8559,13 @@
         <v>450</v>
       </c>
       <c r="H32" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="I32" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="J32" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="K32">
         <v>110</v>
@@ -8589,7 +8604,7 @@
         <v>-13.36666667</v>
       </c>
       <c r="W32" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="X32">
         <v>-0.076389</v>
@@ -8621,7 +8636,7 @@
         <v>25</v>
       </c>
       <c r="B33" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C33" s="2">
         <v>44023.35819207176</v>
@@ -8639,13 +8654,13 @@
         <v>450</v>
       </c>
       <c r="H33" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="I33" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="J33" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="K33">
         <v>115</v>
@@ -8684,7 +8699,7 @@
         <v>-13.3</v>
       </c>
       <c r="W33" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="X33">
         <v>0.002222</v>
@@ -8716,7 +8731,7 @@
         <v>25</v>
       </c>
       <c r="B34" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C34" s="2">
         <v>44023.35847700232</v>
@@ -8734,13 +8749,13 @@
         <v>476</v>
       </c>
       <c r="H34" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="I34" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="J34" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="K34">
         <v>95</v>
@@ -8767,7 +8782,7 @@
         <v>-12.9</v>
       </c>
       <c r="W34" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="X34">
         <v>0.006667</v>
@@ -8799,7 +8814,7 @@
         <v>25</v>
       </c>
       <c r="B35" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C35" s="2">
         <v>44023.35852927083</v>
@@ -8817,13 +8832,13 @@
         <v>480</v>
       </c>
       <c r="H35" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="I35" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="J35" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="K35">
         <v>93</v>
@@ -8862,7 +8877,7 @@
         <v>-12.6</v>
       </c>
       <c r="W35" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="X35">
         <v>0.01</v>
@@ -8894,7 +8909,7 @@
         <v>25</v>
       </c>
       <c r="B36" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C36" s="2">
         <v>44023.3585559375</v>
@@ -8912,13 +8927,13 @@
         <v>480</v>
       </c>
       <c r="H36" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="I36" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="J36" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="K36">
         <v>99</v>
@@ -8957,7 +8972,7 @@
         <v>-12.7</v>
       </c>
       <c r="W36" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="X36">
         <v>-0.003333</v>
@@ -8989,7 +9004,7 @@
         <v>25</v>
       </c>
       <c r="B37" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C37" s="2">
         <v>44023.3588266088</v>
@@ -9007,13 +9022,13 @@
         <v>506</v>
       </c>
       <c r="H37" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="I37" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="J37" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="K37">
         <v>138</v>
@@ -9040,7 +9055,7 @@
         <v>-11.8</v>
       </c>
       <c r="W37" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="X37">
         <v>0.03</v>
@@ -9072,7 +9087,7 @@
         <v>25</v>
       </c>
       <c r="B38" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C38" s="2">
         <v>44023.35887934027</v>
@@ -9090,13 +9105,13 @@
         <v>510</v>
       </c>
       <c r="H38" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="I38" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="J38" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="K38">
         <v>108</v>
@@ -9135,7 +9150,7 @@
         <v>-11.9</v>
       </c>
       <c r="W38" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="X38">
         <v>-0.003333</v>
@@ -9167,7 +9182,7 @@
         <v>25</v>
       </c>
       <c r="B39" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C39" s="2">
         <v>44023.3591712963</v>
@@ -9185,13 +9200,13 @@
         <v>536</v>
       </c>
       <c r="H39" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="I39" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="J39" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="K39">
         <v>133</v>
@@ -9218,7 +9233,7 @@
         <v>-11.16666667</v>
       </c>
       <c r="W39" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="X39">
         <v>0.024444</v>
@@ -9250,7 +9265,7 @@
         <v>25</v>
       </c>
       <c r="B40" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C40" s="2">
         <v>44023.35922280093</v>
@@ -9268,13 +9283,13 @@
         <v>540</v>
       </c>
       <c r="H40" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="I40" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="J40" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="K40">
         <v>120</v>
@@ -9313,7 +9328,7 @@
         <v>-10.9</v>
       </c>
       <c r="W40" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="X40">
         <v>0.008888999999999999</v>
@@ -9345,7 +9360,7 @@
         <v>25</v>
       </c>
       <c r="B41" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C41" s="2">
         <v>44023.35952256944</v>
@@ -9363,13 +9378,13 @@
         <v>566</v>
       </c>
       <c r="H41" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="I41" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="J41" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="K41">
         <v>193</v>
@@ -9396,7 +9411,7 @@
         <v>-11.6</v>
       </c>
       <c r="W41" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="X41">
         <v>-0.023333</v>
@@ -9428,7 +9443,7 @@
         <v>25</v>
       </c>
       <c r="B42" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C42" s="2">
         <v>44023.35956898148</v>
@@ -9446,13 +9461,13 @@
         <v>570</v>
       </c>
       <c r="H42" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="I42" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="J42" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="K42">
         <v>176</v>
@@ -9491,7 +9506,7 @@
         <v>-12.16666667</v>
       </c>
       <c r="W42" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="X42">
         <v>-0.018889</v>
@@ -9523,7 +9538,7 @@
         <v>25</v>
       </c>
       <c r="B43" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C43" s="2">
         <v>44023.35986965278</v>
@@ -9541,13 +9556,13 @@
         <v>596</v>
       </c>
       <c r="H43" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="I43" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="J43" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="K43">
         <v>195</v>
@@ -9574,7 +9589,7 @@
         <v>-11.7</v>
       </c>
       <c r="W43" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="X43">
         <v>0.015556</v>
@@ -9606,7 +9621,7 @@
         <v>25</v>
       </c>
       <c r="B44" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C44" s="2">
         <v>44023.35991907407</v>
@@ -9624,13 +9639,13 @@
         <v>600</v>
       </c>
       <c r="H44" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="I44" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="J44" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="K44">
         <v>200</v>
@@ -9669,7 +9684,7 @@
         <v>-11.13333333</v>
       </c>
       <c r="W44" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="X44">
         <v>0.018889</v>
@@ -9701,7 +9716,7 @@
         <v>25</v>
       </c>
       <c r="B45" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C45" s="2">
         <v>44023.36026780093</v>
@@ -9719,13 +9734,13 @@
         <v>630</v>
       </c>
       <c r="H45" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="I45" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="J45" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="K45">
         <v>193</v>
@@ -9764,7 +9779,7 @@
         <v>-13.3</v>
       </c>
       <c r="W45" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="X45">
         <v>-0.07222199999999999</v>
@@ -9796,7 +9811,7 @@
         <v>25</v>
       </c>
       <c r="B46" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C46" s="2">
         <v>44023.36056296296</v>
@@ -9814,13 +9829,13 @@
         <v>656</v>
       </c>
       <c r="H46" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="I46" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="J46" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="K46">
         <v>203</v>
@@ -9847,7 +9862,7 @@
         <v>-13.78333333</v>
       </c>
       <c r="W46" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="X46">
         <v>-0.008056000000000001</v>
@@ -9879,7 +9894,7 @@
         <v>25</v>
       </c>
       <c r="B47" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C47" s="2">
         <v>44023.36061483796</v>
@@ -9897,13 +9912,13 @@
         <v>660</v>
       </c>
       <c r="H47" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="I47" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="J47" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="K47">
         <v>193</v>
@@ -9942,7 +9957,7 @@
         <v>-14.6</v>
       </c>
       <c r="W47" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="X47">
         <v>-0.027222</v>
@@ -9974,7 +9989,7 @@
         <v>25</v>
       </c>
       <c r="B48" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C48" s="2">
         <v>44023.36369013889</v>
@@ -9992,13 +10007,13 @@
         <v>926</v>
       </c>
       <c r="H48" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="I48" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="J48" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="K48">
         <v>204</v>
@@ -10025,7 +10040,7 @@
         <v>-1.38518519</v>
       </c>
       <c r="W48" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="X48">
         <v>0.048944</v>

</xml_diff>

<commit_message>
Update flight data, addition of parachute data for all flights, and fixups for imperical/metric conversions for balloon sizes
</commit_message>
<xml_diff>
--- a/www/flightdata/xlsx/eoss-300.xlsx
+++ b/www/flightdata/xlsx/eoss-300.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="711" uniqueCount="291">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="721" uniqueCount="301">
   <si>
     <t>flight</t>
   </si>
@@ -57,6 +57,21 @@
     <t>range_distance_traveled_km</t>
   </si>
   <si>
+    <t>parachute.description</t>
+  </si>
+  <si>
+    <t>parachute.size_ft</t>
+  </si>
+  <si>
+    <t>parachute.size_m</t>
+  </si>
+  <si>
+    <t>parachute.weight_lb</t>
+  </si>
+  <si>
+    <t>parachute.weight_kg</t>
+  </si>
+  <si>
     <t>weights.client_lb</t>
   </si>
   <si>
@@ -99,6 +114,15 @@
     <t>weights.necklift_kg</t>
   </si>
   <si>
+    <t>detected_burst.detected</t>
+  </si>
+  <si>
+    <t>detected_burst.burst_ft</t>
+  </si>
+  <si>
+    <t>detected_burst.burst_m</t>
+  </si>
+  <si>
     <t>launch_location.latitude</t>
   </si>
   <si>
@@ -148,6 +172,12 @@
   </si>
   <si>
     <t>0hrs 25mins 26secs</t>
+  </si>
+  <si>
+    <t>Rocketman</t>
+  </si>
+  <si>
+    <t>12</t>
   </si>
   <si>
     <t>flightid</t>
@@ -1250,10 +1280,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AK2"/>
+  <dimension ref="A1:AS2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:37">
+    <row r="1" spans="1:45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1365,25 +1395,49 @@
       <c r="AK1" s="1" t="s">
         <v>36</v>
       </c>
+      <c r="AL1" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="AM1" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="AN1" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="AO1" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="AP1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="AQ1" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="AR1" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="AS1" s="1" t="s">
+        <v>44</v>
+      </c>
     </row>
-    <row r="2" spans="1:37">
+    <row r="2" spans="1:45">
       <c r="A2" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B2" t="s">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="C2" t="s">
-        <v>39</v>
+        <v>47</v>
       </c>
       <c r="D2" t="s">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="E2" t="s">
-        <v>41</v>
+        <v>49</v>
       </c>
       <c r="F2" t="s">
-        <v>42</v>
+        <v>50</v>
       </c>
       <c r="G2">
         <v>11223</v>
@@ -1395,7 +1449,7 @@
         <v>95</v>
       </c>
       <c r="J2" t="s">
-        <v>43</v>
+        <v>51</v>
       </c>
       <c r="K2">
         <v>1526</v>
@@ -1406,76 +1460,100 @@
       <c r="M2">
         <v>6.95</v>
       </c>
-      <c r="N2">
+      <c r="N2" t="s">
+        <v>52</v>
+      </c>
+      <c r="O2" t="s">
+        <v>53</v>
+      </c>
+      <c r="P2">
+        <v>3.66</v>
+      </c>
+      <c r="Q2">
+        <v>1.63</v>
+      </c>
+      <c r="R2">
+        <v>0.74</v>
+      </c>
+      <c r="S2">
         <v>0.12</v>
       </c>
-      <c r="O2">
+      <c r="T2">
         <v>0.05</v>
       </c>
-      <c r="P2">
+      <c r="U2">
         <v>6.66</v>
       </c>
-      <c r="Q2">
+      <c r="V2">
         <v>3.02</v>
       </c>
-      <c r="R2">
+      <c r="W2">
         <v>1.63</v>
       </c>
-      <c r="S2">
+      <c r="X2">
         <v>0.74</v>
       </c>
-      <c r="T2">
+      <c r="Y2">
         <v>8.41</v>
       </c>
-      <c r="U2">
+      <c r="Z2">
         <v>3.81</v>
       </c>
-      <c r="V2">
+      <c r="AA2">
         <v>3.31</v>
       </c>
-      <c r="W2">
+      <c r="AB2">
         <v>1.5</v>
       </c>
-      <c r="X2">
+      <c r="AC2">
         <v>11.72</v>
       </c>
-      <c r="Y2">
+      <c r="AD2">
         <v>5.32</v>
       </c>
-      <c r="Z2">
+      <c r="AE2">
         <v>11.34</v>
       </c>
-      <c r="AA2">
+      <c r="AF2">
         <v>5.14</v>
       </c>
-      <c r="AB2">
+      <c r="AG2" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH2">
+        <v>0</v>
+      </c>
+      <c r="AI2">
+        <v>0</v>
+      </c>
+      <c r="AJ2">
         <v>40.6488333333</v>
       </c>
-      <c r="AC2">
+      <c r="AK2">
         <v>-104.3843333333</v>
       </c>
-      <c r="AD2">
+      <c r="AL2">
         <v>4995</v>
       </c>
-      <c r="AE2">
+      <c r="AM2">
         <v>1522.48</v>
       </c>
-      <c r="AF2">
+      <c r="AN2">
         <v>40.6065166667</v>
       </c>
-      <c r="AG2">
+      <c r="AO2">
         <v>-104.3236833333</v>
       </c>
-      <c r="AH2">
+      <c r="AP2">
         <v>4.32</v>
       </c>
-      <c r="AI2">
+      <c r="AQ2">
         <v>6.95</v>
       </c>
-      <c r="AJ2">
+      <c r="AR2">
         <v>4866</v>
       </c>
-      <c r="AK2">
+      <c r="AS2">
         <v>1483.16</v>
       </c>
     </row>
@@ -1491,156 +1569,156 @@
   <sheetData>
     <row r="1" spans="1:48">
       <c r="A1" s="1" t="s">
-        <v>44</v>
+        <v>54</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>46</v>
+        <v>56</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>47</v>
+        <v>57</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>48</v>
+        <v>58</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>49</v>
+        <v>59</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>53</v>
+        <v>63</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>54</v>
+        <v>64</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>55</v>
+        <v>65</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>56</v>
+        <v>66</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>57</v>
+        <v>67</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>59</v>
+        <v>69</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>61</v>
+        <v>71</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>62</v>
+        <v>72</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>63</v>
+        <v>73</v>
       </c>
       <c r="U1" s="1" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="V1" s="1" t="s">
-        <v>65</v>
+        <v>75</v>
       </c>
       <c r="W1" s="1" t="s">
-        <v>66</v>
+        <v>76</v>
       </c>
       <c r="X1" s="1" t="s">
-        <v>67</v>
+        <v>77</v>
       </c>
       <c r="Y1" s="1" t="s">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="Z1" s="1" t="s">
-        <v>69</v>
+        <v>79</v>
       </c>
       <c r="AA1" s="1" t="s">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="AB1" s="1" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
       <c r="AC1" s="1" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
       <c r="AD1" s="1" t="s">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="AE1" s="1" t="s">
-        <v>74</v>
+        <v>84</v>
       </c>
       <c r="AF1" s="1" t="s">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="AG1" s="1" t="s">
-        <v>76</v>
+        <v>86</v>
       </c>
       <c r="AH1" s="1" t="s">
-        <v>77</v>
+        <v>87</v>
       </c>
       <c r="AI1" s="1" t="s">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="AJ1" s="1" t="s">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="AK1" s="1" t="s">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="AL1" s="1" t="s">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="AM1" s="1" t="s">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="AN1" s="1" t="s">
-        <v>83</v>
+        <v>93</v>
       </c>
       <c r="AO1" s="1" t="s">
-        <v>84</v>
+        <v>94</v>
       </c>
       <c r="AP1" s="1" t="s">
-        <v>85</v>
+        <v>95</v>
       </c>
       <c r="AQ1" s="1" t="s">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="AR1" s="1" t="s">
-        <v>87</v>
+        <v>97</v>
       </c>
       <c r="AS1" s="1" t="s">
-        <v>88</v>
+        <v>98</v>
       </c>
       <c r="AT1" s="1" t="s">
-        <v>89</v>
+        <v>99</v>
       </c>
       <c r="AU1" s="1" t="s">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="AV1" s="1" t="s">
-        <v>91</v>
+        <v>101</v>
       </c>
     </row>
     <row r="2" spans="1:48">
       <c r="A2" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B2" t="s">
-        <v>92</v>
+        <v>102</v>
       </c>
       <c r="C2" s="2">
         <v>44023.34605479167</v>
@@ -1661,16 +1739,16 @@
         <v>0</v>
       </c>
       <c r="I2" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="J2" t="b">
         <v>1</v>
       </c>
       <c r="K2" t="s">
-        <v>96</v>
+        <v>106</v>
       </c>
       <c r="L2" t="s">
-        <v>144</v>
+        <v>154</v>
       </c>
       <c r="M2">
         <v>164</v>
@@ -1727,7 +1805,7 @@
         <v>0.23366667</v>
       </c>
       <c r="AE2" t="s">
-        <v>192</v>
+        <v>202</v>
       </c>
       <c r="AG2">
         <v>0.766667</v>
@@ -1744,10 +1822,10 @@
     </row>
     <row r="3" spans="1:48">
       <c r="A3" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B3" t="s">
-        <v>93</v>
+        <v>103</v>
       </c>
       <c r="C3" s="2">
         <v>44023.34644167824</v>
@@ -1768,16 +1846,16 @@
         <v>30</v>
       </c>
       <c r="I3" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="J3" t="b">
         <v>1</v>
       </c>
       <c r="K3" t="s">
-        <v>97</v>
+        <v>107</v>
       </c>
       <c r="L3" t="s">
-        <v>145</v>
+        <v>155</v>
       </c>
       <c r="M3">
         <v>204</v>
@@ -1834,7 +1912,7 @@
         <v>1.38166667</v>
       </c>
       <c r="AE3" t="s">
-        <v>192</v>
+        <v>202</v>
       </c>
       <c r="AF3">
         <v>0.125556</v>
@@ -1875,10 +1953,10 @@
     </row>
     <row r="4" spans="1:48">
       <c r="A4" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B4" t="s">
-        <v>94</v>
+        <v>104</v>
       </c>
       <c r="C4" s="2">
         <v>44023.34667440972</v>
@@ -1899,16 +1977,16 @@
         <v>56</v>
       </c>
       <c r="I4" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="J4" t="b">
         <v>1</v>
       </c>
       <c r="K4" t="s">
-        <v>98</v>
+        <v>108</v>
       </c>
       <c r="L4" t="s">
-        <v>146</v>
+        <v>156</v>
       </c>
       <c r="M4">
         <v>214</v>
@@ -1944,7 +2022,7 @@
         <v>2.032</v>
       </c>
       <c r="AE4" t="s">
-        <v>192</v>
+        <v>202</v>
       </c>
       <c r="AF4">
         <v>0.035556</v>
@@ -1997,10 +2075,10 @@
     </row>
     <row r="5" spans="1:48">
       <c r="A5" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B5" t="s">
-        <v>93</v>
+        <v>103</v>
       </c>
       <c r="C5" s="2">
         <v>44023.34674237268</v>
@@ -2021,16 +2099,16 @@
         <v>60</v>
       </c>
       <c r="I5" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="J5" t="b">
         <v>1</v>
       </c>
       <c r="K5" t="s">
-        <v>99</v>
+        <v>109</v>
       </c>
       <c r="L5" t="s">
-        <v>147</v>
+        <v>157</v>
       </c>
       <c r="M5">
         <v>209</v>
@@ -2087,7 +2165,7 @@
         <v>4.511</v>
       </c>
       <c r="AE5" t="s">
-        <v>192</v>
+        <v>202</v>
       </c>
       <c r="AF5">
         <v>0.271111</v>
@@ -2140,10 +2218,10 @@
     </row>
     <row r="6" spans="1:48">
       <c r="A6" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B6" t="s">
-        <v>94</v>
+        <v>104</v>
       </c>
       <c r="C6" s="2">
         <v>44023.34702186342</v>
@@ -2164,16 +2242,16 @@
         <v>86</v>
       </c>
       <c r="I6" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="J6" t="b">
         <v>1</v>
       </c>
       <c r="K6" t="s">
-        <v>100</v>
+        <v>110</v>
       </c>
       <c r="L6" t="s">
-        <v>148</v>
+        <v>158</v>
       </c>
       <c r="M6">
         <v>210</v>
@@ -2209,7 +2287,7 @@
         <v>5.10033333</v>
       </c>
       <c r="AE6" t="s">
-        <v>192</v>
+        <v>202</v>
       </c>
       <c r="AF6">
         <v>0.064444</v>
@@ -2262,10 +2340,10 @@
     </row>
     <row r="7" spans="1:48">
       <c r="A7" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B7" t="s">
-        <v>93</v>
+        <v>103</v>
       </c>
       <c r="C7" s="2">
         <v>44023.34707267361</v>
@@ -2286,16 +2364,16 @@
         <v>90</v>
       </c>
       <c r="I7" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="J7" t="b">
         <v>1</v>
       </c>
       <c r="K7" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="L7" t="s">
-        <v>149</v>
+        <v>159</v>
       </c>
       <c r="M7">
         <v>211</v>
@@ -2352,7 +2430,7 @@
         <v>5.02933333</v>
       </c>
       <c r="AE7" t="s">
-        <v>192</v>
+        <v>202</v>
       </c>
       <c r="AF7">
         <v>-0.007778</v>
@@ -2405,10 +2483,10 @@
     </row>
     <row r="8" spans="1:48">
       <c r="A8" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B8" t="s">
-        <v>94</v>
+        <v>104</v>
       </c>
       <c r="C8" s="2">
         <v>44023.3473683912</v>
@@ -2429,16 +2507,16 @@
         <v>116</v>
       </c>
       <c r="I8" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="J8" t="b">
         <v>1</v>
       </c>
       <c r="K8" t="s">
-        <v>102</v>
+        <v>112</v>
       </c>
       <c r="L8" t="s">
-        <v>150</v>
+        <v>160</v>
       </c>
       <c r="M8">
         <v>165</v>
@@ -2474,7 +2552,7 @@
         <v>5.23233333</v>
       </c>
       <c r="AE8" t="s">
-        <v>192</v>
+        <v>202</v>
       </c>
       <c r="AF8">
         <v>0.022222</v>
@@ -2527,10 +2605,10 @@
     </row>
     <row r="9" spans="1:48">
       <c r="A9" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B9" t="s">
-        <v>92</v>
+        <v>102</v>
       </c>
       <c r="C9" s="2">
         <v>44023.34744381945</v>
@@ -2551,16 +2629,16 @@
         <v>120</v>
       </c>
       <c r="I9" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="J9" t="b">
         <v>1</v>
       </c>
       <c r="K9" t="s">
-        <v>103</v>
+        <v>113</v>
       </c>
       <c r="L9" t="s">
-        <v>151</v>
+        <v>161</v>
       </c>
       <c r="M9">
         <v>157</v>
@@ -2617,7 +2695,7 @@
         <v>3.88616667</v>
       </c>
       <c r="AE9" t="s">
-        <v>192</v>
+        <v>202</v>
       </c>
       <c r="AF9">
         <v>-0.036806</v>
@@ -2670,10 +2748,10 @@
     </row>
     <row r="10" spans="1:48">
       <c r="A10" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B10" t="s">
-        <v>93</v>
+        <v>103</v>
       </c>
       <c r="C10" s="2">
         <v>44023.34741728009</v>
@@ -2694,16 +2772,16 @@
         <v>120</v>
       </c>
       <c r="I10" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="J10" t="b">
         <v>1</v>
       </c>
       <c r="K10" t="s">
-        <v>104</v>
+        <v>114</v>
       </c>
       <c r="L10" t="s">
-        <v>152</v>
+        <v>162</v>
       </c>
       <c r="M10">
         <v>157</v>
@@ -2760,7 +2838,7 @@
         <v>5.25266667</v>
       </c>
       <c r="AE10" t="s">
-        <v>192</v>
+        <v>202</v>
       </c>
       <c r="AF10">
         <v>0.149444</v>
@@ -2813,10 +2891,10 @@
     </row>
     <row r="11" spans="1:48">
       <c r="A11" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B11" t="s">
-        <v>94</v>
+        <v>104</v>
       </c>
       <c r="C11" s="2">
         <v>44023.34771681713</v>
@@ -2837,16 +2915,16 @@
         <v>146</v>
       </c>
       <c r="I11" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="J11" t="b">
         <v>1</v>
       </c>
       <c r="K11" t="s">
-        <v>105</v>
+        <v>115</v>
       </c>
       <c r="L11" t="s">
-        <v>153</v>
+        <v>163</v>
       </c>
       <c r="M11">
         <v>119</v>
@@ -2882,7 +2960,7 @@
         <v>5.10033333</v>
       </c>
       <c r="AE11" t="s">
-        <v>192</v>
+        <v>202</v>
       </c>
       <c r="AF11">
         <v>-0.016667</v>
@@ -2935,10 +3013,10 @@
     </row>
     <row r="12" spans="1:48">
       <c r="A12" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B12" t="s">
-        <v>93</v>
+        <v>103</v>
       </c>
       <c r="C12" s="2">
         <v>44023.34776537037</v>
@@ -2959,16 +3037,16 @@
         <v>150</v>
       </c>
       <c r="I12" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="J12" t="b">
         <v>1</v>
       </c>
       <c r="K12" t="s">
-        <v>106</v>
+        <v>116</v>
       </c>
       <c r="L12" t="s">
-        <v>154</v>
+        <v>164</v>
       </c>
       <c r="M12">
         <v>118</v>
@@ -3025,7 +3103,7 @@
         <v>5.19166667</v>
       </c>
       <c r="AE12" t="s">
-        <v>192</v>
+        <v>202</v>
       </c>
       <c r="AF12">
         <v>0.01</v>
@@ -3078,10 +3156,10 @@
     </row>
     <row r="13" spans="1:48">
       <c r="A13" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B13" t="s">
-        <v>94</v>
+        <v>104</v>
       </c>
       <c r="C13" s="2">
         <v>44023.34806101852</v>
@@ -3102,16 +3180,16 @@
         <v>176</v>
       </c>
       <c r="I13" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="J13" t="b">
         <v>1</v>
       </c>
       <c r="K13" t="s">
-        <v>107</v>
+        <v>117</v>
       </c>
       <c r="L13" t="s">
-        <v>155</v>
+        <v>165</v>
       </c>
       <c r="M13">
         <v>178</v>
@@ -3147,7 +3225,7 @@
         <v>4.73466667</v>
       </c>
       <c r="AE13" t="s">
-        <v>192</v>
+        <v>202</v>
       </c>
       <c r="AF13">
         <v>-0.05</v>
@@ -3200,10 +3278,10 @@
     </row>
     <row r="14" spans="1:48">
       <c r="A14" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B14" t="s">
-        <v>92</v>
+        <v>102</v>
       </c>
       <c r="C14" s="2">
         <v>44023.34813881944</v>
@@ -3224,16 +3302,16 @@
         <v>180</v>
       </c>
       <c r="I14" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="J14" t="b">
         <v>1</v>
       </c>
       <c r="K14" t="s">
-        <v>108</v>
+        <v>118</v>
       </c>
       <c r="L14" t="s">
-        <v>156</v>
+        <v>166</v>
       </c>
       <c r="M14">
         <v>103</v>
@@ -3290,7 +3368,7 @@
         <v>4.831</v>
       </c>
       <c r="AE14" t="s">
-        <v>192</v>
+        <v>202</v>
       </c>
       <c r="AF14">
         <v>0.005278</v>
@@ -3343,10 +3421,10 @@
     </row>
     <row r="15" spans="1:48">
       <c r="A15" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B15" t="s">
-        <v>93</v>
+        <v>103</v>
       </c>
       <c r="C15" s="2">
         <v>44023.34811263889</v>
@@ -3367,16 +3445,16 @@
         <v>180</v>
       </c>
       <c r="I15" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="J15" t="b">
         <v>1</v>
       </c>
       <c r="K15" t="s">
-        <v>109</v>
+        <v>119</v>
       </c>
       <c r="L15" t="s">
-        <v>157</v>
+        <v>167</v>
       </c>
       <c r="M15">
         <v>112</v>
@@ -3433,7 +3511,7 @@
         <v>4.60266667</v>
       </c>
       <c r="AE15" t="s">
-        <v>192</v>
+        <v>202</v>
       </c>
       <c r="AF15">
         <v>-0.025</v>
@@ -3486,10 +3564,10 @@
     </row>
     <row r="16" spans="1:48">
       <c r="A16" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B16" t="s">
-        <v>94</v>
+        <v>104</v>
       </c>
       <c r="C16" s="2">
         <v>44023.3484072338</v>
@@ -3510,16 +3588,16 @@
         <v>206</v>
       </c>
       <c r="I16" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="J16" t="b">
         <v>1</v>
       </c>
       <c r="K16" t="s">
-        <v>110</v>
+        <v>120</v>
       </c>
       <c r="L16" t="s">
-        <v>158</v>
+        <v>168</v>
       </c>
       <c r="M16">
         <v>149</v>
@@ -3555,7 +3633,7 @@
         <v>4.206</v>
       </c>
       <c r="AE16" t="s">
-        <v>192</v>
+        <v>202</v>
       </c>
       <c r="AF16">
         <v>-0.043333</v>
@@ -3608,10 +3686,10 @@
     </row>
     <row r="17" spans="1:48">
       <c r="A17" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B17" t="s">
-        <v>93</v>
+        <v>103</v>
       </c>
       <c r="C17" s="2">
         <v>44023.3484581713</v>
@@ -3632,16 +3710,16 @@
         <v>210</v>
       </c>
       <c r="I17" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="J17" t="b">
         <v>1</v>
       </c>
       <c r="K17" t="s">
-        <v>111</v>
+        <v>121</v>
       </c>
       <c r="L17" t="s">
-        <v>159</v>
+        <v>169</v>
       </c>
       <c r="M17">
         <v>137</v>
@@ -3698,7 +3776,7 @@
         <v>4.20633333</v>
       </c>
       <c r="AE17" t="s">
-        <v>192</v>
+        <v>202</v>
       </c>
       <c r="AF17">
         <v>0</v>
@@ -3751,10 +3829,10 @@
     </row>
     <row r="18" spans="1:48">
       <c r="A18" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B18" t="s">
-        <v>92</v>
+        <v>102</v>
       </c>
       <c r="C18" s="2">
         <v>44023.34846752314</v>
@@ -3775,16 +3853,16 @@
         <v>210</v>
       </c>
       <c r="I18" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="J18" t="b">
         <v>1</v>
       </c>
       <c r="K18" t="s">
-        <v>112</v>
+        <v>122</v>
       </c>
       <c r="L18" t="s">
-        <v>160</v>
+        <v>170</v>
       </c>
       <c r="M18">
         <v>134</v>
@@ -3841,7 +3919,7 @@
         <v>4.39933333</v>
       </c>
       <c r="AE18" t="s">
-        <v>192</v>
+        <v>202</v>
       </c>
       <c r="AF18">
         <v>0.021111</v>
@@ -3894,10 +3972,10 @@
     </row>
     <row r="19" spans="1:48">
       <c r="A19" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B19" t="s">
-        <v>93</v>
+        <v>103</v>
       </c>
       <c r="C19" s="2">
         <v>44023.34880686343</v>
@@ -3918,16 +3996,16 @@
         <v>240</v>
       </c>
       <c r="I19" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="J19" t="b">
         <v>1</v>
       </c>
       <c r="K19" t="s">
-        <v>113</v>
+        <v>123</v>
       </c>
       <c r="L19" t="s">
-        <v>161</v>
+        <v>171</v>
       </c>
       <c r="M19">
         <v>95</v>
@@ -3984,7 +4062,7 @@
         <v>4.064</v>
       </c>
       <c r="AE19" t="s">
-        <v>192</v>
+        <v>202</v>
       </c>
       <c r="AF19">
         <v>-0.036667</v>
@@ -4037,10 +4115,10 @@
     </row>
     <row r="20" spans="1:48">
       <c r="A20" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B20" t="s">
-        <v>92</v>
+        <v>102</v>
       </c>
       <c r="C20" s="2">
         <v>44023.34883809028</v>
@@ -4061,16 +4139,16 @@
         <v>240</v>
       </c>
       <c r="I20" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="J20" t="b">
         <v>1</v>
       </c>
       <c r="K20" t="s">
-        <v>114</v>
+        <v>124</v>
       </c>
       <c r="L20" t="s">
-        <v>162</v>
+        <v>172</v>
       </c>
       <c r="M20">
         <v>100</v>
@@ -4127,7 +4205,7 @@
         <v>3.82033333</v>
       </c>
       <c r="AE20" t="s">
-        <v>192</v>
+        <v>202</v>
       </c>
       <c r="AF20">
         <v>-0.026667</v>
@@ -4180,10 +4258,10 @@
     </row>
     <row r="21" spans="1:48">
       <c r="A21" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B21" t="s">
-        <v>93</v>
+        <v>103</v>
       </c>
       <c r="C21" s="2">
         <v>44023.34915288194</v>
@@ -4204,16 +4282,16 @@
         <v>270</v>
       </c>
       <c r="I21" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="J21" t="b">
         <v>1</v>
       </c>
       <c r="K21" t="s">
-        <v>115</v>
+        <v>125</v>
       </c>
       <c r="L21" t="s">
-        <v>163</v>
+        <v>173</v>
       </c>
       <c r="M21">
         <v>106</v>
@@ -4270,7 +4348,7 @@
         <v>4.75466667</v>
       </c>
       <c r="AE21" t="s">
-        <v>192</v>
+        <v>202</v>
       </c>
       <c r="AF21">
         <v>0.102222</v>
@@ -4323,10 +4401,10 @@
     </row>
     <row r="22" spans="1:48">
       <c r="A22" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B22" t="s">
-        <v>92</v>
+        <v>102</v>
       </c>
       <c r="C22" s="2">
         <v>44023.34916229167</v>
@@ -4347,16 +4425,16 @@
         <v>270</v>
       </c>
       <c r="I22" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="J22" t="b">
         <v>1</v>
       </c>
       <c r="K22" t="s">
-        <v>116</v>
+        <v>126</v>
       </c>
       <c r="L22" t="s">
-        <v>164</v>
+        <v>174</v>
       </c>
       <c r="M22">
         <v>111</v>
@@ -4413,7 +4491,7 @@
         <v>4.54133333</v>
       </c>
       <c r="AE22" t="s">
-        <v>192</v>
+        <v>202</v>
       </c>
       <c r="AF22">
         <v>-0.023333</v>
@@ -4466,10 +4544,10 @@
     </row>
     <row r="23" spans="1:48">
       <c r="A23" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B23" t="s">
-        <v>94</v>
+        <v>104</v>
       </c>
       <c r="C23" s="2">
         <v>44023.34945041667</v>
@@ -4490,16 +4568,16 @@
         <v>296</v>
       </c>
       <c r="I23" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="J23" t="b">
         <v>1</v>
       </c>
       <c r="K23" t="s">
-        <v>117</v>
+        <v>127</v>
       </c>
       <c r="L23" t="s">
-        <v>165</v>
+        <v>175</v>
       </c>
       <c r="M23">
         <v>109</v>
@@ -4535,7 +4613,7 @@
         <v>4.423</v>
       </c>
       <c r="AE23" t="s">
-        <v>192</v>
+        <v>202</v>
       </c>
       <c r="AF23">
         <v>-0.004321</v>
@@ -4588,10 +4666,10 @@
     </row>
     <row r="24" spans="1:48">
       <c r="A24" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B24" t="s">
-        <v>93</v>
+        <v>103</v>
       </c>
       <c r="C24" s="2">
         <v>44023.34949959491</v>
@@ -4612,16 +4690,16 @@
         <v>300</v>
       </c>
       <c r="I24" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="J24" t="b">
         <v>1</v>
       </c>
       <c r="K24" t="s">
-        <v>118</v>
+        <v>128</v>
       </c>
       <c r="L24" t="s">
-        <v>166</v>
+        <v>176</v>
       </c>
       <c r="M24">
         <v>102</v>
@@ -4678,7 +4756,7 @@
         <v>4.39933333</v>
       </c>
       <c r="AE24" t="s">
-        <v>192</v>
+        <v>202</v>
       </c>
       <c r="AF24">
         <v>-0.002593</v>
@@ -4731,10 +4809,10 @@
     </row>
     <row r="25" spans="1:48">
       <c r="A25" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B25" t="s">
-        <v>92</v>
+        <v>102</v>
       </c>
       <c r="C25" s="2">
         <v>44023.34952732639</v>
@@ -4755,16 +4833,16 @@
         <v>300</v>
       </c>
       <c r="I25" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="J25" t="b">
         <v>1</v>
       </c>
       <c r="K25" t="s">
-        <v>119</v>
+        <v>129</v>
       </c>
       <c r="L25" t="s">
-        <v>167</v>
+        <v>177</v>
       </c>
       <c r="M25">
         <v>104</v>
@@ -4821,7 +4899,7 @@
         <v>4.684</v>
       </c>
       <c r="AE25" t="s">
-        <v>192</v>
+        <v>202</v>
       </c>
       <c r="AF25">
         <v>0.031111</v>
@@ -4874,10 +4952,10 @@
     </row>
     <row r="26" spans="1:48">
       <c r="A26" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B26" t="s">
-        <v>94</v>
+        <v>104</v>
       </c>
       <c r="C26" s="2">
         <v>44023.34979804398</v>
@@ -4898,16 +4976,16 @@
         <v>326</v>
       </c>
       <c r="I26" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="J26" t="b">
         <v>1</v>
       </c>
       <c r="K26" t="s">
-        <v>120</v>
+        <v>130</v>
       </c>
       <c r="L26" t="s">
-        <v>168</v>
+        <v>178</v>
       </c>
       <c r="M26">
         <v>128</v>
@@ -4943,7 +5021,7 @@
         <v>3.932</v>
       </c>
       <c r="AE26" t="s">
-        <v>192</v>
+        <v>202</v>
       </c>
       <c r="AF26">
         <v>-0.082222</v>
@@ -4996,10 +5074,10 @@
     </row>
     <row r="27" spans="1:48">
       <c r="A27" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B27" t="s">
-        <v>93</v>
+        <v>103</v>
       </c>
       <c r="C27" s="2">
         <v>44023.34984708334</v>
@@ -5020,16 +5098,16 @@
         <v>330</v>
       </c>
       <c r="I27" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="J27" t="b">
         <v>1</v>
       </c>
       <c r="K27" t="s">
-        <v>121</v>
+        <v>131</v>
       </c>
       <c r="L27" t="s">
-        <v>169</v>
+        <v>179</v>
       </c>
       <c r="M27">
         <v>111</v>
@@ -5086,7 +5164,7 @@
         <v>4.15533333</v>
       </c>
       <c r="AE27" t="s">
-        <v>192</v>
+        <v>202</v>
       </c>
       <c r="AF27">
         <v>0.024444</v>
@@ -5139,10 +5217,10 @@
     </row>
     <row r="28" spans="1:48">
       <c r="A28" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B28" t="s">
-        <v>93</v>
+        <v>103</v>
       </c>
       <c r="C28" s="2">
         <v>44023.35019421297</v>
@@ -5163,16 +5241,16 @@
         <v>360</v>
       </c>
       <c r="I28" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="J28" t="b">
         <v>1</v>
       </c>
       <c r="K28" t="s">
-        <v>122</v>
+        <v>132</v>
       </c>
       <c r="L28" t="s">
-        <v>170</v>
+        <v>180</v>
       </c>
       <c r="M28">
         <v>122</v>
@@ -5229,7 +5307,7 @@
         <v>4.28766667</v>
       </c>
       <c r="AE28" t="s">
-        <v>193</v>
+        <v>203</v>
       </c>
       <c r="AF28">
         <v>0.014444</v>
@@ -5280,15 +5358,15 @@
         <v>3.763535</v>
       </c>
       <c r="AV28" t="s">
-        <v>194</v>
+        <v>204</v>
       </c>
     </row>
     <row r="29" spans="1:48">
       <c r="A29" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B29" t="s">
-        <v>92</v>
+        <v>102</v>
       </c>
       <c r="C29" s="2">
         <v>44023.3502215625</v>
@@ -5309,16 +5387,16 @@
         <v>360</v>
       </c>
       <c r="I29" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="J29" t="b">
         <v>1</v>
       </c>
       <c r="K29" t="s">
-        <v>123</v>
+        <v>133</v>
       </c>
       <c r="L29" t="s">
-        <v>171</v>
+        <v>181</v>
       </c>
       <c r="M29">
         <v>125</v>
@@ -5375,7 +5453,7 @@
         <v>4.17566667</v>
       </c>
       <c r="AE29" t="s">
-        <v>193</v>
+        <v>203</v>
       </c>
       <c r="AF29">
         <v>-0.006111</v>
@@ -5428,10 +5506,10 @@
     </row>
     <row r="30" spans="1:48">
       <c r="A30" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B30" t="s">
-        <v>92</v>
+        <v>102</v>
       </c>
       <c r="C30" s="2">
         <v>44023.35055107639</v>
@@ -5452,16 +5530,16 @@
         <v>390</v>
       </c>
       <c r="I30" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="J30" t="b">
         <v>1</v>
       </c>
       <c r="K30" t="s">
-        <v>124</v>
+        <v>134</v>
       </c>
       <c r="L30" t="s">
-        <v>172</v>
+        <v>182</v>
       </c>
       <c r="M30">
         <v>121</v>
@@ -5518,7 +5596,7 @@
         <v>2.89566667</v>
       </c>
       <c r="AE30" t="s">
-        <v>193</v>
+        <v>203</v>
       </c>
       <c r="AF30">
         <v>-0.14</v>
@@ -5571,10 +5649,10 @@
     </row>
     <row r="31" spans="1:48">
       <c r="A31" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B31" t="s">
-        <v>93</v>
+        <v>103</v>
       </c>
       <c r="C31" s="2">
         <v>44023.35054172454</v>
@@ -5595,16 +5673,16 @@
         <v>390</v>
       </c>
       <c r="I31" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="J31" t="b">
         <v>1</v>
       </c>
       <c r="K31" t="s">
-        <v>125</v>
+        <v>135</v>
       </c>
       <c r="L31" t="s">
-        <v>173</v>
+        <v>183</v>
       </c>
       <c r="M31">
         <v>123</v>
@@ -5661,7 +5739,7 @@
         <v>2.48933333</v>
       </c>
       <c r="AE31" t="s">
-        <v>193</v>
+        <v>203</v>
       </c>
       <c r="AF31">
         <v>-0.044444</v>
@@ -5714,10 +5792,10 @@
     </row>
     <row r="32" spans="1:48">
       <c r="A32" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B32" t="s">
-        <v>94</v>
+        <v>104</v>
       </c>
       <c r="C32" s="2">
         <v>44023.35083818287</v>
@@ -5738,16 +5816,16 @@
         <v>416</v>
       </c>
       <c r="I32" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="J32" t="b">
         <v>1</v>
       </c>
       <c r="K32" t="s">
-        <v>126</v>
+        <v>136</v>
       </c>
       <c r="L32" t="s">
-        <v>174</v>
+        <v>184</v>
       </c>
       <c r="M32">
         <v>125</v>
@@ -5783,7 +5861,7 @@
         <v>2.99044444</v>
       </c>
       <c r="AE32" t="s">
-        <v>193</v>
+        <v>203</v>
       </c>
       <c r="AF32">
         <v>0.018272</v>
@@ -5836,10 +5914,10 @@
     </row>
     <row r="33" spans="1:47">
       <c r="A33" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B33" t="s">
-        <v>92</v>
+        <v>102</v>
       </c>
       <c r="C33" s="2">
         <v>44023.35091582176</v>
@@ -5860,16 +5938,16 @@
         <v>419</v>
       </c>
       <c r="I33" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="J33" t="b">
         <v>1</v>
       </c>
       <c r="K33" t="s">
-        <v>127</v>
+        <v>137</v>
       </c>
       <c r="L33" t="s">
-        <v>175</v>
+        <v>185</v>
       </c>
       <c r="M33">
         <v>117</v>
@@ -5926,7 +6004,7 @@
         <v>1.22965517</v>
       </c>
       <c r="AE33" t="s">
-        <v>193</v>
+        <v>203</v>
       </c>
       <c r="AF33">
         <v>-0.199194</v>
@@ -5979,10 +6057,10 @@
     </row>
     <row r="34" spans="1:47">
       <c r="A34" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B34" t="s">
-        <v>93</v>
+        <v>103</v>
       </c>
       <c r="C34" s="2">
         <v>44023.35088921296</v>
@@ -6003,16 +6081,16 @@
         <v>420</v>
       </c>
       <c r="I34" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="J34" t="b">
         <v>1</v>
       </c>
       <c r="K34" t="s">
-        <v>128</v>
+        <v>138</v>
       </c>
       <c r="L34" t="s">
-        <v>176</v>
+        <v>186</v>
       </c>
       <c r="M34">
         <v>117</v>
@@ -6069,7 +6147,7 @@
         <v>1.76766667</v>
       </c>
       <c r="AE34" t="s">
-        <v>193</v>
+        <v>203</v>
       </c>
       <c r="AF34">
         <v>0.058851</v>
@@ -6122,10 +6200,10 @@
     </row>
     <row r="35" spans="1:47">
       <c r="A35" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B35" t="s">
-        <v>94</v>
+        <v>104</v>
       </c>
       <c r="C35" s="2">
         <v>44023.35118658565</v>
@@ -6146,16 +6224,16 @@
         <v>446</v>
       </c>
       <c r="I35" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="J35" t="b">
         <v>1</v>
       </c>
       <c r="K35" t="s">
-        <v>129</v>
+        <v>139</v>
       </c>
       <c r="L35" t="s">
-        <v>177</v>
+        <v>187</v>
       </c>
       <c r="M35">
         <v>109</v>
@@ -6191,7 +6269,7 @@
         <v>1.66633333</v>
       </c>
       <c r="AE35" t="s">
-        <v>193</v>
+        <v>203</v>
       </c>
       <c r="AF35">
         <v>-0.011111</v>
@@ -6244,10 +6322,10 @@
     </row>
     <row r="36" spans="1:47">
       <c r="A36" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B36" t="s">
-        <v>93</v>
+        <v>103</v>
       </c>
       <c r="C36" s="2">
         <v>44023.35123702546</v>
@@ -6268,16 +6346,16 @@
         <v>450</v>
       </c>
       <c r="I36" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="J36" t="b">
         <v>1</v>
       </c>
       <c r="K36" t="s">
-        <v>130</v>
+        <v>140</v>
       </c>
       <c r="L36" t="s">
-        <v>178</v>
+        <v>188</v>
       </c>
       <c r="M36">
         <v>110</v>
@@ -6334,7 +6412,7 @@
         <v>1.646</v>
       </c>
       <c r="AE36" t="s">
-        <v>193</v>
+        <v>203</v>
       </c>
       <c r="AF36">
         <v>-0.002222</v>
@@ -6387,10 +6465,10 @@
     </row>
     <row r="37" spans="1:47">
       <c r="A37" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B37" t="s">
-        <v>92</v>
+        <v>102</v>
       </c>
       <c r="C37" s="2">
         <v>44023.35124731481</v>
@@ -6411,16 +6489,16 @@
         <v>450</v>
       </c>
       <c r="I37" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="J37" t="b">
         <v>1</v>
       </c>
       <c r="K37" t="s">
-        <v>131</v>
+        <v>141</v>
       </c>
       <c r="L37" t="s">
-        <v>179</v>
+        <v>189</v>
       </c>
       <c r="M37">
         <v>111</v>
@@ -6477,7 +6555,7 @@
         <v>1.8483871</v>
       </c>
       <c r="AE37" t="s">
-        <v>193</v>
+        <v>203</v>
       </c>
       <c r="AF37">
         <v>0.021436</v>
@@ -6530,10 +6608,10 @@
     </row>
     <row r="38" spans="1:47">
       <c r="A38" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B38" t="s">
-        <v>94</v>
+        <v>104</v>
       </c>
       <c r="C38" s="2">
         <v>44023.35153310185</v>
@@ -6554,16 +6632,16 @@
         <v>476</v>
       </c>
       <c r="I38" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="J38" t="b">
         <v>1</v>
       </c>
       <c r="K38" t="s">
-        <v>132</v>
+        <v>142</v>
       </c>
       <c r="L38" t="s">
-        <v>180</v>
+        <v>190</v>
       </c>
       <c r="M38">
         <v>114</v>
@@ -6599,7 +6677,7 @@
         <v>1.727</v>
       </c>
       <c r="AE38" t="s">
-        <v>193</v>
+        <v>203</v>
       </c>
       <c r="AF38">
         <v>-0.013262</v>
@@ -6652,10 +6730,10 @@
     </row>
     <row r="39" spans="1:47">
       <c r="A39" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B39" t="s">
-        <v>93</v>
+        <v>103</v>
       </c>
       <c r="C39" s="2">
         <v>44023.35158375</v>
@@ -6676,16 +6754,16 @@
         <v>480</v>
       </c>
       <c r="I39" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="J39" t="b">
         <v>1</v>
       </c>
       <c r="K39" t="s">
-        <v>133</v>
+        <v>143</v>
       </c>
       <c r="L39" t="s">
-        <v>181</v>
+        <v>191</v>
       </c>
       <c r="M39">
         <v>116</v>
@@ -6742,7 +6820,7 @@
         <v>1.76766667</v>
       </c>
       <c r="AE39" t="s">
-        <v>193</v>
+        <v>203</v>
       </c>
       <c r="AF39">
         <v>0.004444</v>
@@ -6795,10 +6873,10 @@
     </row>
     <row r="40" spans="1:47">
       <c r="A40" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B40" t="s">
-        <v>92</v>
+        <v>102</v>
       </c>
       <c r="C40" s="2">
         <v>44023.35161115741</v>
@@ -6819,16 +6897,16 @@
         <v>480</v>
       </c>
       <c r="I40" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="J40" t="b">
         <v>1</v>
       </c>
       <c r="K40" t="s">
-        <v>134</v>
+        <v>144</v>
       </c>
       <c r="L40" t="s">
-        <v>182</v>
+        <v>192</v>
       </c>
       <c r="M40">
         <v>114</v>
@@ -6885,7 +6963,7 @@
         <v>1.87966667</v>
       </c>
       <c r="AE40" t="s">
-        <v>193</v>
+        <v>203</v>
       </c>
       <c r="AF40">
         <v>0.012222</v>
@@ -6938,10 +7016,10 @@
     </row>
     <row r="41" spans="1:47">
       <c r="A41" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B41" t="s">
-        <v>94</v>
+        <v>104</v>
       </c>
       <c r="C41" s="2">
         <v>44023.35187935185</v>
@@ -6962,16 +7040,16 @@
         <v>506</v>
       </c>
       <c r="I41" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="J41" t="b">
         <v>1</v>
       </c>
       <c r="K41" t="s">
-        <v>135</v>
+        <v>145</v>
       </c>
       <c r="L41" t="s">
-        <v>183</v>
+        <v>193</v>
       </c>
       <c r="M41">
         <v>118</v>
@@ -7007,7 +7085,7 @@
         <v>1.73733333</v>
       </c>
       <c r="AE41" t="s">
-        <v>193</v>
+        <v>203</v>
       </c>
       <c r="AF41">
         <v>-0.015556</v>
@@ -7060,10 +7138,10 @@
     </row>
     <row r="42" spans="1:47">
       <c r="A42" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B42" t="s">
-        <v>93</v>
+        <v>103</v>
       </c>
       <c r="C42" s="2">
         <v>44023.35193064815</v>
@@ -7084,16 +7162,16 @@
         <v>510</v>
       </c>
       <c r="I42" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="J42" t="b">
         <v>1</v>
       </c>
       <c r="K42" t="s">
-        <v>136</v>
+        <v>146</v>
       </c>
       <c r="L42" t="s">
-        <v>184</v>
+        <v>194</v>
       </c>
       <c r="M42">
         <v>118</v>
@@ -7150,7 +7228,7 @@
         <v>1.636</v>
       </c>
       <c r="AE42" t="s">
-        <v>193</v>
+        <v>203</v>
       </c>
       <c r="AF42">
         <v>-0.011111</v>
@@ -7203,10 +7281,10 @@
     </row>
     <row r="43" spans="1:47">
       <c r="A43" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B43" t="s">
-        <v>92</v>
+        <v>102</v>
       </c>
       <c r="C43" s="2">
         <v>44023.35194001158</v>
@@ -7227,16 +7305,16 @@
         <v>510</v>
       </c>
       <c r="I43" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="J43" t="b">
         <v>1</v>
       </c>
       <c r="K43" t="s">
-        <v>137</v>
+        <v>147</v>
       </c>
       <c r="L43" t="s">
-        <v>185</v>
+        <v>195</v>
       </c>
       <c r="M43">
         <v>118</v>
@@ -7293,7 +7371,7 @@
         <v>1.61566667</v>
       </c>
       <c r="AE43" t="s">
-        <v>193</v>
+        <v>203</v>
       </c>
       <c r="AF43">
         <v>-0.002222</v>
@@ -7346,10 +7424,10 @@
     </row>
     <row r="44" spans="1:47">
       <c r="A44" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B44" t="s">
-        <v>93</v>
+        <v>103</v>
       </c>
       <c r="C44" s="2">
         <v>44023.35227842593</v>
@@ -7370,16 +7448,16 @@
         <v>540</v>
       </c>
       <c r="I44" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="J44" t="b">
         <v>1</v>
       </c>
       <c r="K44" t="s">
-        <v>138</v>
+        <v>148</v>
       </c>
       <c r="L44" t="s">
-        <v>186</v>
+        <v>196</v>
       </c>
       <c r="M44">
         <v>120</v>
@@ -7436,7 +7514,7 @@
         <v>1.148</v>
       </c>
       <c r="AE44" t="s">
-        <v>193</v>
+        <v>203</v>
       </c>
       <c r="AF44">
         <v>-0.051111</v>
@@ -7489,10 +7567,10 @@
     </row>
     <row r="45" spans="1:47">
       <c r="A45" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B45" t="s">
-        <v>92</v>
+        <v>102</v>
       </c>
       <c r="C45" s="2">
         <v>44023.35230556713</v>
@@ -7513,16 +7591,16 @@
         <v>540</v>
       </c>
       <c r="I45" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="J45" t="b">
         <v>1</v>
       </c>
       <c r="K45" t="s">
-        <v>139</v>
+        <v>149</v>
       </c>
       <c r="L45" t="s">
-        <v>187</v>
+        <v>197</v>
       </c>
       <c r="M45">
         <v>119</v>
@@ -7579,7 +7657,7 @@
         <v>0.93466667</v>
       </c>
       <c r="AE45" t="s">
-        <v>193</v>
+        <v>203</v>
       </c>
       <c r="AF45">
         <v>-0.023333</v>
@@ -7632,10 +7710,10 @@
     </row>
     <row r="46" spans="1:47">
       <c r="A46" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B46" t="s">
-        <v>94</v>
+        <v>104</v>
       </c>
       <c r="C46" s="2">
         <v>44023.35257471065</v>
@@ -7656,16 +7734,16 @@
         <v>566</v>
       </c>
       <c r="I46" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="J46" t="b">
         <v>1</v>
       </c>
       <c r="K46" t="s">
-        <v>140</v>
+        <v>150</v>
       </c>
       <c r="L46" t="s">
-        <v>188</v>
+        <v>198</v>
       </c>
       <c r="M46">
         <v>121</v>
@@ -7701,7 +7779,7 @@
         <v>1.03133333</v>
       </c>
       <c r="AE46" t="s">
-        <v>193</v>
+        <v>203</v>
       </c>
       <c r="AF46">
         <v>0.005278</v>
@@ -7754,10 +7832,10 @@
     </row>
     <row r="47" spans="1:47">
       <c r="A47" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B47" t="s">
-        <v>93</v>
+        <v>103</v>
       </c>
       <c r="C47" s="2">
         <v>44023.35262537037</v>
@@ -7778,16 +7856,16 @@
         <v>570</v>
       </c>
       <c r="I47" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="J47" t="b">
         <v>1</v>
       </c>
       <c r="K47" t="s">
-        <v>141</v>
+        <v>151</v>
       </c>
       <c r="L47" t="s">
-        <v>189</v>
+        <v>199</v>
       </c>
       <c r="M47">
         <v>121</v>
@@ -7844,7 +7922,7 @@
         <v>0.833</v>
       </c>
       <c r="AE47" t="s">
-        <v>193</v>
+        <v>203</v>
       </c>
       <c r="AF47">
         <v>-0.021667</v>
@@ -7897,10 +7975,10 @@
     </row>
     <row r="48" spans="1:47">
       <c r="A48" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B48" t="s">
-        <v>94</v>
+        <v>104</v>
       </c>
       <c r="C48" s="2">
         <v>44023.35292203704</v>
@@ -7921,16 +7999,16 @@
         <v>596</v>
       </c>
       <c r="I48" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="J48" t="b">
         <v>1</v>
       </c>
       <c r="K48" t="s">
-        <v>142</v>
+        <v>152</v>
       </c>
       <c r="L48" t="s">
-        <v>190</v>
+        <v>200</v>
       </c>
       <c r="M48">
         <v>121</v>
@@ -7966,7 +8044,7 @@
         <v>0.43666667</v>
       </c>
       <c r="AE48" t="s">
-        <v>193</v>
+        <v>203</v>
       </c>
       <c r="AF48">
         <v>-0.043333</v>
@@ -8019,10 +8097,10 @@
     </row>
     <row r="49" spans="1:47">
       <c r="A49" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B49" t="s">
-        <v>93</v>
+        <v>103</v>
       </c>
       <c r="C49" s="2">
         <v>44023.35297302083</v>
@@ -8043,16 +8121,16 @@
         <v>600</v>
       </c>
       <c r="I49" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="J49" t="b">
         <v>1</v>
       </c>
       <c r="K49" t="s">
-        <v>143</v>
+        <v>153</v>
       </c>
       <c r="L49" t="s">
-        <v>191</v>
+        <v>201</v>
       </c>
       <c r="M49">
         <v>121</v>
@@ -8109,7 +8187,7 @@
         <v>0.376</v>
       </c>
       <c r="AE49" t="s">
-        <v>193</v>
+        <v>203</v>
       </c>
       <c r="AF49">
         <v>-0.006667</v>
@@ -8172,156 +8250,156 @@
   <sheetData>
     <row r="1" spans="1:48">
       <c r="A1" s="1" t="s">
-        <v>44</v>
+        <v>54</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>46</v>
+        <v>56</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>47</v>
+        <v>57</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>48</v>
+        <v>58</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>49</v>
+        <v>59</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>53</v>
+        <v>63</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>54</v>
+        <v>64</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>55</v>
+        <v>65</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>56</v>
+        <v>66</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>57</v>
+        <v>67</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>59</v>
+        <v>69</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>61</v>
+        <v>71</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>62</v>
+        <v>72</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>63</v>
+        <v>73</v>
       </c>
       <c r="U1" s="1" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="V1" s="1" t="s">
-        <v>65</v>
+        <v>75</v>
       </c>
       <c r="W1" s="1" t="s">
-        <v>66</v>
+        <v>76</v>
       </c>
       <c r="X1" s="1" t="s">
-        <v>67</v>
+        <v>77</v>
       </c>
       <c r="Y1" s="1" t="s">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="Z1" s="1" t="s">
-        <v>69</v>
+        <v>79</v>
       </c>
       <c r="AA1" s="1" t="s">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="AB1" s="1" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
       <c r="AC1" s="1" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
       <c r="AD1" s="1" t="s">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="AE1" s="1" t="s">
-        <v>74</v>
+        <v>84</v>
       </c>
       <c r="AF1" s="1" t="s">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="AG1" s="1" t="s">
-        <v>76</v>
+        <v>86</v>
       </c>
       <c r="AH1" s="1" t="s">
-        <v>77</v>
+        <v>87</v>
       </c>
       <c r="AI1" s="1" t="s">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="AJ1" s="1" t="s">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="AK1" s="1" t="s">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="AL1" s="1" t="s">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="AM1" s="1" t="s">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="AN1" s="1" t="s">
-        <v>83</v>
+        <v>93</v>
       </c>
       <c r="AO1" s="1" t="s">
-        <v>84</v>
+        <v>94</v>
       </c>
       <c r="AP1" s="1" t="s">
-        <v>85</v>
+        <v>95</v>
       </c>
       <c r="AQ1" s="1" t="s">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="AR1" s="1" t="s">
-        <v>87</v>
+        <v>97</v>
       </c>
       <c r="AS1" s="1" t="s">
-        <v>88</v>
+        <v>98</v>
       </c>
       <c r="AT1" s="1" t="s">
-        <v>89</v>
+        <v>99</v>
       </c>
       <c r="AU1" s="1" t="s">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="AV1" s="1" t="s">
-        <v>91</v>
+        <v>101</v>
       </c>
     </row>
     <row r="2" spans="1:48">
       <c r="A2" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B2" t="s">
-        <v>92</v>
+        <v>102</v>
       </c>
       <c r="C2" s="2">
         <v>44023.35299995371</v>
@@ -8342,16 +8420,16 @@
         <v>0</v>
       </c>
       <c r="I2" t="s">
-        <v>195</v>
+        <v>205</v>
       </c>
       <c r="J2" t="b">
         <v>1</v>
       </c>
       <c r="K2" t="s">
-        <v>196</v>
+        <v>206</v>
       </c>
       <c r="L2" t="s">
-        <v>243</v>
+        <v>253</v>
       </c>
       <c r="M2">
         <v>120</v>
@@ -8408,7 +8486,7 @@
         <v>0.65533333</v>
       </c>
       <c r="AE2" t="s">
-        <v>290</v>
+        <v>300</v>
       </c>
       <c r="AG2">
         <v>2.15</v>
@@ -8425,10 +8503,10 @@
     </row>
     <row r="3" spans="1:48">
       <c r="A3" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B3" t="s">
-        <v>92</v>
+        <v>102</v>
       </c>
       <c r="C3" s="2">
         <v>44023.35333020833</v>
@@ -8449,16 +8527,16 @@
         <v>29</v>
       </c>
       <c r="I3" t="s">
-        <v>195</v>
+        <v>205</v>
       </c>
       <c r="J3" t="b">
         <v>1</v>
       </c>
       <c r="K3" t="s">
-        <v>197</v>
+        <v>207</v>
       </c>
       <c r="L3" t="s">
-        <v>244</v>
+        <v>254</v>
       </c>
       <c r="M3">
         <v>121</v>
@@ -8515,7 +8593,7 @@
         <v>-0.03172414</v>
       </c>
       <c r="AE3" t="s">
-        <v>290</v>
+        <v>300</v>
       </c>
       <c r="AF3">
         <v>-0.077705</v>
@@ -8556,10 +8634,10 @@
     </row>
     <row r="4" spans="1:48">
       <c r="A4" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B4" t="s">
-        <v>93</v>
+        <v>103</v>
       </c>
       <c r="C4" s="2">
         <v>44023.35331981481</v>
@@ -8580,16 +8658,16 @@
         <v>30</v>
       </c>
       <c r="I4" t="s">
-        <v>195</v>
+        <v>205</v>
       </c>
       <c r="J4" t="b">
         <v>1</v>
       </c>
       <c r="K4" t="s">
-        <v>198</v>
+        <v>208</v>
       </c>
       <c r="L4" t="s">
-        <v>245</v>
+        <v>255</v>
       </c>
       <c r="M4">
         <v>121</v>
@@ -8646,7 +8724,7 @@
         <v>-0.21333333</v>
       </c>
       <c r="AE4" t="s">
-        <v>290</v>
+        <v>300</v>
       </c>
       <c r="AF4">
         <v>-0.019885</v>
@@ -8699,10 +8777,10 @@
     </row>
     <row r="5" spans="1:48">
       <c r="A5" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B5" t="s">
-        <v>94</v>
+        <v>104</v>
       </c>
       <c r="C5" s="2">
         <v>44023.35361952546</v>
@@ -8723,16 +8801,16 @@
         <v>56</v>
       </c>
       <c r="I5" t="s">
-        <v>195</v>
+        <v>205</v>
       </c>
       <c r="J5" t="b">
         <v>1</v>
       </c>
       <c r="K5" t="s">
-        <v>199</v>
+        <v>209</v>
       </c>
       <c r="L5" t="s">
-        <v>246</v>
+        <v>256</v>
       </c>
       <c r="M5">
         <v>122</v>
@@ -8768,7 +8846,7 @@
         <v>-0.43166667</v>
       </c>
       <c r="AE5" t="s">
-        <v>290</v>
+        <v>300</v>
       </c>
       <c r="AF5">
         <v>-0.011944</v>
@@ -8821,10 +8899,10 @@
     </row>
     <row r="6" spans="1:48">
       <c r="A6" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B6" t="s">
-        <v>92</v>
+        <v>102</v>
       </c>
       <c r="C6" s="2">
         <v>44023.35369785879</v>
@@ -8845,16 +8923,16 @@
         <v>60</v>
       </c>
       <c r="I6" t="s">
-        <v>195</v>
+        <v>205</v>
       </c>
       <c r="J6" t="b">
         <v>1</v>
       </c>
       <c r="K6" t="s">
-        <v>200</v>
+        <v>210</v>
       </c>
       <c r="L6" t="s">
-        <v>247</v>
+        <v>257</v>
       </c>
       <c r="M6">
         <v>121</v>
@@ -8911,7 +8989,7 @@
         <v>-1.04225806</v>
       </c>
       <c r="AE6" t="s">
-        <v>290</v>
+        <v>300</v>
       </c>
       <c r="AF6">
         <v>-0.06460299999999999</v>
@@ -8964,10 +9042,10 @@
     </row>
     <row r="7" spans="1:48">
       <c r="A7" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B7" t="s">
-        <v>93</v>
+        <v>103</v>
       </c>
       <c r="C7" s="2">
         <v>44023.35366663194</v>
@@ -8988,16 +9066,16 @@
         <v>60</v>
       </c>
       <c r="I7" t="s">
-        <v>195</v>
+        <v>205</v>
       </c>
       <c r="J7" t="b">
         <v>1</v>
       </c>
       <c r="K7" t="s">
-        <v>201</v>
+        <v>211</v>
       </c>
       <c r="L7" t="s">
-        <v>248</v>
+        <v>258</v>
       </c>
       <c r="M7">
         <v>122</v>
@@ -9054,7 +9132,7 @@
         <v>-0.85333333</v>
       </c>
       <c r="AE7" t="s">
-        <v>290</v>
+        <v>300</v>
       </c>
       <c r="AF7">
         <v>0.020645</v>
@@ -9107,10 +9185,10 @@
     </row>
     <row r="8" spans="1:48">
       <c r="A8" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B8" t="s">
-        <v>94</v>
+        <v>104</v>
       </c>
       <c r="C8" s="2">
         <v>44023.35396462963</v>
@@ -9131,16 +9209,16 @@
         <v>86</v>
       </c>
       <c r="I8" t="s">
-        <v>195</v>
+        <v>205</v>
       </c>
       <c r="J8" t="b">
         <v>1</v>
       </c>
       <c r="K8" t="s">
-        <v>202</v>
+        <v>212</v>
       </c>
       <c r="L8" t="s">
-        <v>249</v>
+        <v>259</v>
       </c>
       <c r="M8">
         <v>122</v>
@@ -9176,7 +9254,7 @@
         <v>-1.006</v>
       </c>
       <c r="AE8" t="s">
-        <v>290</v>
+        <v>300</v>
       </c>
       <c r="AF8">
         <v>-0.016667</v>
@@ -9229,10 +9307,10 @@
     </row>
     <row r="9" spans="1:48">
       <c r="A9" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B9" t="s">
-        <v>93</v>
+        <v>103</v>
       </c>
       <c r="C9" s="2">
         <v>44023.35401414352</v>
@@ -9253,16 +9331,16 @@
         <v>90</v>
       </c>
       <c r="I9" t="s">
-        <v>195</v>
+        <v>205</v>
       </c>
       <c r="J9" t="b">
         <v>1</v>
       </c>
       <c r="K9" t="s">
-        <v>203</v>
+        <v>213</v>
       </c>
       <c r="L9" t="s">
-        <v>250</v>
+        <v>260</v>
       </c>
       <c r="M9">
         <v>122</v>
@@ -9319,7 +9397,7 @@
         <v>-1.04666667</v>
       </c>
       <c r="AE9" t="s">
-        <v>290</v>
+        <v>300</v>
       </c>
       <c r="AF9">
         <v>-0.004444</v>
@@ -9372,10 +9450,10 @@
     </row>
     <row r="10" spans="1:48">
       <c r="A10" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B10" t="s">
-        <v>94</v>
+        <v>104</v>
       </c>
       <c r="C10" s="2">
         <v>44023.35431188657</v>
@@ -9396,16 +9474,16 @@
         <v>116</v>
       </c>
       <c r="I10" t="s">
-        <v>195</v>
+        <v>205</v>
       </c>
       <c r="J10" t="b">
         <v>1</v>
       </c>
       <c r="K10" t="s">
-        <v>204</v>
+        <v>214</v>
       </c>
       <c r="L10" t="s">
-        <v>251</v>
+        <v>261</v>
       </c>
       <c r="M10">
         <v>122</v>
@@ -9441,7 +9519,7 @@
         <v>-1.331</v>
       </c>
       <c r="AE10" t="s">
-        <v>290</v>
+        <v>300</v>
       </c>
       <c r="AF10">
         <v>-0.031111</v>
@@ -9494,10 +9572,10 @@
     </row>
     <row r="11" spans="1:48">
       <c r="A11" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B11" t="s">
-        <v>93</v>
+        <v>103</v>
       </c>
       <c r="C11" s="2">
         <v>44023.35436167824</v>
@@ -9518,16 +9596,16 @@
         <v>120</v>
       </c>
       <c r="I11" t="s">
-        <v>195</v>
+        <v>205</v>
       </c>
       <c r="J11" t="b">
         <v>1</v>
       </c>
       <c r="K11" t="s">
-        <v>205</v>
+        <v>215</v>
       </c>
       <c r="L11" t="s">
-        <v>252</v>
+        <v>262</v>
       </c>
       <c r="M11">
         <v>119</v>
@@ -9584,7 +9662,7 @@
         <v>-1.38166667</v>
       </c>
       <c r="AE11" t="s">
-        <v>290</v>
+        <v>300</v>
       </c>
       <c r="AF11">
         <v>-0.005556</v>
@@ -9637,10 +9715,10 @@
     </row>
     <row r="12" spans="1:48">
       <c r="A12" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B12" t="s">
-        <v>92</v>
+        <v>102</v>
       </c>
       <c r="C12" s="2">
         <v>44023.35438840277</v>
@@ -9661,16 +9739,16 @@
         <v>120</v>
       </c>
       <c r="I12" t="s">
-        <v>195</v>
+        <v>205</v>
       </c>
       <c r="J12" t="b">
         <v>1</v>
       </c>
       <c r="K12" t="s">
-        <v>206</v>
+        <v>216</v>
       </c>
       <c r="L12" t="s">
-        <v>253</v>
+        <v>263</v>
       </c>
       <c r="M12">
         <v>119</v>
@@ -9727,7 +9805,7 @@
         <v>-1.22416667</v>
       </c>
       <c r="AE12" t="s">
-        <v>290</v>
+        <v>300</v>
       </c>
       <c r="AF12">
         <v>0.008611000000000001</v>
@@ -9780,10 +9858,10 @@
     </row>
     <row r="13" spans="1:48">
       <c r="A13" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B13" t="s">
-        <v>93</v>
+        <v>103</v>
       </c>
       <c r="C13" s="2">
         <v>44023.35470967593</v>
@@ -9804,16 +9882,16 @@
         <v>150</v>
       </c>
       <c r="I13" t="s">
-        <v>195</v>
+        <v>205</v>
       </c>
       <c r="J13" t="b">
         <v>1</v>
       </c>
       <c r="K13" t="s">
-        <v>207</v>
+        <v>217</v>
       </c>
       <c r="L13" t="s">
-        <v>254</v>
+        <v>264</v>
       </c>
       <c r="M13">
         <v>119</v>
@@ -9870,7 +9948,7 @@
         <v>-1.78833333</v>
       </c>
       <c r="AE13" t="s">
-        <v>290</v>
+        <v>300</v>
       </c>
       <c r="AF13">
         <v>-0.061667</v>
@@ -9923,10 +10001,10 @@
     </row>
     <row r="14" spans="1:48">
       <c r="A14" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B14" t="s">
-        <v>94</v>
+        <v>104</v>
       </c>
       <c r="C14" s="2">
         <v>44023.35500557871</v>
@@ -9947,16 +10025,16 @@
         <v>176</v>
       </c>
       <c r="I14" t="s">
-        <v>195</v>
+        <v>205</v>
       </c>
       <c r="J14" t="b">
         <v>1</v>
       </c>
       <c r="K14" t="s">
-        <v>208</v>
+        <v>218</v>
       </c>
       <c r="L14" t="s">
-        <v>255</v>
+        <v>265</v>
       </c>
       <c r="M14">
         <v>122</v>
@@ -9992,7 +10070,7 @@
         <v>-1.79833333</v>
       </c>
       <c r="AE14" t="s">
-        <v>290</v>
+        <v>300</v>
       </c>
       <c r="AF14">
         <v>-0.000556</v>
@@ -10045,10 +10123,10 @@
     </row>
     <row r="15" spans="1:48">
       <c r="A15" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B15" t="s">
-        <v>93</v>
+        <v>103</v>
       </c>
       <c r="C15" s="2">
         <v>44023.35505572917</v>
@@ -10069,16 +10147,16 @@
         <v>180</v>
       </c>
       <c r="I15" t="s">
-        <v>195</v>
+        <v>205</v>
       </c>
       <c r="J15" t="b">
         <v>1</v>
       </c>
       <c r="K15" t="s">
-        <v>209</v>
+        <v>219</v>
       </c>
       <c r="L15" t="s">
-        <v>256</v>
+        <v>266</v>
       </c>
       <c r="M15">
         <v>119</v>
@@ -10135,7 +10213,7 @@
         <v>-1.81833333</v>
       </c>
       <c r="AE15" t="s">
-        <v>290</v>
+        <v>300</v>
       </c>
       <c r="AF15">
         <v>-0.002222</v>
@@ -10188,10 +10266,10 @@
     </row>
     <row r="16" spans="1:48">
       <c r="A16" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B16" t="s">
-        <v>94</v>
+        <v>104</v>
       </c>
       <c r="C16" s="2">
         <v>44023.35535255787</v>
@@ -10212,16 +10290,16 @@
         <v>206</v>
       </c>
       <c r="I16" t="s">
-        <v>195</v>
+        <v>205</v>
       </c>
       <c r="J16" t="b">
         <v>1</v>
       </c>
       <c r="K16" t="s">
-        <v>210</v>
+        <v>220</v>
       </c>
       <c r="L16" t="s">
-        <v>257</v>
+        <v>267</v>
       </c>
       <c r="M16">
         <v>118</v>
@@ -10257,7 +10335,7 @@
         <v>-1.73733333</v>
       </c>
       <c r="AE16" t="s">
-        <v>290</v>
+        <v>300</v>
       </c>
       <c r="AF16">
         <v>0.008888999999999999</v>
@@ -10310,10 +10388,10 @@
     </row>
     <row r="17" spans="1:47">
       <c r="A17" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B17" t="s">
-        <v>93</v>
+        <v>103</v>
       </c>
       <c r="C17" s="2">
         <v>44023.3554027662</v>
@@ -10334,16 +10412,16 @@
         <v>210</v>
       </c>
       <c r="I17" t="s">
-        <v>195</v>
+        <v>205</v>
       </c>
       <c r="J17" t="b">
         <v>1</v>
       </c>
       <c r="K17" t="s">
-        <v>211</v>
+        <v>221</v>
       </c>
       <c r="L17" t="s">
-        <v>258</v>
+        <v>268</v>
       </c>
       <c r="M17">
         <v>124</v>
@@ -10400,7 +10478,7 @@
         <v>-1.74766667</v>
       </c>
       <c r="AE17" t="s">
-        <v>290</v>
+        <v>300</v>
       </c>
       <c r="AF17">
         <v>-0.001111</v>
@@ -10453,10 +10531,10 @@
     </row>
     <row r="18" spans="1:47">
       <c r="A18" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B18" t="s">
-        <v>94</v>
+        <v>104</v>
       </c>
       <c r="C18" s="2">
         <v>44023.35569953704</v>
@@ -10477,16 +10555,16 @@
         <v>236</v>
       </c>
       <c r="I18" t="s">
-        <v>195</v>
+        <v>205</v>
       </c>
       <c r="J18" t="b">
         <v>1</v>
       </c>
       <c r="K18" t="s">
-        <v>212</v>
+        <v>222</v>
       </c>
       <c r="L18" t="s">
-        <v>259</v>
+        <v>269</v>
       </c>
       <c r="M18">
         <v>113</v>
@@ -10522,7 +10600,7 @@
         <v>-2.164</v>
       </c>
       <c r="AE18" t="s">
-        <v>290</v>
+        <v>300</v>
       </c>
       <c r="AF18">
         <v>-0.045556</v>
@@ -10575,10 +10653,10 @@
     </row>
     <row r="19" spans="1:47">
       <c r="A19" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B19" t="s">
-        <v>93</v>
+        <v>103</v>
       </c>
       <c r="C19" s="2">
         <v>44023.35575015046</v>
@@ -10599,16 +10677,16 @@
         <v>240</v>
       </c>
       <c r="I19" t="s">
-        <v>195</v>
+        <v>205</v>
       </c>
       <c r="J19" t="b">
         <v>1</v>
       </c>
       <c r="K19" t="s">
-        <v>213</v>
+        <v>223</v>
       </c>
       <c r="L19" t="s">
-        <v>260</v>
+        <v>270</v>
       </c>
       <c r="M19">
         <v>118</v>
@@ -10665,7 +10743,7 @@
         <v>-2.225</v>
       </c>
       <c r="AE19" t="s">
-        <v>290</v>
+        <v>300</v>
       </c>
       <c r="AF19">
         <v>-0.006667</v>
@@ -10718,10 +10796,10 @@
     </row>
     <row r="20" spans="1:47">
       <c r="A20" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B20" t="s">
-        <v>94</v>
+        <v>104</v>
       </c>
       <c r="C20" s="2">
         <v>44023.35604671296</v>
@@ -10742,16 +10820,16 @@
         <v>266</v>
       </c>
       <c r="I20" t="s">
-        <v>195</v>
+        <v>205</v>
       </c>
       <c r="J20" t="b">
         <v>1</v>
       </c>
       <c r="K20" t="s">
-        <v>214</v>
+        <v>224</v>
       </c>
       <c r="L20" t="s">
-        <v>261</v>
+        <v>271</v>
       </c>
       <c r="M20">
         <v>107</v>
@@ -10787,7 +10865,7 @@
         <v>-2.57066667</v>
       </c>
       <c r="AE20" t="s">
-        <v>290</v>
+        <v>300</v>
       </c>
       <c r="AF20">
         <v>-0.037778</v>
@@ -10840,10 +10918,10 @@
     </row>
     <row r="21" spans="1:47">
       <c r="A21" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B21" t="s">
-        <v>93</v>
+        <v>103</v>
       </c>
       <c r="C21" s="2">
         <v>44023.35609765046</v>
@@ -10864,16 +10942,16 @@
         <v>270</v>
       </c>
       <c r="I21" t="s">
-        <v>195</v>
+        <v>205</v>
       </c>
       <c r="J21" t="b">
         <v>1</v>
       </c>
       <c r="K21" t="s">
-        <v>215</v>
+        <v>225</v>
       </c>
       <c r="L21" t="s">
-        <v>262</v>
+        <v>272</v>
       </c>
       <c r="M21">
         <v>109</v>
@@ -10930,7 +11008,7 @@
         <v>-2.49933333</v>
       </c>
       <c r="AE21" t="s">
-        <v>290</v>
+        <v>300</v>
       </c>
       <c r="AF21">
         <v>0.007778</v>
@@ -10983,10 +11061,10 @@
     </row>
     <row r="22" spans="1:47">
       <c r="A22" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B22" t="s">
-        <v>92</v>
+        <v>102</v>
       </c>
       <c r="C22" s="2">
         <v>44023.35647199074</v>
@@ -11007,16 +11085,16 @@
         <v>300</v>
       </c>
       <c r="I22" t="s">
-        <v>195</v>
+        <v>205</v>
       </c>
       <c r="J22" t="b">
         <v>1</v>
       </c>
       <c r="K22" t="s">
-        <v>216</v>
+        <v>226</v>
       </c>
       <c r="L22" t="s">
-        <v>263</v>
+        <v>273</v>
       </c>
       <c r="M22">
         <v>102</v>
@@ -11073,7 +11151,7 @@
         <v>-2.11838889</v>
       </c>
       <c r="AE22" t="s">
-        <v>290</v>
+        <v>300</v>
       </c>
       <c r="AF22">
         <v>0.006944</v>
@@ -11126,10 +11204,10 @@
     </row>
     <row r="23" spans="1:47">
       <c r="A23" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B23" t="s">
-        <v>93</v>
+        <v>103</v>
       </c>
       <c r="C23" s="2">
         <v>44023.35644489584</v>
@@ -11150,16 +11228,16 @@
         <v>300</v>
       </c>
       <c r="I23" t="s">
-        <v>195</v>
+        <v>205</v>
       </c>
       <c r="J23" t="b">
         <v>1</v>
       </c>
       <c r="K23" t="s">
-        <v>217</v>
+        <v>227</v>
       </c>
       <c r="L23" t="s">
-        <v>264</v>
+        <v>274</v>
       </c>
       <c r="M23">
         <v>99</v>
@@ -11216,7 +11294,7 @@
         <v>-2.784</v>
       </c>
       <c r="AE23" t="s">
-        <v>290</v>
+        <v>300</v>
       </c>
       <c r="AF23">
         <v>-0.072778</v>
@@ -11269,10 +11347,10 @@
     </row>
     <row r="24" spans="1:47">
       <c r="A24" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B24" t="s">
-        <v>94</v>
+        <v>104</v>
       </c>
       <c r="C24" s="2">
         <v>44023.35674206018</v>
@@ -11293,16 +11371,16 @@
         <v>326</v>
       </c>
       <c r="I24" t="s">
-        <v>195</v>
+        <v>205</v>
       </c>
       <c r="J24" t="b">
         <v>1</v>
       </c>
       <c r="K24" t="s">
-        <v>218</v>
+        <v>228</v>
       </c>
       <c r="L24" t="s">
-        <v>265</v>
+        <v>275</v>
       </c>
       <c r="M24">
         <v>102</v>
@@ -11338,7 +11416,7 @@
         <v>-2.90066667</v>
       </c>
       <c r="AE24" t="s">
-        <v>290</v>
+        <v>300</v>
       </c>
       <c r="AF24">
         <v>-0.006389</v>
@@ -11391,10 +11469,10 @@
     </row>
     <row r="25" spans="1:47">
       <c r="A25" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B25" t="s">
-        <v>93</v>
+        <v>103</v>
       </c>
       <c r="C25" s="2">
         <v>44023.35679211806</v>
@@ -11415,16 +11493,16 @@
         <v>330</v>
       </c>
       <c r="I25" t="s">
-        <v>195</v>
+        <v>205</v>
       </c>
       <c r="J25" t="b">
         <v>1</v>
       </c>
       <c r="K25" t="s">
-        <v>219</v>
+        <v>229</v>
       </c>
       <c r="L25" t="s">
-        <v>266</v>
+        <v>276</v>
       </c>
       <c r="M25">
         <v>98</v>
@@ -11481,7 +11559,7 @@
         <v>-3.20033333</v>
       </c>
       <c r="AE25" t="s">
-        <v>290</v>
+        <v>300</v>
       </c>
       <c r="AF25">
         <v>-0.032778</v>
@@ -11534,10 +11612,10 @@
     </row>
     <row r="26" spans="1:47">
       <c r="A26" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B26" t="s">
-        <v>93</v>
+        <v>103</v>
       </c>
       <c r="C26" s="2">
         <v>44023.35713885417</v>
@@ -11558,16 +11636,16 @@
         <v>360</v>
       </c>
       <c r="I26" t="s">
-        <v>195</v>
+        <v>205</v>
       </c>
       <c r="J26" t="b">
         <v>1</v>
       </c>
       <c r="K26" t="s">
-        <v>220</v>
+        <v>230</v>
       </c>
       <c r="L26" t="s">
-        <v>267</v>
+        <v>277</v>
       </c>
       <c r="M26">
         <v>98</v>
@@ -11624,7 +11702,7 @@
         <v>-3.424</v>
       </c>
       <c r="AE26" t="s">
-        <v>290</v>
+        <v>300</v>
       </c>
       <c r="AF26">
         <v>-0.024444</v>
@@ -11677,10 +11755,10 @@
     </row>
     <row r="27" spans="1:47">
       <c r="A27" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B27" t="s">
-        <v>94</v>
+        <v>104</v>
       </c>
       <c r="C27" s="2">
         <v>44023.35743622685</v>
@@ -11701,16 +11779,16 @@
         <v>386</v>
       </c>
       <c r="I27" t="s">
-        <v>195</v>
+        <v>205</v>
       </c>
       <c r="J27" t="b">
         <v>1</v>
       </c>
       <c r="K27" t="s">
-        <v>221</v>
+        <v>231</v>
       </c>
       <c r="L27" t="s">
-        <v>268</v>
+        <v>278</v>
       </c>
       <c r="M27">
         <v>118</v>
@@ -11746,7 +11824,7 @@
         <v>-3.302</v>
       </c>
       <c r="AE27" t="s">
-        <v>290</v>
+        <v>300</v>
       </c>
       <c r="AF27">
         <v>0.006667</v>
@@ -11799,10 +11877,10 @@
     </row>
     <row r="28" spans="1:47">
       <c r="A28" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B28" t="s">
-        <v>93</v>
+        <v>103</v>
       </c>
       <c r="C28" s="2">
         <v>44023.35748664352</v>
@@ -11823,16 +11901,16 @@
         <v>390</v>
       </c>
       <c r="I28" t="s">
-        <v>195</v>
+        <v>205</v>
       </c>
       <c r="J28" t="b">
         <v>1</v>
       </c>
       <c r="K28" t="s">
-        <v>222</v>
+        <v>232</v>
       </c>
       <c r="L28" t="s">
-        <v>269</v>
+        <v>279</v>
       </c>
       <c r="M28">
         <v>118</v>
@@ -11889,7 +11967,7 @@
         <v>-3.09866667</v>
       </c>
       <c r="AE28" t="s">
-        <v>290</v>
+        <v>300</v>
       </c>
       <c r="AF28">
         <v>0.022222</v>
@@ -11942,10 +12020,10 @@
     </row>
     <row r="29" spans="1:47">
       <c r="A29" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B29" t="s">
-        <v>94</v>
+        <v>104</v>
       </c>
       <c r="C29" s="2">
         <v>44023.35778332176</v>
@@ -11966,16 +12044,16 @@
         <v>416</v>
       </c>
       <c r="I29" t="s">
-        <v>195</v>
+        <v>205</v>
       </c>
       <c r="J29" t="b">
         <v>1</v>
       </c>
       <c r="K29" t="s">
-        <v>223</v>
+        <v>233</v>
       </c>
       <c r="L29" t="s">
-        <v>270</v>
+        <v>280</v>
       </c>
       <c r="M29">
         <v>84</v>
@@ -12011,7 +12089,7 @@
         <v>-3.566</v>
       </c>
       <c r="AE29" t="s">
-        <v>290</v>
+        <v>300</v>
       </c>
       <c r="AF29">
         <v>-0.051111</v>
@@ -12064,10 +12142,10 @@
     </row>
     <row r="30" spans="1:47">
       <c r="A30" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B30" t="s">
-        <v>93</v>
+        <v>103</v>
       </c>
       <c r="C30" s="2">
         <v>44023.35783324074</v>
@@ -12088,16 +12166,16 @@
         <v>420</v>
       </c>
       <c r="I30" t="s">
-        <v>195</v>
+        <v>205</v>
       </c>
       <c r="J30" t="b">
         <v>1</v>
       </c>
       <c r="K30" t="s">
-        <v>224</v>
+        <v>234</v>
       </c>
       <c r="L30" t="s">
-        <v>271</v>
+        <v>281</v>
       </c>
       <c r="M30">
         <v>119</v>
@@ -12154,7 +12232,7 @@
         <v>-3.63733333</v>
       </c>
       <c r="AE30" t="s">
-        <v>290</v>
+        <v>300</v>
       </c>
       <c r="AF30">
         <v>-0.007778</v>
@@ -12207,10 +12285,10 @@
     </row>
     <row r="31" spans="1:47">
       <c r="A31" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B31" t="s">
-        <v>92</v>
+        <v>102</v>
       </c>
       <c r="C31" s="2">
         <v>44023.35786231481</v>
@@ -12231,16 +12309,16 @@
         <v>420</v>
       </c>
       <c r="I31" t="s">
-        <v>195</v>
+        <v>205</v>
       </c>
       <c r="J31" t="b">
         <v>1</v>
       </c>
       <c r="K31" t="s">
-        <v>225</v>
+        <v>235</v>
       </c>
       <c r="L31" t="s">
-        <v>272</v>
+        <v>282</v>
       </c>
       <c r="M31">
         <v>120</v>
@@ -12297,7 +12375,7 @@
         <v>-3.37566667</v>
       </c>
       <c r="AE31" t="s">
-        <v>290</v>
+        <v>300</v>
       </c>
       <c r="AF31">
         <v>0.007153</v>
@@ -12350,10 +12428,10 @@
     </row>
     <row r="32" spans="1:47">
       <c r="A32" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B32" t="s">
-        <v>93</v>
+        <v>103</v>
       </c>
       <c r="C32" s="2">
         <v>44023.35818081019</v>
@@ -12374,16 +12452,16 @@
         <v>450</v>
       </c>
       <c r="I32" t="s">
-        <v>195</v>
+        <v>205</v>
       </c>
       <c r="J32" t="b">
         <v>1</v>
       </c>
       <c r="K32" t="s">
-        <v>226</v>
+        <v>236</v>
       </c>
       <c r="L32" t="s">
-        <v>273</v>
+        <v>283</v>
       </c>
       <c r="M32">
         <v>110</v>
@@ -12440,7 +12518,7 @@
         <v>-4.074</v>
       </c>
       <c r="AE32" t="s">
-        <v>290</v>
+        <v>300</v>
       </c>
       <c r="AF32">
         <v>-0.076389</v>
@@ -12493,10 +12571,10 @@
     </row>
     <row r="33" spans="1:47">
       <c r="A33" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B33" t="s">
-        <v>92</v>
+        <v>102</v>
       </c>
       <c r="C33" s="2">
         <v>44023.35819207176</v>
@@ -12517,16 +12595,16 @@
         <v>450</v>
       </c>
       <c r="I33" t="s">
-        <v>195</v>
+        <v>205</v>
       </c>
       <c r="J33" t="b">
         <v>1</v>
       </c>
       <c r="K33" t="s">
-        <v>227</v>
+        <v>237</v>
       </c>
       <c r="L33" t="s">
-        <v>274</v>
+        <v>284</v>
       </c>
       <c r="M33">
         <v>115</v>
@@ -12583,7 +12661,7 @@
         <v>-4.05366667</v>
       </c>
       <c r="AE33" t="s">
-        <v>290</v>
+        <v>300</v>
       </c>
       <c r="AF33">
         <v>0.002222</v>
@@ -12636,10 +12714,10 @@
     </row>
     <row r="34" spans="1:47">
       <c r="A34" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B34" t="s">
-        <v>94</v>
+        <v>104</v>
       </c>
       <c r="C34" s="2">
         <v>44023.35847700232</v>
@@ -12660,16 +12738,16 @@
         <v>476</v>
       </c>
       <c r="I34" t="s">
-        <v>195</v>
+        <v>205</v>
       </c>
       <c r="J34" t="b">
         <v>1</v>
       </c>
       <c r="K34" t="s">
-        <v>228</v>
+        <v>238</v>
       </c>
       <c r="L34" t="s">
-        <v>275</v>
+        <v>285</v>
       </c>
       <c r="M34">
         <v>95</v>
@@ -12705,7 +12783,7 @@
         <v>-3.932</v>
       </c>
       <c r="AE34" t="s">
-        <v>290</v>
+        <v>300</v>
       </c>
       <c r="AF34">
         <v>0.006667</v>
@@ -12758,10 +12836,10 @@
     </row>
     <row r="35" spans="1:47">
       <c r="A35" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B35" t="s">
-        <v>92</v>
+        <v>102</v>
       </c>
       <c r="C35" s="2">
         <v>44023.3585559375</v>
@@ -12782,16 +12860,16 @@
         <v>480</v>
       </c>
       <c r="I35" t="s">
-        <v>195</v>
+        <v>205</v>
       </c>
       <c r="J35" t="b">
         <v>1</v>
       </c>
       <c r="K35" t="s">
-        <v>229</v>
+        <v>239</v>
       </c>
       <c r="L35" t="s">
-        <v>276</v>
+        <v>286</v>
       </c>
       <c r="M35">
         <v>99</v>
@@ -12848,7 +12926,7 @@
         <v>-3.871</v>
       </c>
       <c r="AE35" t="s">
-        <v>290</v>
+        <v>300</v>
       </c>
       <c r="AF35">
         <v>0.006667</v>
@@ -12901,10 +12979,10 @@
     </row>
     <row r="36" spans="1:47">
       <c r="A36" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B36" t="s">
-        <v>93</v>
+        <v>103</v>
       </c>
       <c r="C36" s="2">
         <v>44023.35852927083</v>
@@ -12925,16 +13003,16 @@
         <v>480</v>
       </c>
       <c r="I36" t="s">
-        <v>195</v>
+        <v>205</v>
       </c>
       <c r="J36" t="b">
         <v>1</v>
       </c>
       <c r="K36" t="s">
-        <v>230</v>
+        <v>240</v>
       </c>
       <c r="L36" t="s">
-        <v>277</v>
+        <v>287</v>
       </c>
       <c r="M36">
         <v>93</v>
@@ -12991,7 +13069,7 @@
         <v>-3.84066667</v>
       </c>
       <c r="AE36" t="s">
-        <v>290</v>
+        <v>300</v>
       </c>
       <c r="AF36">
         <v>0.003333</v>
@@ -13044,10 +13122,10 @@
     </row>
     <row r="37" spans="1:47">
       <c r="A37" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B37" t="s">
-        <v>94</v>
+        <v>104</v>
       </c>
       <c r="C37" s="2">
         <v>44023.3588266088</v>
@@ -13068,16 +13146,16 @@
         <v>506</v>
       </c>
       <c r="I37" t="s">
-        <v>195</v>
+        <v>205</v>
       </c>
       <c r="J37" t="b">
         <v>1</v>
       </c>
       <c r="K37" t="s">
-        <v>231</v>
+        <v>241</v>
       </c>
       <c r="L37" t="s">
-        <v>278</v>
+        <v>288</v>
       </c>
       <c r="M37">
         <v>138</v>
@@ -13113,7 +13191,7 @@
         <v>-3.59666667</v>
       </c>
       <c r="AE37" t="s">
-        <v>290</v>
+        <v>300</v>
       </c>
       <c r="AF37">
         <v>0.026667</v>
@@ -13166,10 +13244,10 @@
     </row>
     <row r="38" spans="1:47">
       <c r="A38" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B38" t="s">
-        <v>93</v>
+        <v>103</v>
       </c>
       <c r="C38" s="2">
         <v>44023.35887934027</v>
@@ -13190,16 +13268,16 @@
         <v>510</v>
       </c>
       <c r="I38" t="s">
-        <v>195</v>
+        <v>205</v>
       </c>
       <c r="J38" t="b">
         <v>1</v>
       </c>
       <c r="K38" t="s">
-        <v>232</v>
+        <v>242</v>
       </c>
       <c r="L38" t="s">
-        <v>279</v>
+        <v>289</v>
       </c>
       <c r="M38">
         <v>108</v>
@@ -13256,7 +13334,7 @@
         <v>-3.627</v>
       </c>
       <c r="AE38" t="s">
-        <v>290</v>
+        <v>300</v>
       </c>
       <c r="AF38">
         <v>-0.003333</v>
@@ -13309,10 +13387,10 @@
     </row>
     <row r="39" spans="1:47">
       <c r="A39" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B39" t="s">
-        <v>94</v>
+        <v>104</v>
       </c>
       <c r="C39" s="2">
         <v>44023.3591712963</v>
@@ -13333,16 +13411,16 @@
         <v>536</v>
       </c>
       <c r="I39" t="s">
-        <v>195</v>
+        <v>205</v>
       </c>
       <c r="J39" t="b">
         <v>1</v>
       </c>
       <c r="K39" t="s">
-        <v>233</v>
+        <v>243</v>
       </c>
       <c r="L39" t="s">
-        <v>280</v>
+        <v>290</v>
       </c>
       <c r="M39">
         <v>133</v>
@@ -13378,7 +13456,7 @@
         <v>-3.40333333</v>
       </c>
       <c r="AE39" t="s">
-        <v>290</v>
+        <v>300</v>
       </c>
       <c r="AF39">
         <v>0.024444</v>
@@ -13431,10 +13509,10 @@
     </row>
     <row r="40" spans="1:47">
       <c r="A40" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B40" t="s">
-        <v>93</v>
+        <v>103</v>
       </c>
       <c r="C40" s="2">
         <v>44023.35922280093</v>
@@ -13455,16 +13533,16 @@
         <v>540</v>
       </c>
       <c r="I40" t="s">
-        <v>195</v>
+        <v>205</v>
       </c>
       <c r="J40" t="b">
         <v>1</v>
       </c>
       <c r="K40" t="s">
-        <v>234</v>
+        <v>244</v>
       </c>
       <c r="L40" t="s">
-        <v>281</v>
+        <v>291</v>
       </c>
       <c r="M40">
         <v>120</v>
@@ -13521,7 +13599,7 @@
         <v>-3.32233333</v>
       </c>
       <c r="AE40" t="s">
-        <v>290</v>
+        <v>300</v>
       </c>
       <c r="AF40">
         <v>0.008888999999999999</v>
@@ -13574,10 +13652,10 @@
     </row>
     <row r="41" spans="1:47">
       <c r="A41" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B41" t="s">
-        <v>94</v>
+        <v>104</v>
       </c>
       <c r="C41" s="2">
         <v>44023.35952256944</v>
@@ -13598,16 +13676,16 @@
         <v>566</v>
       </c>
       <c r="I41" t="s">
-        <v>195</v>
+        <v>205</v>
       </c>
       <c r="J41" t="b">
         <v>1</v>
       </c>
       <c r="K41" t="s">
-        <v>235</v>
+        <v>245</v>
       </c>
       <c r="L41" t="s">
-        <v>282</v>
+        <v>292</v>
       </c>
       <c r="M41">
         <v>193</v>
@@ -13643,7 +13721,7 @@
         <v>-3.53566667</v>
       </c>
       <c r="AE41" t="s">
-        <v>290</v>
+        <v>300</v>
       </c>
       <c r="AF41">
         <v>-0.023333</v>
@@ -13696,10 +13774,10 @@
     </row>
     <row r="42" spans="1:47">
       <c r="A42" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B42" t="s">
-        <v>93</v>
+        <v>103</v>
       </c>
       <c r="C42" s="2">
         <v>44023.35956898148</v>
@@ -13720,16 +13798,16 @@
         <v>570</v>
       </c>
       <c r="I42" t="s">
-        <v>195</v>
+        <v>205</v>
       </c>
       <c r="J42" t="b">
         <v>1</v>
       </c>
       <c r="K42" t="s">
-        <v>236</v>
+        <v>246</v>
       </c>
       <c r="L42" t="s">
-        <v>283</v>
+        <v>293</v>
       </c>
       <c r="M42">
         <v>176</v>
@@ -13786,7 +13864,7 @@
         <v>-3.70833333</v>
       </c>
       <c r="AE42" t="s">
-        <v>290</v>
+        <v>300</v>
       </c>
       <c r="AF42">
         <v>-0.018889</v>
@@ -13839,10 +13917,10 @@
     </row>
     <row r="43" spans="1:47">
       <c r="A43" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B43" t="s">
-        <v>94</v>
+        <v>104</v>
       </c>
       <c r="C43" s="2">
         <v>44023.35986965278</v>
@@ -13863,16 +13941,16 @@
         <v>596</v>
       </c>
       <c r="I43" t="s">
-        <v>195</v>
+        <v>205</v>
       </c>
       <c r="J43" t="b">
         <v>1</v>
       </c>
       <c r="K43" t="s">
-        <v>237</v>
+        <v>247</v>
       </c>
       <c r="L43" t="s">
-        <v>284</v>
+        <v>294</v>
       </c>
       <c r="M43">
         <v>195</v>
@@ -13908,7 +13986,7 @@
         <v>-3.56633333</v>
       </c>
       <c r="AE43" t="s">
-        <v>290</v>
+        <v>300</v>
       </c>
       <c r="AF43">
         <v>0.015556</v>
@@ -13961,10 +14039,10 @@
     </row>
     <row r="44" spans="1:47">
       <c r="A44" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B44" t="s">
-        <v>93</v>
+        <v>103</v>
       </c>
       <c r="C44" s="2">
         <v>44023.35991907407</v>
@@ -13985,16 +14063,16 @@
         <v>600</v>
       </c>
       <c r="I44" t="s">
-        <v>195</v>
+        <v>205</v>
       </c>
       <c r="J44" t="b">
         <v>1</v>
       </c>
       <c r="K44" t="s">
-        <v>238</v>
+        <v>248</v>
       </c>
       <c r="L44" t="s">
-        <v>285</v>
+        <v>295</v>
       </c>
       <c r="M44">
         <v>200</v>
@@ -14051,7 +14129,7 @@
         <v>-3.39366667</v>
       </c>
       <c r="AE44" t="s">
-        <v>290</v>
+        <v>300</v>
       </c>
       <c r="AF44">
         <v>0.018889</v>
@@ -14104,10 +14182,10 @@
     </row>
     <row r="45" spans="1:47">
       <c r="A45" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B45" t="s">
-        <v>93</v>
+        <v>103</v>
       </c>
       <c r="C45" s="2">
         <v>44023.36026780093</v>
@@ -14128,16 +14206,16 @@
         <v>630</v>
       </c>
       <c r="I45" t="s">
-        <v>195</v>
+        <v>205</v>
       </c>
       <c r="J45" t="b">
         <v>1</v>
       </c>
       <c r="K45" t="s">
-        <v>239</v>
+        <v>249</v>
       </c>
       <c r="L45" t="s">
-        <v>286</v>
+        <v>296</v>
       </c>
       <c r="M45">
         <v>193</v>
@@ -14194,7 +14272,7 @@
         <v>-4.05366667</v>
       </c>
       <c r="AE45" t="s">
-        <v>290</v>
+        <v>300</v>
       </c>
       <c r="AF45">
         <v>-0.07222199999999999</v>
@@ -14247,10 +14325,10 @@
     </row>
     <row r="46" spans="1:47">
       <c r="A46" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B46" t="s">
-        <v>94</v>
+        <v>104</v>
       </c>
       <c r="C46" s="2">
         <v>44023.36056296296</v>
@@ -14271,16 +14349,16 @@
         <v>656</v>
       </c>
       <c r="I46" t="s">
-        <v>195</v>
+        <v>205</v>
       </c>
       <c r="J46" t="b">
         <v>1</v>
       </c>
       <c r="K46" t="s">
-        <v>240</v>
+        <v>250</v>
       </c>
       <c r="L46" t="s">
-        <v>287</v>
+        <v>297</v>
       </c>
       <c r="M46">
         <v>203</v>
@@ -14316,7 +14394,7 @@
         <v>-4.20116667</v>
       </c>
       <c r="AE46" t="s">
-        <v>290</v>
+        <v>300</v>
       </c>
       <c r="AF46">
         <v>-0.008056000000000001</v>
@@ -14369,10 +14447,10 @@
     </row>
     <row r="47" spans="1:47">
       <c r="A47" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B47" t="s">
-        <v>93</v>
+        <v>103</v>
       </c>
       <c r="C47" s="2">
         <v>44023.36061483796</v>
@@ -14393,16 +14471,16 @@
         <v>660</v>
       </c>
       <c r="I47" t="s">
-        <v>195</v>
+        <v>205</v>
       </c>
       <c r="J47" t="b">
         <v>1</v>
       </c>
       <c r="K47" t="s">
-        <v>241</v>
+        <v>251</v>
       </c>
       <c r="L47" t="s">
-        <v>288</v>
+        <v>298</v>
       </c>
       <c r="M47">
         <v>193</v>
@@ -14459,7 +14537,7 @@
         <v>-4.45</v>
       </c>
       <c r="AE47" t="s">
-        <v>290</v>
+        <v>300</v>
       </c>
       <c r="AF47">
         <v>-0.027222</v>
@@ -14512,10 +14590,10 @@
     </row>
     <row r="48" spans="1:47">
       <c r="A48" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B48" t="s">
-        <v>94</v>
+        <v>104</v>
       </c>
       <c r="C48" s="2">
         <v>44023.36369013889</v>
@@ -14536,16 +14614,16 @@
         <v>926</v>
       </c>
       <c r="I48" t="s">
-        <v>195</v>
+        <v>205</v>
       </c>
       <c r="J48" t="b">
         <v>1</v>
       </c>
       <c r="K48" t="s">
-        <v>242</v>
+        <v>252</v>
       </c>
       <c r="L48" t="s">
-        <v>289</v>
+        <v>299</v>
       </c>
       <c r="M48">
         <v>204</v>
@@ -14581,7 +14659,7 @@
         <v>-0.42218519</v>
       </c>
       <c r="AE48" t="s">
-        <v>290</v>
+        <v>300</v>
       </c>
       <c r="AF48">
         <v>0.048944</v>

</xml_diff>